<commit_message>
fix(plate-config): regenerate Stations 2-4 from fresh real-hardware corner measurements
Station 2 had drifted by a real, consistent (+39.293, -6.051)mm offset
from the previously-stored data (same offset across A1/A12/H1, confirming
the plate/nest physically shifted, not a data-entry error). Stations 3
and 4 were already correct -- fresh measurements differed by under 1mm
(0.03-0.68mm), within normal jog precision, not a real shift -- but
regenerated anyway from the fresh numbers for consistency. All three
produce clean, exact 9.00mm grids. Station 1 untouched (already correct).

U remains 200.023 for Stations 3-4 (matches left_home) and 170.065 for
Station 2 (matches right_home) -- unchanged, per config/machine_config.yaml.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/config/plate_configs/plate_stations.xlsx
+++ b/config/plate_configs/plate_stations.xlsx
@@ -2192,10 +2192,10 @@
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>249.543</v>
+        <v>288.836</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>227.725</v>
+        <v>221.674</v>
       </c>
       <c r="D2" s="2" t="n"/>
       <c r="E2" s="2" t="n"/>
@@ -2209,10 +2209,10 @@
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>249.543</v>
+        <v>288.836</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>218.725</v>
+        <v>212.674</v>
       </c>
       <c r="D3" s="2" t="n"/>
       <c r="E3" s="2" t="n"/>
@@ -2226,10 +2226,10 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>249.543</v>
+        <v>288.836</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>209.725</v>
+        <v>203.674</v>
       </c>
       <c r="D4" s="2" t="n"/>
       <c r="E4" s="2" t="n"/>
@@ -2243,10 +2243,10 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>249.543</v>
+        <v>288.836</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>200.725</v>
+        <v>194.674</v>
       </c>
       <c r="D5" s="2" t="n"/>
       <c r="E5" s="2" t="n"/>
@@ -2260,10 +2260,10 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>249.543</v>
+        <v>288.836</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>191.725</v>
+        <v>185.674</v>
       </c>
       <c r="D6" s="2" t="n"/>
       <c r="E6" s="2" t="n"/>
@@ -2277,10 +2277,10 @@
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>249.543</v>
+        <v>288.836</v>
       </c>
       <c r="C7" s="2" t="n">
-        <v>182.725</v>
+        <v>176.674</v>
       </c>
       <c r="D7" s="2" t="n"/>
       <c r="E7" s="2" t="n"/>
@@ -2294,10 +2294,10 @@
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>249.543</v>
+        <v>288.836</v>
       </c>
       <c r="C8" s="2" t="n">
-        <v>173.725</v>
+        <v>167.674</v>
       </c>
       <c r="D8" s="2" t="n"/>
       <c r="E8" s="2" t="n"/>
@@ -2311,10 +2311,10 @@
         </is>
       </c>
       <c r="B9" s="2" t="n">
-        <v>249.543</v>
+        <v>288.836</v>
       </c>
       <c r="C9" s="2" t="n">
-        <v>164.725</v>
+        <v>158.674</v>
       </c>
       <c r="D9" s="2" t="n"/>
       <c r="E9" s="2" t="n"/>
@@ -2328,10 +2328,10 @@
         </is>
       </c>
       <c r="B10" s="2" t="n">
-        <v>249.543</v>
+        <v>288.836</v>
       </c>
       <c r="C10" s="2" t="n">
-        <v>155.725</v>
+        <v>149.674</v>
       </c>
       <c r="D10" s="2" t="n"/>
       <c r="E10" s="2" t="n"/>
@@ -2345,10 +2345,10 @@
         </is>
       </c>
       <c r="B11" s="2" t="n">
-        <v>249.543</v>
+        <v>288.836</v>
       </c>
       <c r="C11" s="2" t="n">
-        <v>146.725</v>
+        <v>140.674</v>
       </c>
       <c r="D11" s="2" t="n"/>
       <c r="E11" s="2" t="n"/>
@@ -2362,10 +2362,10 @@
         </is>
       </c>
       <c r="B12" s="2" t="n">
-        <v>249.543</v>
+        <v>288.836</v>
       </c>
       <c r="C12" s="2" t="n">
-        <v>137.725</v>
+        <v>131.674</v>
       </c>
       <c r="D12" s="2" t="n"/>
       <c r="E12" s="2" t="n"/>
@@ -2379,10 +2379,10 @@
         </is>
       </c>
       <c r="B13" s="2" t="n">
-        <v>249.543</v>
+        <v>288.836</v>
       </c>
       <c r="C13" s="2" t="n">
-        <v>128.725</v>
+        <v>122.674</v>
       </c>
       <c r="D13" s="2" t="n"/>
       <c r="E13" s="2" t="n"/>
@@ -2396,10 +2396,10 @@
         </is>
       </c>
       <c r="B14" s="2" t="n">
-        <v>258.543</v>
+        <v>297.836</v>
       </c>
       <c r="C14" s="2" t="n">
-        <v>227.725</v>
+        <v>221.674</v>
       </c>
       <c r="D14" s="2" t="n"/>
       <c r="E14" s="2" t="n"/>
@@ -2413,10 +2413,10 @@
         </is>
       </c>
       <c r="B15" s="2" t="n">
-        <v>258.543</v>
+        <v>297.836</v>
       </c>
       <c r="C15" s="2" t="n">
-        <v>218.725</v>
+        <v>212.674</v>
       </c>
       <c r="D15" s="2" t="n"/>
       <c r="E15" s="2" t="n"/>
@@ -2430,10 +2430,10 @@
         </is>
       </c>
       <c r="B16" s="2" t="n">
-        <v>258.543</v>
+        <v>297.836</v>
       </c>
       <c r="C16" s="2" t="n">
-        <v>209.725</v>
+        <v>203.674</v>
       </c>
       <c r="D16" s="2" t="n"/>
       <c r="E16" s="2" t="n"/>
@@ -2447,10 +2447,10 @@
         </is>
       </c>
       <c r="B17" s="2" t="n">
-        <v>258.543</v>
+        <v>297.836</v>
       </c>
       <c r="C17" s="2" t="n">
-        <v>200.725</v>
+        <v>194.674</v>
       </c>
       <c r="D17" s="2" t="n"/>
       <c r="E17" s="2" t="n"/>
@@ -2464,10 +2464,10 @@
         </is>
       </c>
       <c r="B18" s="2" t="n">
-        <v>258.543</v>
+        <v>297.836</v>
       </c>
       <c r="C18" s="2" t="n">
-        <v>191.725</v>
+        <v>185.674</v>
       </c>
       <c r="D18" s="2" t="n"/>
       <c r="E18" s="2" t="n"/>
@@ -2481,10 +2481,10 @@
         </is>
       </c>
       <c r="B19" s="2" t="n">
-        <v>258.543</v>
+        <v>297.836</v>
       </c>
       <c r="C19" s="2" t="n">
-        <v>182.725</v>
+        <v>176.674</v>
       </c>
       <c r="D19" s="2" t="n"/>
       <c r="E19" s="2" t="n"/>
@@ -2498,10 +2498,10 @@
         </is>
       </c>
       <c r="B20" s="2" t="n">
-        <v>258.543</v>
+        <v>297.836</v>
       </c>
       <c r="C20" s="2" t="n">
-        <v>173.725</v>
+        <v>167.674</v>
       </c>
       <c r="D20" s="2" t="n"/>
       <c r="E20" s="2" t="n"/>
@@ -2515,10 +2515,10 @@
         </is>
       </c>
       <c r="B21" s="2" t="n">
-        <v>258.543</v>
+        <v>297.836</v>
       </c>
       <c r="C21" s="2" t="n">
-        <v>164.725</v>
+        <v>158.674</v>
       </c>
       <c r="D21" s="2" t="n"/>
       <c r="E21" s="2" t="n"/>
@@ -2532,10 +2532,10 @@
         </is>
       </c>
       <c r="B22" s="2" t="n">
-        <v>258.543</v>
+        <v>297.836</v>
       </c>
       <c r="C22" s="2" t="n">
-        <v>155.725</v>
+        <v>149.674</v>
       </c>
       <c r="D22" s="2" t="n"/>
       <c r="E22" s="2" t="n"/>
@@ -2549,10 +2549,10 @@
         </is>
       </c>
       <c r="B23" s="2" t="n">
-        <v>258.543</v>
+        <v>297.836</v>
       </c>
       <c r="C23" s="2" t="n">
-        <v>146.725</v>
+        <v>140.674</v>
       </c>
       <c r="D23" s="2" t="n"/>
       <c r="E23" s="2" t="n"/>
@@ -2566,10 +2566,10 @@
         </is>
       </c>
       <c r="B24" s="2" t="n">
-        <v>258.543</v>
+        <v>297.836</v>
       </c>
       <c r="C24" s="2" t="n">
-        <v>137.725</v>
+        <v>131.674</v>
       </c>
       <c r="D24" s="2" t="n"/>
       <c r="E24" s="2" t="n"/>
@@ -2583,10 +2583,10 @@
         </is>
       </c>
       <c r="B25" s="2" t="n">
-        <v>258.543</v>
+        <v>297.836</v>
       </c>
       <c r="C25" s="2" t="n">
-        <v>128.725</v>
+        <v>122.674</v>
       </c>
       <c r="D25" s="2" t="n"/>
       <c r="E25" s="2" t="n"/>
@@ -2600,10 +2600,10 @@
         </is>
       </c>
       <c r="B26" s="2" t="n">
-        <v>267.543</v>
+        <v>306.836</v>
       </c>
       <c r="C26" s="2" t="n">
-        <v>227.725</v>
+        <v>221.674</v>
       </c>
       <c r="D26" s="2" t="n"/>
       <c r="E26" s="2" t="n"/>
@@ -2617,10 +2617,10 @@
         </is>
       </c>
       <c r="B27" s="2" t="n">
-        <v>267.543</v>
+        <v>306.836</v>
       </c>
       <c r="C27" s="2" t="n">
-        <v>218.725</v>
+        <v>212.674</v>
       </c>
       <c r="D27" s="2" t="n"/>
       <c r="E27" s="2" t="n"/>
@@ -2634,10 +2634,10 @@
         </is>
       </c>
       <c r="B28" s="2" t="n">
-        <v>267.543</v>
+        <v>306.836</v>
       </c>
       <c r="C28" s="2" t="n">
-        <v>209.725</v>
+        <v>203.674</v>
       </c>
       <c r="D28" s="2" t="n"/>
       <c r="E28" s="2" t="n"/>
@@ -2651,10 +2651,10 @@
         </is>
       </c>
       <c r="B29" s="2" t="n">
-        <v>267.543</v>
+        <v>306.836</v>
       </c>
       <c r="C29" s="2" t="n">
-        <v>200.725</v>
+        <v>194.674</v>
       </c>
       <c r="D29" s="2" t="n"/>
       <c r="E29" s="2" t="n"/>
@@ -2668,10 +2668,10 @@
         </is>
       </c>
       <c r="B30" s="2" t="n">
-        <v>267.543</v>
+        <v>306.836</v>
       </c>
       <c r="C30" s="2" t="n">
-        <v>191.725</v>
+        <v>185.674</v>
       </c>
       <c r="D30" s="2" t="n"/>
       <c r="E30" s="2" t="n"/>
@@ -2685,10 +2685,10 @@
         </is>
       </c>
       <c r="B31" s="2" t="n">
-        <v>267.543</v>
+        <v>306.836</v>
       </c>
       <c r="C31" s="2" t="n">
-        <v>182.725</v>
+        <v>176.674</v>
       </c>
       <c r="D31" s="2" t="n"/>
       <c r="E31" s="2" t="n"/>
@@ -2702,10 +2702,10 @@
         </is>
       </c>
       <c r="B32" s="2" t="n">
-        <v>267.543</v>
+        <v>306.836</v>
       </c>
       <c r="C32" s="2" t="n">
-        <v>173.725</v>
+        <v>167.674</v>
       </c>
       <c r="D32" s="2" t="n"/>
       <c r="E32" s="2" t="n"/>
@@ -2719,10 +2719,10 @@
         </is>
       </c>
       <c r="B33" s="2" t="n">
-        <v>267.543</v>
+        <v>306.836</v>
       </c>
       <c r="C33" s="2" t="n">
-        <v>164.725</v>
+        <v>158.674</v>
       </c>
       <c r="D33" s="2" t="n"/>
       <c r="E33" s="2" t="n"/>
@@ -2736,10 +2736,10 @@
         </is>
       </c>
       <c r="B34" s="2" t="n">
-        <v>267.543</v>
+        <v>306.836</v>
       </c>
       <c r="C34" s="2" t="n">
-        <v>155.725</v>
+        <v>149.674</v>
       </c>
       <c r="D34" s="2" t="n"/>
       <c r="E34" s="2" t="n"/>
@@ -2753,10 +2753,10 @@
         </is>
       </c>
       <c r="B35" s="2" t="n">
-        <v>267.543</v>
+        <v>306.836</v>
       </c>
       <c r="C35" s="2" t="n">
-        <v>146.725</v>
+        <v>140.674</v>
       </c>
       <c r="D35" s="2" t="n"/>
       <c r="E35" s="2" t="n"/>
@@ -2770,10 +2770,10 @@
         </is>
       </c>
       <c r="B36" s="2" t="n">
-        <v>267.543</v>
+        <v>306.836</v>
       </c>
       <c r="C36" s="2" t="n">
-        <v>137.725</v>
+        <v>131.674</v>
       </c>
       <c r="D36" s="2" t="n"/>
       <c r="E36" s="2" t="n"/>
@@ -2787,10 +2787,10 @@
         </is>
       </c>
       <c r="B37" s="2" t="n">
-        <v>267.543</v>
+        <v>306.836</v>
       </c>
       <c r="C37" s="2" t="n">
-        <v>128.725</v>
+        <v>122.674</v>
       </c>
       <c r="D37" s="2" t="n"/>
       <c r="E37" s="2" t="n"/>
@@ -2804,10 +2804,10 @@
         </is>
       </c>
       <c r="B38" s="2" t="n">
-        <v>276.543</v>
+        <v>315.836</v>
       </c>
       <c r="C38" s="2" t="n">
-        <v>227.725</v>
+        <v>221.674</v>
       </c>
       <c r="D38" s="2" t="n"/>
       <c r="E38" s="2" t="n"/>
@@ -2821,10 +2821,10 @@
         </is>
       </c>
       <c r="B39" s="2" t="n">
-        <v>276.543</v>
+        <v>315.836</v>
       </c>
       <c r="C39" s="2" t="n">
-        <v>218.725</v>
+        <v>212.674</v>
       </c>
       <c r="D39" s="2" t="n"/>
       <c r="E39" s="2" t="n"/>
@@ -2838,10 +2838,10 @@
         </is>
       </c>
       <c r="B40" s="2" t="n">
-        <v>276.543</v>
+        <v>315.836</v>
       </c>
       <c r="C40" s="2" t="n">
-        <v>209.725</v>
+        <v>203.674</v>
       </c>
       <c r="D40" s="2" t="n"/>
       <c r="E40" s="2" t="n"/>
@@ -2855,10 +2855,10 @@
         </is>
       </c>
       <c r="B41" s="2" t="n">
-        <v>276.543</v>
+        <v>315.836</v>
       </c>
       <c r="C41" s="2" t="n">
-        <v>200.725</v>
+        <v>194.674</v>
       </c>
       <c r="D41" s="2" t="n"/>
       <c r="E41" s="2" t="n"/>
@@ -2872,10 +2872,10 @@
         </is>
       </c>
       <c r="B42" s="2" t="n">
-        <v>276.543</v>
+        <v>315.836</v>
       </c>
       <c r="C42" s="2" t="n">
-        <v>191.725</v>
+        <v>185.674</v>
       </c>
       <c r="D42" s="2" t="n"/>
       <c r="E42" s="2" t="n"/>
@@ -2889,10 +2889,10 @@
         </is>
       </c>
       <c r="B43" s="2" t="n">
-        <v>276.543</v>
+        <v>315.836</v>
       </c>
       <c r="C43" s="2" t="n">
-        <v>182.725</v>
+        <v>176.674</v>
       </c>
       <c r="D43" s="2" t="n"/>
       <c r="E43" s="2" t="n"/>
@@ -2906,10 +2906,10 @@
         </is>
       </c>
       <c r="B44" s="2" t="n">
-        <v>276.543</v>
+        <v>315.836</v>
       </c>
       <c r="C44" s="2" t="n">
-        <v>173.725</v>
+        <v>167.674</v>
       </c>
       <c r="D44" s="2" t="n"/>
       <c r="E44" s="2" t="n"/>
@@ -2923,10 +2923,10 @@
         </is>
       </c>
       <c r="B45" s="2" t="n">
-        <v>276.543</v>
+        <v>315.836</v>
       </c>
       <c r="C45" s="2" t="n">
-        <v>164.725</v>
+        <v>158.674</v>
       </c>
       <c r="D45" s="2" t="n"/>
       <c r="E45" s="2" t="n"/>
@@ -2940,10 +2940,10 @@
         </is>
       </c>
       <c r="B46" s="2" t="n">
-        <v>276.543</v>
+        <v>315.836</v>
       </c>
       <c r="C46" s="2" t="n">
-        <v>155.725</v>
+        <v>149.674</v>
       </c>
       <c r="D46" s="2" t="n"/>
       <c r="E46" s="2" t="n"/>
@@ -2957,10 +2957,10 @@
         </is>
       </c>
       <c r="B47" s="2" t="n">
-        <v>276.543</v>
+        <v>315.836</v>
       </c>
       <c r="C47" s="2" t="n">
-        <v>146.725</v>
+        <v>140.674</v>
       </c>
       <c r="D47" s="2" t="n"/>
       <c r="E47" s="2" t="n"/>
@@ -2974,10 +2974,10 @@
         </is>
       </c>
       <c r="B48" s="2" t="n">
-        <v>276.543</v>
+        <v>315.836</v>
       </c>
       <c r="C48" s="2" t="n">
-        <v>137.725</v>
+        <v>131.674</v>
       </c>
       <c r="D48" s="2" t="n"/>
       <c r="E48" s="2" t="n"/>
@@ -2991,10 +2991,10 @@
         </is>
       </c>
       <c r="B49" s="2" t="n">
-        <v>276.543</v>
+        <v>315.836</v>
       </c>
       <c r="C49" s="2" t="n">
-        <v>128.725</v>
+        <v>122.674</v>
       </c>
       <c r="D49" s="2" t="n"/>
       <c r="E49" s="2" t="n"/>
@@ -3008,10 +3008,10 @@
         </is>
       </c>
       <c r="B50" s="2" t="n">
-        <v>285.543</v>
+        <v>324.836</v>
       </c>
       <c r="C50" s="2" t="n">
-        <v>227.725</v>
+        <v>221.674</v>
       </c>
       <c r="D50" s="2" t="n"/>
       <c r="E50" s="2" t="n"/>
@@ -3025,10 +3025,10 @@
         </is>
       </c>
       <c r="B51" s="2" t="n">
-        <v>285.543</v>
+        <v>324.836</v>
       </c>
       <c r="C51" s="2" t="n">
-        <v>218.725</v>
+        <v>212.674</v>
       </c>
       <c r="D51" s="2" t="n"/>
       <c r="E51" s="2" t="n"/>
@@ -3042,10 +3042,10 @@
         </is>
       </c>
       <c r="B52" s="2" t="n">
-        <v>285.543</v>
+        <v>324.836</v>
       </c>
       <c r="C52" s="2" t="n">
-        <v>209.725</v>
+        <v>203.674</v>
       </c>
       <c r="D52" s="2" t="n"/>
       <c r="E52" s="2" t="n"/>
@@ -3059,10 +3059,10 @@
         </is>
       </c>
       <c r="B53" s="2" t="n">
-        <v>285.543</v>
+        <v>324.836</v>
       </c>
       <c r="C53" s="2" t="n">
-        <v>200.725</v>
+        <v>194.674</v>
       </c>
       <c r="D53" s="2" t="n"/>
       <c r="E53" s="2" t="n"/>
@@ -3076,10 +3076,10 @@
         </is>
       </c>
       <c r="B54" s="2" t="n">
-        <v>285.543</v>
+        <v>324.836</v>
       </c>
       <c r="C54" s="2" t="n">
-        <v>191.725</v>
+        <v>185.674</v>
       </c>
       <c r="D54" s="2" t="n"/>
       <c r="E54" s="2" t="n"/>
@@ -3093,10 +3093,10 @@
         </is>
       </c>
       <c r="B55" s="2" t="n">
-        <v>285.543</v>
+        <v>324.836</v>
       </c>
       <c r="C55" s="2" t="n">
-        <v>182.725</v>
+        <v>176.674</v>
       </c>
       <c r="D55" s="2" t="n"/>
       <c r="E55" s="2" t="n"/>
@@ -3110,10 +3110,10 @@
         </is>
       </c>
       <c r="B56" s="2" t="n">
-        <v>285.543</v>
+        <v>324.836</v>
       </c>
       <c r="C56" s="2" t="n">
-        <v>173.725</v>
+        <v>167.674</v>
       </c>
       <c r="D56" s="2" t="n"/>
       <c r="E56" s="2" t="n"/>
@@ -3127,10 +3127,10 @@
         </is>
       </c>
       <c r="B57" s="2" t="n">
-        <v>285.543</v>
+        <v>324.836</v>
       </c>
       <c r="C57" s="2" t="n">
-        <v>164.725</v>
+        <v>158.674</v>
       </c>
       <c r="D57" s="2" t="n"/>
       <c r="E57" s="2" t="n"/>
@@ -3144,10 +3144,10 @@
         </is>
       </c>
       <c r="B58" s="2" t="n">
-        <v>285.543</v>
+        <v>324.836</v>
       </c>
       <c r="C58" s="2" t="n">
-        <v>155.725</v>
+        <v>149.674</v>
       </c>
       <c r="D58" s="2" t="n"/>
       <c r="E58" s="2" t="n"/>
@@ -3161,10 +3161,10 @@
         </is>
       </c>
       <c r="B59" s="2" t="n">
-        <v>285.543</v>
+        <v>324.836</v>
       </c>
       <c r="C59" s="2" t="n">
-        <v>146.725</v>
+        <v>140.674</v>
       </c>
       <c r="D59" s="2" t="n"/>
       <c r="E59" s="2" t="n"/>
@@ -3178,10 +3178,10 @@
         </is>
       </c>
       <c r="B60" s="2" t="n">
-        <v>285.543</v>
+        <v>324.836</v>
       </c>
       <c r="C60" s="2" t="n">
-        <v>137.725</v>
+        <v>131.674</v>
       </c>
       <c r="D60" s="2" t="n"/>
       <c r="E60" s="2" t="n"/>
@@ -3195,10 +3195,10 @@
         </is>
       </c>
       <c r="B61" s="2" t="n">
-        <v>285.543</v>
+        <v>324.836</v>
       </c>
       <c r="C61" s="2" t="n">
-        <v>128.725</v>
+        <v>122.674</v>
       </c>
       <c r="D61" s="2" t="n"/>
       <c r="E61" s="2" t="n"/>
@@ -3212,10 +3212,10 @@
         </is>
       </c>
       <c r="B62" s="2" t="n">
-        <v>294.543</v>
+        <v>333.836</v>
       </c>
       <c r="C62" s="2" t="n">
-        <v>227.725</v>
+        <v>221.674</v>
       </c>
       <c r="D62" s="2" t="n"/>
       <c r="E62" s="2" t="n"/>
@@ -3229,10 +3229,10 @@
         </is>
       </c>
       <c r="B63" s="2" t="n">
-        <v>294.543</v>
+        <v>333.836</v>
       </c>
       <c r="C63" s="2" t="n">
-        <v>218.725</v>
+        <v>212.674</v>
       </c>
       <c r="D63" s="2" t="n"/>
       <c r="E63" s="2" t="n"/>
@@ -3246,10 +3246,10 @@
         </is>
       </c>
       <c r="B64" s="2" t="n">
-        <v>294.543</v>
+        <v>333.836</v>
       </c>
       <c r="C64" s="2" t="n">
-        <v>209.725</v>
+        <v>203.674</v>
       </c>
       <c r="D64" s="2" t="n"/>
       <c r="E64" s="2" t="n"/>
@@ -3263,10 +3263,10 @@
         </is>
       </c>
       <c r="B65" s="2" t="n">
-        <v>294.543</v>
+        <v>333.836</v>
       </c>
       <c r="C65" s="2" t="n">
-        <v>200.725</v>
+        <v>194.674</v>
       </c>
       <c r="D65" s="2" t="n"/>
       <c r="E65" s="2" t="n"/>
@@ -3280,10 +3280,10 @@
         </is>
       </c>
       <c r="B66" s="2" t="n">
-        <v>294.543</v>
+        <v>333.836</v>
       </c>
       <c r="C66" s="2" t="n">
-        <v>191.725</v>
+        <v>185.674</v>
       </c>
       <c r="D66" s="2" t="n"/>
       <c r="E66" s="2" t="n"/>
@@ -3297,10 +3297,10 @@
         </is>
       </c>
       <c r="B67" s="2" t="n">
-        <v>294.543</v>
+        <v>333.836</v>
       </c>
       <c r="C67" s="2" t="n">
-        <v>182.725</v>
+        <v>176.674</v>
       </c>
       <c r="D67" s="2" t="n"/>
       <c r="E67" s="2" t="n"/>
@@ -3314,10 +3314,10 @@
         </is>
       </c>
       <c r="B68" s="2" t="n">
-        <v>294.543</v>
+        <v>333.836</v>
       </c>
       <c r="C68" s="2" t="n">
-        <v>173.725</v>
+        <v>167.674</v>
       </c>
       <c r="D68" s="2" t="n"/>
       <c r="E68" s="2" t="n"/>
@@ -3331,10 +3331,10 @@
         </is>
       </c>
       <c r="B69" s="2" t="n">
-        <v>294.543</v>
+        <v>333.836</v>
       </c>
       <c r="C69" s="2" t="n">
-        <v>164.725</v>
+        <v>158.674</v>
       </c>
       <c r="D69" s="2" t="n"/>
       <c r="E69" s="2" t="n"/>
@@ -3348,10 +3348,10 @@
         </is>
       </c>
       <c r="B70" s="2" t="n">
-        <v>294.543</v>
+        <v>333.836</v>
       </c>
       <c r="C70" s="2" t="n">
-        <v>155.725</v>
+        <v>149.674</v>
       </c>
       <c r="D70" s="2" t="n"/>
       <c r="E70" s="2" t="n"/>
@@ -3365,10 +3365,10 @@
         </is>
       </c>
       <c r="B71" s="2" t="n">
-        <v>294.543</v>
+        <v>333.836</v>
       </c>
       <c r="C71" s="2" t="n">
-        <v>146.725</v>
+        <v>140.674</v>
       </c>
       <c r="D71" s="2" t="n"/>
       <c r="E71" s="2" t="n"/>
@@ -3382,10 +3382,10 @@
         </is>
       </c>
       <c r="B72" s="2" t="n">
-        <v>294.543</v>
+        <v>333.836</v>
       </c>
       <c r="C72" s="2" t="n">
-        <v>137.725</v>
+        <v>131.674</v>
       </c>
       <c r="D72" s="2" t="n"/>
       <c r="E72" s="2" t="n"/>
@@ -3399,10 +3399,10 @@
         </is>
       </c>
       <c r="B73" s="2" t="n">
-        <v>294.543</v>
+        <v>333.836</v>
       </c>
       <c r="C73" s="2" t="n">
-        <v>128.725</v>
+        <v>122.674</v>
       </c>
       <c r="D73" s="2" t="n"/>
       <c r="E73" s="2" t="n"/>
@@ -3416,10 +3416,10 @@
         </is>
       </c>
       <c r="B74" s="2" t="n">
-        <v>303.543</v>
+        <v>342.836</v>
       </c>
       <c r="C74" s="2" t="n">
-        <v>227.725</v>
+        <v>221.674</v>
       </c>
       <c r="D74" s="2" t="n"/>
       <c r="E74" s="2" t="n"/>
@@ -3433,10 +3433,10 @@
         </is>
       </c>
       <c r="B75" s="2" t="n">
-        <v>303.543</v>
+        <v>342.836</v>
       </c>
       <c r="C75" s="2" t="n">
-        <v>218.725</v>
+        <v>212.674</v>
       </c>
       <c r="D75" s="2" t="n"/>
       <c r="E75" s="2" t="n"/>
@@ -3450,10 +3450,10 @@
         </is>
       </c>
       <c r="B76" s="2" t="n">
-        <v>303.543</v>
+        <v>342.836</v>
       </c>
       <c r="C76" s="2" t="n">
-        <v>209.725</v>
+        <v>203.674</v>
       </c>
       <c r="D76" s="2" t="n"/>
       <c r="E76" s="2" t="n"/>
@@ -3467,10 +3467,10 @@
         </is>
       </c>
       <c r="B77" s="2" t="n">
-        <v>303.543</v>
+        <v>342.836</v>
       </c>
       <c r="C77" s="2" t="n">
-        <v>200.725</v>
+        <v>194.674</v>
       </c>
       <c r="D77" s="2" t="n"/>
       <c r="E77" s="2" t="n"/>
@@ -3484,10 +3484,10 @@
         </is>
       </c>
       <c r="B78" s="2" t="n">
-        <v>303.543</v>
+        <v>342.836</v>
       </c>
       <c r="C78" s="2" t="n">
-        <v>191.725</v>
+        <v>185.674</v>
       </c>
       <c r="D78" s="2" t="n"/>
       <c r="E78" s="2" t="n"/>
@@ -3501,10 +3501,10 @@
         </is>
       </c>
       <c r="B79" s="2" t="n">
-        <v>303.543</v>
+        <v>342.836</v>
       </c>
       <c r="C79" s="2" t="n">
-        <v>182.725</v>
+        <v>176.674</v>
       </c>
       <c r="D79" s="2" t="n"/>
       <c r="E79" s="2" t="n"/>
@@ -3518,10 +3518,10 @@
         </is>
       </c>
       <c r="B80" s="2" t="n">
-        <v>303.543</v>
+        <v>342.836</v>
       </c>
       <c r="C80" s="2" t="n">
-        <v>173.725</v>
+        <v>167.674</v>
       </c>
       <c r="D80" s="2" t="n"/>
       <c r="E80" s="2" t="n"/>
@@ -3535,10 +3535,10 @@
         </is>
       </c>
       <c r="B81" s="2" t="n">
-        <v>303.543</v>
+        <v>342.836</v>
       </c>
       <c r="C81" s="2" t="n">
-        <v>164.725</v>
+        <v>158.674</v>
       </c>
       <c r="D81" s="2" t="n"/>
       <c r="E81" s="2" t="n"/>
@@ -3552,10 +3552,10 @@
         </is>
       </c>
       <c r="B82" s="2" t="n">
-        <v>303.543</v>
+        <v>342.836</v>
       </c>
       <c r="C82" s="2" t="n">
-        <v>155.725</v>
+        <v>149.674</v>
       </c>
       <c r="D82" s="2" t="n"/>
       <c r="E82" s="2" t="n"/>
@@ -3569,10 +3569,10 @@
         </is>
       </c>
       <c r="B83" s="2" t="n">
-        <v>303.543</v>
+        <v>342.836</v>
       </c>
       <c r="C83" s="2" t="n">
-        <v>146.725</v>
+        <v>140.674</v>
       </c>
       <c r="D83" s="2" t="n"/>
       <c r="E83" s="2" t="n"/>
@@ -3586,10 +3586,10 @@
         </is>
       </c>
       <c r="B84" s="2" t="n">
-        <v>303.543</v>
+        <v>342.836</v>
       </c>
       <c r="C84" s="2" t="n">
-        <v>137.725</v>
+        <v>131.674</v>
       </c>
       <c r="D84" s="2" t="n"/>
       <c r="E84" s="2" t="n"/>
@@ -3603,10 +3603,10 @@
         </is>
       </c>
       <c r="B85" s="2" t="n">
-        <v>303.543</v>
+        <v>342.836</v>
       </c>
       <c r="C85" s="2" t="n">
-        <v>128.725</v>
+        <v>122.674</v>
       </c>
       <c r="D85" s="2" t="n"/>
       <c r="E85" s="2" t="n"/>
@@ -3620,10 +3620,10 @@
         </is>
       </c>
       <c r="B86" s="2" t="n">
-        <v>312.543</v>
+        <v>351.836</v>
       </c>
       <c r="C86" s="2" t="n">
-        <v>227.725</v>
+        <v>221.674</v>
       </c>
       <c r="D86" s="2" t="n"/>
       <c r="E86" s="2" t="n"/>
@@ -3637,10 +3637,10 @@
         </is>
       </c>
       <c r="B87" s="2" t="n">
-        <v>312.543</v>
+        <v>351.836</v>
       </c>
       <c r="C87" s="2" t="n">
-        <v>218.725</v>
+        <v>212.674</v>
       </c>
       <c r="D87" s="2" t="n"/>
       <c r="E87" s="2" t="n"/>
@@ -3654,10 +3654,10 @@
         </is>
       </c>
       <c r="B88" s="2" t="n">
-        <v>312.543</v>
+        <v>351.836</v>
       </c>
       <c r="C88" s="2" t="n">
-        <v>209.725</v>
+        <v>203.674</v>
       </c>
       <c r="D88" s="2" t="n"/>
       <c r="E88" s="2" t="n"/>
@@ -3671,10 +3671,10 @@
         </is>
       </c>
       <c r="B89" s="2" t="n">
-        <v>312.543</v>
+        <v>351.836</v>
       </c>
       <c r="C89" s="2" t="n">
-        <v>200.725</v>
+        <v>194.674</v>
       </c>
       <c r="D89" s="2" t="n"/>
       <c r="E89" s="2" t="n"/>
@@ -3688,10 +3688,10 @@
         </is>
       </c>
       <c r="B90" s="2" t="n">
-        <v>312.543</v>
+        <v>351.836</v>
       </c>
       <c r="C90" s="2" t="n">
-        <v>191.725</v>
+        <v>185.674</v>
       </c>
       <c r="D90" s="2" t="n"/>
       <c r="E90" s="2" t="n"/>
@@ -3705,10 +3705,10 @@
         </is>
       </c>
       <c r="B91" s="2" t="n">
-        <v>312.543</v>
+        <v>351.836</v>
       </c>
       <c r="C91" s="2" t="n">
-        <v>182.725</v>
+        <v>176.674</v>
       </c>
       <c r="D91" s="2" t="n"/>
       <c r="E91" s="2" t="n"/>
@@ -3722,10 +3722,10 @@
         </is>
       </c>
       <c r="B92" s="2" t="n">
-        <v>312.543</v>
+        <v>351.836</v>
       </c>
       <c r="C92" s="2" t="n">
-        <v>173.725</v>
+        <v>167.674</v>
       </c>
       <c r="D92" s="2" t="n"/>
       <c r="E92" s="2" t="n"/>
@@ -3739,10 +3739,10 @@
         </is>
       </c>
       <c r="B93" s="2" t="n">
-        <v>312.543</v>
+        <v>351.836</v>
       </c>
       <c r="C93" s="2" t="n">
-        <v>164.725</v>
+        <v>158.674</v>
       </c>
       <c r="D93" s="2" t="n"/>
       <c r="E93" s="2" t="n"/>
@@ -3756,10 +3756,10 @@
         </is>
       </c>
       <c r="B94" s="2" t="n">
-        <v>312.543</v>
+        <v>351.836</v>
       </c>
       <c r="C94" s="2" t="n">
-        <v>155.725</v>
+        <v>149.674</v>
       </c>
       <c r="D94" s="2" t="n"/>
       <c r="E94" s="2" t="n"/>
@@ -3773,10 +3773,10 @@
         </is>
       </c>
       <c r="B95" s="2" t="n">
-        <v>312.543</v>
+        <v>351.836</v>
       </c>
       <c r="C95" s="2" t="n">
-        <v>146.725</v>
+        <v>140.674</v>
       </c>
       <c r="D95" s="2" t="n"/>
       <c r="E95" s="2" t="n"/>
@@ -3790,10 +3790,10 @@
         </is>
       </c>
       <c r="B96" s="2" t="n">
-        <v>312.543</v>
+        <v>351.836</v>
       </c>
       <c r="C96" s="2" t="n">
-        <v>137.725</v>
+        <v>131.674</v>
       </c>
       <c r="D96" s="2" t="n"/>
       <c r="E96" s="2" t="n"/>
@@ -3807,10 +3807,10 @@
         </is>
       </c>
       <c r="B97" s="2" t="n">
-        <v>312.543</v>
+        <v>351.836</v>
       </c>
       <c r="C97" s="2" t="n">
-        <v>128.725</v>
+        <v>122.674</v>
       </c>
       <c r="D97" s="2" t="n"/>
       <c r="E97" s="2" t="n"/>
@@ -3884,10 +3884,10 @@
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>-229.636</v>
+        <v>-229.662</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>269.4</v>
+        <v>270.084</v>
       </c>
       <c r="D2" s="2" t="n"/>
       <c r="E2" s="2" t="n"/>
@@ -3901,10 +3901,10 @@
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>-229.636</v>
+        <v>-229.662</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>260.4</v>
+        <v>261.084</v>
       </c>
       <c r="D3" s="2" t="n"/>
       <c r="E3" s="2" t="n"/>
@@ -3918,10 +3918,10 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>-229.636</v>
+        <v>-229.662</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>251.4</v>
+        <v>252.084</v>
       </c>
       <c r="D4" s="2" t="n"/>
       <c r="E4" s="2" t="n"/>
@@ -3935,10 +3935,10 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>-229.636</v>
+        <v>-229.662</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>242.4</v>
+        <v>243.084</v>
       </c>
       <c r="D5" s="2" t="n"/>
       <c r="E5" s="2" t="n"/>
@@ -3952,10 +3952,10 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>-229.636</v>
+        <v>-229.662</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>233.4</v>
+        <v>234.084</v>
       </c>
       <c r="D6" s="2" t="n"/>
       <c r="E6" s="2" t="n"/>
@@ -3969,10 +3969,10 @@
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>-229.636</v>
+        <v>-229.662</v>
       </c>
       <c r="C7" s="2" t="n">
-        <v>224.4</v>
+        <v>225.084</v>
       </c>
       <c r="D7" s="2" t="n"/>
       <c r="E7" s="2" t="n"/>
@@ -3986,10 +3986,10 @@
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>-229.636</v>
+        <v>-229.662</v>
       </c>
       <c r="C8" s="2" t="n">
-        <v>215.4</v>
+        <v>216.084</v>
       </c>
       <c r="D8" s="2" t="n"/>
       <c r="E8" s="2" t="n"/>
@@ -4003,10 +4003,10 @@
         </is>
       </c>
       <c r="B9" s="2" t="n">
-        <v>-229.636</v>
+        <v>-229.662</v>
       </c>
       <c r="C9" s="2" t="n">
-        <v>206.4</v>
+        <v>207.084</v>
       </c>
       <c r="D9" s="2" t="n"/>
       <c r="E9" s="2" t="n"/>
@@ -4020,10 +4020,10 @@
         </is>
       </c>
       <c r="B10" s="2" t="n">
-        <v>-229.636</v>
+        <v>-229.662</v>
       </c>
       <c r="C10" s="2" t="n">
-        <v>197.4</v>
+        <v>198.084</v>
       </c>
       <c r="D10" s="2" t="n"/>
       <c r="E10" s="2" t="n"/>
@@ -4037,10 +4037,10 @@
         </is>
       </c>
       <c r="B11" s="2" t="n">
-        <v>-229.636</v>
+        <v>-229.662</v>
       </c>
       <c r="C11" s="2" t="n">
-        <v>188.4</v>
+        <v>189.084</v>
       </c>
       <c r="D11" s="2" t="n"/>
       <c r="E11" s="2" t="n"/>
@@ -4054,10 +4054,10 @@
         </is>
       </c>
       <c r="B12" s="2" t="n">
-        <v>-229.636</v>
+        <v>-229.662</v>
       </c>
       <c r="C12" s="2" t="n">
-        <v>179.4</v>
+        <v>180.084</v>
       </c>
       <c r="D12" s="2" t="n"/>
       <c r="E12" s="2" t="n"/>
@@ -4071,10 +4071,10 @@
         </is>
       </c>
       <c r="B13" s="2" t="n">
-        <v>-229.636</v>
+        <v>-229.662</v>
       </c>
       <c r="C13" s="2" t="n">
-        <v>170.4</v>
+        <v>171.084</v>
       </c>
       <c r="D13" s="2" t="n"/>
       <c r="E13" s="2" t="n"/>
@@ -4088,10 +4088,10 @@
         </is>
       </c>
       <c r="B14" s="2" t="n">
-        <v>-238.636</v>
+        <v>-238.662</v>
       </c>
       <c r="C14" s="2" t="n">
-        <v>269.4</v>
+        <v>270.084</v>
       </c>
       <c r="D14" s="2" t="n"/>
       <c r="E14" s="2" t="n"/>
@@ -4105,10 +4105,10 @@
         </is>
       </c>
       <c r="B15" s="2" t="n">
-        <v>-238.636</v>
+        <v>-238.662</v>
       </c>
       <c r="C15" s="2" t="n">
-        <v>260.4</v>
+        <v>261.084</v>
       </c>
       <c r="D15" s="2" t="n"/>
       <c r="E15" s="2" t="n"/>
@@ -4122,10 +4122,10 @@
         </is>
       </c>
       <c r="B16" s="2" t="n">
-        <v>-238.636</v>
+        <v>-238.662</v>
       </c>
       <c r="C16" s="2" t="n">
-        <v>251.4</v>
+        <v>252.084</v>
       </c>
       <c r="D16" s="2" t="n"/>
       <c r="E16" s="2" t="n"/>
@@ -4139,10 +4139,10 @@
         </is>
       </c>
       <c r="B17" s="2" t="n">
-        <v>-238.636</v>
+        <v>-238.662</v>
       </c>
       <c r="C17" s="2" t="n">
-        <v>242.4</v>
+        <v>243.084</v>
       </c>
       <c r="D17" s="2" t="n"/>
       <c r="E17" s="2" t="n"/>
@@ -4156,10 +4156,10 @@
         </is>
       </c>
       <c r="B18" s="2" t="n">
-        <v>-238.636</v>
+        <v>-238.662</v>
       </c>
       <c r="C18" s="2" t="n">
-        <v>233.4</v>
+        <v>234.084</v>
       </c>
       <c r="D18" s="2" t="n"/>
       <c r="E18" s="2" t="n"/>
@@ -4173,10 +4173,10 @@
         </is>
       </c>
       <c r="B19" s="2" t="n">
-        <v>-238.636</v>
+        <v>-238.662</v>
       </c>
       <c r="C19" s="2" t="n">
-        <v>224.4</v>
+        <v>225.084</v>
       </c>
       <c r="D19" s="2" t="n"/>
       <c r="E19" s="2" t="n"/>
@@ -4190,10 +4190,10 @@
         </is>
       </c>
       <c r="B20" s="2" t="n">
-        <v>-238.636</v>
+        <v>-238.662</v>
       </c>
       <c r="C20" s="2" t="n">
-        <v>215.4</v>
+        <v>216.084</v>
       </c>
       <c r="D20" s="2" t="n"/>
       <c r="E20" s="2" t="n"/>
@@ -4207,10 +4207,10 @@
         </is>
       </c>
       <c r="B21" s="2" t="n">
-        <v>-238.636</v>
+        <v>-238.662</v>
       </c>
       <c r="C21" s="2" t="n">
-        <v>206.4</v>
+        <v>207.084</v>
       </c>
       <c r="D21" s="2" t="n"/>
       <c r="E21" s="2" t="n"/>
@@ -4224,10 +4224,10 @@
         </is>
       </c>
       <c r="B22" s="2" t="n">
-        <v>-238.636</v>
+        <v>-238.662</v>
       </c>
       <c r="C22" s="2" t="n">
-        <v>197.4</v>
+        <v>198.084</v>
       </c>
       <c r="D22" s="2" t="n"/>
       <c r="E22" s="2" t="n"/>
@@ -4241,10 +4241,10 @@
         </is>
       </c>
       <c r="B23" s="2" t="n">
-        <v>-238.636</v>
+        <v>-238.662</v>
       </c>
       <c r="C23" s="2" t="n">
-        <v>188.4</v>
+        <v>189.084</v>
       </c>
       <c r="D23" s="2" t="n"/>
       <c r="E23" s="2" t="n"/>
@@ -4258,10 +4258,10 @@
         </is>
       </c>
       <c r="B24" s="2" t="n">
-        <v>-238.636</v>
+        <v>-238.662</v>
       </c>
       <c r="C24" s="2" t="n">
-        <v>179.4</v>
+        <v>180.084</v>
       </c>
       <c r="D24" s="2" t="n"/>
       <c r="E24" s="2" t="n"/>
@@ -4275,10 +4275,10 @@
         </is>
       </c>
       <c r="B25" s="2" t="n">
-        <v>-238.636</v>
+        <v>-238.662</v>
       </c>
       <c r="C25" s="2" t="n">
-        <v>170.4</v>
+        <v>171.084</v>
       </c>
       <c r="D25" s="2" t="n"/>
       <c r="E25" s="2" t="n"/>
@@ -4292,10 +4292,10 @@
         </is>
       </c>
       <c r="B26" s="2" t="n">
-        <v>-247.636</v>
+        <v>-247.662</v>
       </c>
       <c r="C26" s="2" t="n">
-        <v>269.4</v>
+        <v>270.084</v>
       </c>
       <c r="D26" s="2" t="n"/>
       <c r="E26" s="2" t="n"/>
@@ -4309,10 +4309,10 @@
         </is>
       </c>
       <c r="B27" s="2" t="n">
-        <v>-247.636</v>
+        <v>-247.662</v>
       </c>
       <c r="C27" s="2" t="n">
-        <v>260.4</v>
+        <v>261.084</v>
       </c>
       <c r="D27" s="2" t="n"/>
       <c r="E27" s="2" t="n"/>
@@ -4326,10 +4326,10 @@
         </is>
       </c>
       <c r="B28" s="2" t="n">
-        <v>-247.636</v>
+        <v>-247.662</v>
       </c>
       <c r="C28" s="2" t="n">
-        <v>251.4</v>
+        <v>252.084</v>
       </c>
       <c r="D28" s="2" t="n"/>
       <c r="E28" s="2" t="n"/>
@@ -4343,10 +4343,10 @@
         </is>
       </c>
       <c r="B29" s="2" t="n">
-        <v>-247.636</v>
+        <v>-247.662</v>
       </c>
       <c r="C29" s="2" t="n">
-        <v>242.4</v>
+        <v>243.084</v>
       </c>
       <c r="D29" s="2" t="n"/>
       <c r="E29" s="2" t="n"/>
@@ -4360,10 +4360,10 @@
         </is>
       </c>
       <c r="B30" s="2" t="n">
-        <v>-247.636</v>
+        <v>-247.662</v>
       </c>
       <c r="C30" s="2" t="n">
-        <v>233.4</v>
+        <v>234.084</v>
       </c>
       <c r="D30" s="2" t="n"/>
       <c r="E30" s="2" t="n"/>
@@ -4377,10 +4377,10 @@
         </is>
       </c>
       <c r="B31" s="2" t="n">
-        <v>-247.636</v>
+        <v>-247.662</v>
       </c>
       <c r="C31" s="2" t="n">
-        <v>224.4</v>
+        <v>225.084</v>
       </c>
       <c r="D31" s="2" t="n"/>
       <c r="E31" s="2" t="n"/>
@@ -4394,10 +4394,10 @@
         </is>
       </c>
       <c r="B32" s="2" t="n">
-        <v>-247.636</v>
+        <v>-247.662</v>
       </c>
       <c r="C32" s="2" t="n">
-        <v>215.4</v>
+        <v>216.084</v>
       </c>
       <c r="D32" s="2" t="n"/>
       <c r="E32" s="2" t="n"/>
@@ -4411,10 +4411,10 @@
         </is>
       </c>
       <c r="B33" s="2" t="n">
-        <v>-247.636</v>
+        <v>-247.662</v>
       </c>
       <c r="C33" s="2" t="n">
-        <v>206.4</v>
+        <v>207.084</v>
       </c>
       <c r="D33" s="2" t="n"/>
       <c r="E33" s="2" t="n"/>
@@ -4428,10 +4428,10 @@
         </is>
       </c>
       <c r="B34" s="2" t="n">
-        <v>-247.636</v>
+        <v>-247.662</v>
       </c>
       <c r="C34" s="2" t="n">
-        <v>197.4</v>
+        <v>198.084</v>
       </c>
       <c r="D34" s="2" t="n"/>
       <c r="E34" s="2" t="n"/>
@@ -4445,10 +4445,10 @@
         </is>
       </c>
       <c r="B35" s="2" t="n">
-        <v>-247.636</v>
+        <v>-247.662</v>
       </c>
       <c r="C35" s="2" t="n">
-        <v>188.4</v>
+        <v>189.084</v>
       </c>
       <c r="D35" s="2" t="n"/>
       <c r="E35" s="2" t="n"/>
@@ -4462,10 +4462,10 @@
         </is>
       </c>
       <c r="B36" s="2" t="n">
-        <v>-247.636</v>
+        <v>-247.662</v>
       </c>
       <c r="C36" s="2" t="n">
-        <v>179.4</v>
+        <v>180.084</v>
       </c>
       <c r="D36" s="2" t="n"/>
       <c r="E36" s="2" t="n"/>
@@ -4479,10 +4479,10 @@
         </is>
       </c>
       <c r="B37" s="2" t="n">
-        <v>-247.636</v>
+        <v>-247.662</v>
       </c>
       <c r="C37" s="2" t="n">
-        <v>170.4</v>
+        <v>171.084</v>
       </c>
       <c r="D37" s="2" t="n"/>
       <c r="E37" s="2" t="n"/>
@@ -4496,10 +4496,10 @@
         </is>
       </c>
       <c r="B38" s="2" t="n">
-        <v>-256.636</v>
+        <v>-256.662</v>
       </c>
       <c r="C38" s="2" t="n">
-        <v>269.4</v>
+        <v>270.084</v>
       </c>
       <c r="D38" s="2" t="n"/>
       <c r="E38" s="2" t="n"/>
@@ -4513,10 +4513,10 @@
         </is>
       </c>
       <c r="B39" s="2" t="n">
-        <v>-256.636</v>
+        <v>-256.662</v>
       </c>
       <c r="C39" s="2" t="n">
-        <v>260.4</v>
+        <v>261.084</v>
       </c>
       <c r="D39" s="2" t="n"/>
       <c r="E39" s="2" t="n"/>
@@ -4530,10 +4530,10 @@
         </is>
       </c>
       <c r="B40" s="2" t="n">
-        <v>-256.636</v>
+        <v>-256.662</v>
       </c>
       <c r="C40" s="2" t="n">
-        <v>251.4</v>
+        <v>252.084</v>
       </c>
       <c r="D40" s="2" t="n"/>
       <c r="E40" s="2" t="n"/>
@@ -4547,10 +4547,10 @@
         </is>
       </c>
       <c r="B41" s="2" t="n">
-        <v>-256.636</v>
+        <v>-256.662</v>
       </c>
       <c r="C41" s="2" t="n">
-        <v>242.4</v>
+        <v>243.084</v>
       </c>
       <c r="D41" s="2" t="n"/>
       <c r="E41" s="2" t="n"/>
@@ -4564,10 +4564,10 @@
         </is>
       </c>
       <c r="B42" s="2" t="n">
-        <v>-256.636</v>
+        <v>-256.662</v>
       </c>
       <c r="C42" s="2" t="n">
-        <v>233.4</v>
+        <v>234.084</v>
       </c>
       <c r="D42" s="2" t="n"/>
       <c r="E42" s="2" t="n"/>
@@ -4581,10 +4581,10 @@
         </is>
       </c>
       <c r="B43" s="2" t="n">
-        <v>-256.636</v>
+        <v>-256.662</v>
       </c>
       <c r="C43" s="2" t="n">
-        <v>224.4</v>
+        <v>225.084</v>
       </c>
       <c r="D43" s="2" t="n"/>
       <c r="E43" s="2" t="n"/>
@@ -4598,10 +4598,10 @@
         </is>
       </c>
       <c r="B44" s="2" t="n">
-        <v>-256.636</v>
+        <v>-256.662</v>
       </c>
       <c r="C44" s="2" t="n">
-        <v>215.4</v>
+        <v>216.084</v>
       </c>
       <c r="D44" s="2" t="n"/>
       <c r="E44" s="2" t="n"/>
@@ -4615,10 +4615,10 @@
         </is>
       </c>
       <c r="B45" s="2" t="n">
-        <v>-256.636</v>
+        <v>-256.662</v>
       </c>
       <c r="C45" s="2" t="n">
-        <v>206.4</v>
+        <v>207.084</v>
       </c>
       <c r="D45" s="2" t="n"/>
       <c r="E45" s="2" t="n"/>
@@ -4632,10 +4632,10 @@
         </is>
       </c>
       <c r="B46" s="2" t="n">
-        <v>-256.636</v>
+        <v>-256.662</v>
       </c>
       <c r="C46" s="2" t="n">
-        <v>197.4</v>
+        <v>198.084</v>
       </c>
       <c r="D46" s="2" t="n"/>
       <c r="E46" s="2" t="n"/>
@@ -4649,10 +4649,10 @@
         </is>
       </c>
       <c r="B47" s="2" t="n">
-        <v>-256.636</v>
+        <v>-256.662</v>
       </c>
       <c r="C47" s="2" t="n">
-        <v>188.4</v>
+        <v>189.084</v>
       </c>
       <c r="D47" s="2" t="n"/>
       <c r="E47" s="2" t="n"/>
@@ -4666,10 +4666,10 @@
         </is>
       </c>
       <c r="B48" s="2" t="n">
-        <v>-256.636</v>
+        <v>-256.662</v>
       </c>
       <c r="C48" s="2" t="n">
-        <v>179.4</v>
+        <v>180.084</v>
       </c>
       <c r="D48" s="2" t="n"/>
       <c r="E48" s="2" t="n"/>
@@ -4683,10 +4683,10 @@
         </is>
       </c>
       <c r="B49" s="2" t="n">
-        <v>-256.636</v>
+        <v>-256.662</v>
       </c>
       <c r="C49" s="2" t="n">
-        <v>170.4</v>
+        <v>171.084</v>
       </c>
       <c r="D49" s="2" t="n"/>
       <c r="E49" s="2" t="n"/>
@@ -4700,10 +4700,10 @@
         </is>
       </c>
       <c r="B50" s="2" t="n">
-        <v>-265.636</v>
+        <v>-265.662</v>
       </c>
       <c r="C50" s="2" t="n">
-        <v>269.4</v>
+        <v>270.084</v>
       </c>
       <c r="D50" s="2" t="n"/>
       <c r="E50" s="2" t="n"/>
@@ -4717,10 +4717,10 @@
         </is>
       </c>
       <c r="B51" s="2" t="n">
-        <v>-265.636</v>
+        <v>-265.662</v>
       </c>
       <c r="C51" s="2" t="n">
-        <v>260.4</v>
+        <v>261.084</v>
       </c>
       <c r="D51" s="2" t="n"/>
       <c r="E51" s="2" t="n"/>
@@ -4734,10 +4734,10 @@
         </is>
       </c>
       <c r="B52" s="2" t="n">
-        <v>-265.636</v>
+        <v>-265.662</v>
       </c>
       <c r="C52" s="2" t="n">
-        <v>251.4</v>
+        <v>252.084</v>
       </c>
       <c r="D52" s="2" t="n"/>
       <c r="E52" s="2" t="n"/>
@@ -4751,10 +4751,10 @@
         </is>
       </c>
       <c r="B53" s="2" t="n">
-        <v>-265.636</v>
+        <v>-265.662</v>
       </c>
       <c r="C53" s="2" t="n">
-        <v>242.4</v>
+        <v>243.084</v>
       </c>
       <c r="D53" s="2" t="n"/>
       <c r="E53" s="2" t="n"/>
@@ -4768,10 +4768,10 @@
         </is>
       </c>
       <c r="B54" s="2" t="n">
-        <v>-265.636</v>
+        <v>-265.662</v>
       </c>
       <c r="C54" s="2" t="n">
-        <v>233.4</v>
+        <v>234.084</v>
       </c>
       <c r="D54" s="2" t="n"/>
       <c r="E54" s="2" t="n"/>
@@ -4785,10 +4785,10 @@
         </is>
       </c>
       <c r="B55" s="2" t="n">
-        <v>-265.636</v>
+        <v>-265.662</v>
       </c>
       <c r="C55" s="2" t="n">
-        <v>224.4</v>
+        <v>225.084</v>
       </c>
       <c r="D55" s="2" t="n"/>
       <c r="E55" s="2" t="n"/>
@@ -4802,10 +4802,10 @@
         </is>
       </c>
       <c r="B56" s="2" t="n">
-        <v>-265.636</v>
+        <v>-265.662</v>
       </c>
       <c r="C56" s="2" t="n">
-        <v>215.4</v>
+        <v>216.084</v>
       </c>
       <c r="D56" s="2" t="n"/>
       <c r="E56" s="2" t="n"/>
@@ -4819,10 +4819,10 @@
         </is>
       </c>
       <c r="B57" s="2" t="n">
-        <v>-265.636</v>
+        <v>-265.662</v>
       </c>
       <c r="C57" s="2" t="n">
-        <v>206.4</v>
+        <v>207.084</v>
       </c>
       <c r="D57" s="2" t="n"/>
       <c r="E57" s="2" t="n"/>
@@ -4836,10 +4836,10 @@
         </is>
       </c>
       <c r="B58" s="2" t="n">
-        <v>-265.636</v>
+        <v>-265.662</v>
       </c>
       <c r="C58" s="2" t="n">
-        <v>197.4</v>
+        <v>198.084</v>
       </c>
       <c r="D58" s="2" t="n"/>
       <c r="E58" s="2" t="n"/>
@@ -4853,10 +4853,10 @@
         </is>
       </c>
       <c r="B59" s="2" t="n">
-        <v>-265.636</v>
+        <v>-265.662</v>
       </c>
       <c r="C59" s="2" t="n">
-        <v>188.4</v>
+        <v>189.084</v>
       </c>
       <c r="D59" s="2" t="n"/>
       <c r="E59" s="2" t="n"/>
@@ -4870,10 +4870,10 @@
         </is>
       </c>
       <c r="B60" s="2" t="n">
-        <v>-265.636</v>
+        <v>-265.662</v>
       </c>
       <c r="C60" s="2" t="n">
-        <v>179.4</v>
+        <v>180.084</v>
       </c>
       <c r="D60" s="2" t="n"/>
       <c r="E60" s="2" t="n"/>
@@ -4887,10 +4887,10 @@
         </is>
       </c>
       <c r="B61" s="2" t="n">
-        <v>-265.636</v>
+        <v>-265.662</v>
       </c>
       <c r="C61" s="2" t="n">
-        <v>170.4</v>
+        <v>171.084</v>
       </c>
       <c r="D61" s="2" t="n"/>
       <c r="E61" s="2" t="n"/>
@@ -4904,10 +4904,10 @@
         </is>
       </c>
       <c r="B62" s="2" t="n">
-        <v>-274.636</v>
+        <v>-274.662</v>
       </c>
       <c r="C62" s="2" t="n">
-        <v>269.4</v>
+        <v>270.084</v>
       </c>
       <c r="D62" s="2" t="n"/>
       <c r="E62" s="2" t="n"/>
@@ -4921,10 +4921,10 @@
         </is>
       </c>
       <c r="B63" s="2" t="n">
-        <v>-274.636</v>
+        <v>-274.662</v>
       </c>
       <c r="C63" s="2" t="n">
-        <v>260.4</v>
+        <v>261.084</v>
       </c>
       <c r="D63" s="2" t="n"/>
       <c r="E63" s="2" t="n"/>
@@ -4938,10 +4938,10 @@
         </is>
       </c>
       <c r="B64" s="2" t="n">
-        <v>-274.636</v>
+        <v>-274.662</v>
       </c>
       <c r="C64" s="2" t="n">
-        <v>251.4</v>
+        <v>252.084</v>
       </c>
       <c r="D64" s="2" t="n"/>
       <c r="E64" s="2" t="n"/>
@@ -4955,10 +4955,10 @@
         </is>
       </c>
       <c r="B65" s="2" t="n">
-        <v>-274.636</v>
+        <v>-274.662</v>
       </c>
       <c r="C65" s="2" t="n">
-        <v>242.4</v>
+        <v>243.084</v>
       </c>
       <c r="D65" s="2" t="n"/>
       <c r="E65" s="2" t="n"/>
@@ -4972,10 +4972,10 @@
         </is>
       </c>
       <c r="B66" s="2" t="n">
-        <v>-274.636</v>
+        <v>-274.662</v>
       </c>
       <c r="C66" s="2" t="n">
-        <v>233.4</v>
+        <v>234.084</v>
       </c>
       <c r="D66" s="2" t="n"/>
       <c r="E66" s="2" t="n"/>
@@ -4989,10 +4989,10 @@
         </is>
       </c>
       <c r="B67" s="2" t="n">
-        <v>-274.636</v>
+        <v>-274.662</v>
       </c>
       <c r="C67" s="2" t="n">
-        <v>224.4</v>
+        <v>225.084</v>
       </c>
       <c r="D67" s="2" t="n"/>
       <c r="E67" s="2" t="n"/>
@@ -5006,10 +5006,10 @@
         </is>
       </c>
       <c r="B68" s="2" t="n">
-        <v>-274.636</v>
+        <v>-274.662</v>
       </c>
       <c r="C68" s="2" t="n">
-        <v>215.4</v>
+        <v>216.084</v>
       </c>
       <c r="D68" s="2" t="n"/>
       <c r="E68" s="2" t="n"/>
@@ -5023,10 +5023,10 @@
         </is>
       </c>
       <c r="B69" s="2" t="n">
-        <v>-274.636</v>
+        <v>-274.662</v>
       </c>
       <c r="C69" s="2" t="n">
-        <v>206.4</v>
+        <v>207.084</v>
       </c>
       <c r="D69" s="2" t="n"/>
       <c r="E69" s="2" t="n"/>
@@ -5040,10 +5040,10 @@
         </is>
       </c>
       <c r="B70" s="2" t="n">
-        <v>-274.636</v>
+        <v>-274.662</v>
       </c>
       <c r="C70" s="2" t="n">
-        <v>197.4</v>
+        <v>198.084</v>
       </c>
       <c r="D70" s="2" t="n"/>
       <c r="E70" s="2" t="n"/>
@@ -5057,10 +5057,10 @@
         </is>
       </c>
       <c r="B71" s="2" t="n">
-        <v>-274.636</v>
+        <v>-274.662</v>
       </c>
       <c r="C71" s="2" t="n">
-        <v>188.4</v>
+        <v>189.084</v>
       </c>
       <c r="D71" s="2" t="n"/>
       <c r="E71" s="2" t="n"/>
@@ -5074,10 +5074,10 @@
         </is>
       </c>
       <c r="B72" s="2" t="n">
-        <v>-274.636</v>
+        <v>-274.662</v>
       </c>
       <c r="C72" s="2" t="n">
-        <v>179.4</v>
+        <v>180.084</v>
       </c>
       <c r="D72" s="2" t="n"/>
       <c r="E72" s="2" t="n"/>
@@ -5091,10 +5091,10 @@
         </is>
       </c>
       <c r="B73" s="2" t="n">
-        <v>-274.636</v>
+        <v>-274.662</v>
       </c>
       <c r="C73" s="2" t="n">
-        <v>170.4</v>
+        <v>171.084</v>
       </c>
       <c r="D73" s="2" t="n"/>
       <c r="E73" s="2" t="n"/>
@@ -5108,10 +5108,10 @@
         </is>
       </c>
       <c r="B74" s="2" t="n">
-        <v>-283.636</v>
+        <v>-283.662</v>
       </c>
       <c r="C74" s="2" t="n">
-        <v>269.4</v>
+        <v>270.084</v>
       </c>
       <c r="D74" s="2" t="n"/>
       <c r="E74" s="2" t="n"/>
@@ -5125,10 +5125,10 @@
         </is>
       </c>
       <c r="B75" s="2" t="n">
-        <v>-283.636</v>
+        <v>-283.662</v>
       </c>
       <c r="C75" s="2" t="n">
-        <v>260.4</v>
+        <v>261.084</v>
       </c>
       <c r="D75" s="2" t="n"/>
       <c r="E75" s="2" t="n"/>
@@ -5142,10 +5142,10 @@
         </is>
       </c>
       <c r="B76" s="2" t="n">
-        <v>-283.636</v>
+        <v>-283.662</v>
       </c>
       <c r="C76" s="2" t="n">
-        <v>251.4</v>
+        <v>252.084</v>
       </c>
       <c r="D76" s="2" t="n"/>
       <c r="E76" s="2" t="n"/>
@@ -5159,10 +5159,10 @@
         </is>
       </c>
       <c r="B77" s="2" t="n">
-        <v>-283.636</v>
+        <v>-283.662</v>
       </c>
       <c r="C77" s="2" t="n">
-        <v>242.4</v>
+        <v>243.084</v>
       </c>
       <c r="D77" s="2" t="n"/>
       <c r="E77" s="2" t="n"/>
@@ -5176,10 +5176,10 @@
         </is>
       </c>
       <c r="B78" s="2" t="n">
-        <v>-283.636</v>
+        <v>-283.662</v>
       </c>
       <c r="C78" s="2" t="n">
-        <v>233.4</v>
+        <v>234.084</v>
       </c>
       <c r="D78" s="2" t="n"/>
       <c r="E78" s="2" t="n"/>
@@ -5193,10 +5193,10 @@
         </is>
       </c>
       <c r="B79" s="2" t="n">
-        <v>-283.636</v>
+        <v>-283.662</v>
       </c>
       <c r="C79" s="2" t="n">
-        <v>224.4</v>
+        <v>225.084</v>
       </c>
       <c r="D79" s="2" t="n"/>
       <c r="E79" s="2" t="n"/>
@@ -5210,10 +5210,10 @@
         </is>
       </c>
       <c r="B80" s="2" t="n">
-        <v>-283.636</v>
+        <v>-283.662</v>
       </c>
       <c r="C80" s="2" t="n">
-        <v>215.4</v>
+        <v>216.084</v>
       </c>
       <c r="D80" s="2" t="n"/>
       <c r="E80" s="2" t="n"/>
@@ -5227,10 +5227,10 @@
         </is>
       </c>
       <c r="B81" s="2" t="n">
-        <v>-283.636</v>
+        <v>-283.662</v>
       </c>
       <c r="C81" s="2" t="n">
-        <v>206.4</v>
+        <v>207.084</v>
       </c>
       <c r="D81" s="2" t="n"/>
       <c r="E81" s="2" t="n"/>
@@ -5244,10 +5244,10 @@
         </is>
       </c>
       <c r="B82" s="2" t="n">
-        <v>-283.636</v>
+        <v>-283.662</v>
       </c>
       <c r="C82" s="2" t="n">
-        <v>197.4</v>
+        <v>198.084</v>
       </c>
       <c r="D82" s="2" t="n"/>
       <c r="E82" s="2" t="n"/>
@@ -5261,10 +5261,10 @@
         </is>
       </c>
       <c r="B83" s="2" t="n">
-        <v>-283.636</v>
+        <v>-283.662</v>
       </c>
       <c r="C83" s="2" t="n">
-        <v>188.4</v>
+        <v>189.084</v>
       </c>
       <c r="D83" s="2" t="n"/>
       <c r="E83" s="2" t="n"/>
@@ -5278,10 +5278,10 @@
         </is>
       </c>
       <c r="B84" s="2" t="n">
-        <v>-283.636</v>
+        <v>-283.662</v>
       </c>
       <c r="C84" s="2" t="n">
-        <v>179.4</v>
+        <v>180.084</v>
       </c>
       <c r="D84" s="2" t="n"/>
       <c r="E84" s="2" t="n"/>
@@ -5295,10 +5295,10 @@
         </is>
       </c>
       <c r="B85" s="2" t="n">
-        <v>-283.636</v>
+        <v>-283.662</v>
       </c>
       <c r="C85" s="2" t="n">
-        <v>170.4</v>
+        <v>171.084</v>
       </c>
       <c r="D85" s="2" t="n"/>
       <c r="E85" s="2" t="n"/>
@@ -5312,10 +5312,10 @@
         </is>
       </c>
       <c r="B86" s="2" t="n">
-        <v>-292.636</v>
+        <v>-292.662</v>
       </c>
       <c r="C86" s="2" t="n">
-        <v>269.4</v>
+        <v>270.084</v>
       </c>
       <c r="D86" s="2" t="n"/>
       <c r="E86" s="2" t="n"/>
@@ -5329,10 +5329,10 @@
         </is>
       </c>
       <c r="B87" s="2" t="n">
-        <v>-292.636</v>
+        <v>-292.662</v>
       </c>
       <c r="C87" s="2" t="n">
-        <v>260.4</v>
+        <v>261.084</v>
       </c>
       <c r="D87" s="2" t="n"/>
       <c r="E87" s="2" t="n"/>
@@ -5346,10 +5346,10 @@
         </is>
       </c>
       <c r="B88" s="2" t="n">
-        <v>-292.636</v>
+        <v>-292.662</v>
       </c>
       <c r="C88" s="2" t="n">
-        <v>251.4</v>
+        <v>252.084</v>
       </c>
       <c r="D88" s="2" t="n"/>
       <c r="E88" s="2" t="n"/>
@@ -5363,10 +5363,10 @@
         </is>
       </c>
       <c r="B89" s="2" t="n">
-        <v>-292.636</v>
+        <v>-292.662</v>
       </c>
       <c r="C89" s="2" t="n">
-        <v>242.4</v>
+        <v>243.084</v>
       </c>
       <c r="D89" s="2" t="n"/>
       <c r="E89" s="2" t="n"/>
@@ -5380,10 +5380,10 @@
         </is>
       </c>
       <c r="B90" s="2" t="n">
-        <v>-292.636</v>
+        <v>-292.662</v>
       </c>
       <c r="C90" s="2" t="n">
-        <v>233.4</v>
+        <v>234.084</v>
       </c>
       <c r="D90" s="2" t="n"/>
       <c r="E90" s="2" t="n"/>
@@ -5397,10 +5397,10 @@
         </is>
       </c>
       <c r="B91" s="2" t="n">
-        <v>-292.636</v>
+        <v>-292.662</v>
       </c>
       <c r="C91" s="2" t="n">
-        <v>224.4</v>
+        <v>225.084</v>
       </c>
       <c r="D91" s="2" t="n"/>
       <c r="E91" s="2" t="n"/>
@@ -5414,10 +5414,10 @@
         </is>
       </c>
       <c r="B92" s="2" t="n">
-        <v>-292.636</v>
+        <v>-292.662</v>
       </c>
       <c r="C92" s="2" t="n">
-        <v>215.4</v>
+        <v>216.084</v>
       </c>
       <c r="D92" s="2" t="n"/>
       <c r="E92" s="2" t="n"/>
@@ -5431,10 +5431,10 @@
         </is>
       </c>
       <c r="B93" s="2" t="n">
-        <v>-292.636</v>
+        <v>-292.662</v>
       </c>
       <c r="C93" s="2" t="n">
-        <v>206.4</v>
+        <v>207.084</v>
       </c>
       <c r="D93" s="2" t="n"/>
       <c r="E93" s="2" t="n"/>
@@ -5448,10 +5448,10 @@
         </is>
       </c>
       <c r="B94" s="2" t="n">
-        <v>-292.636</v>
+        <v>-292.662</v>
       </c>
       <c r="C94" s="2" t="n">
-        <v>197.4</v>
+        <v>198.084</v>
       </c>
       <c r="D94" s="2" t="n"/>
       <c r="E94" s="2" t="n"/>
@@ -5465,10 +5465,10 @@
         </is>
       </c>
       <c r="B95" s="2" t="n">
-        <v>-292.636</v>
+        <v>-292.662</v>
       </c>
       <c r="C95" s="2" t="n">
-        <v>188.4</v>
+        <v>189.084</v>
       </c>
       <c r="D95" s="2" t="n"/>
       <c r="E95" s="2" t="n"/>
@@ -5482,10 +5482,10 @@
         </is>
       </c>
       <c r="B96" s="2" t="n">
-        <v>-292.636</v>
+        <v>-292.662</v>
       </c>
       <c r="C96" s="2" t="n">
-        <v>179.4</v>
+        <v>180.084</v>
       </c>
       <c r="D96" s="2" t="n"/>
       <c r="E96" s="2" t="n"/>
@@ -5499,10 +5499,10 @@
         </is>
       </c>
       <c r="B97" s="2" t="n">
-        <v>-292.636</v>
+        <v>-292.662</v>
       </c>
       <c r="C97" s="2" t="n">
-        <v>170.4</v>
+        <v>171.084</v>
       </c>
       <c r="D97" s="2" t="n"/>
       <c r="E97" s="2" t="n"/>
@@ -5576,10 +5576,10 @@
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>-329.729</v>
+        <v>-329.796</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>204.202</v>
+        <v>204.488</v>
       </c>
       <c r="D2" s="2" t="n"/>
       <c r="E2" s="2" t="n"/>
@@ -5593,10 +5593,10 @@
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>-329.729</v>
+        <v>-329.796</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>195.202</v>
+        <v>195.488</v>
       </c>
       <c r="D3" s="2" t="n"/>
       <c r="E3" s="2" t="n"/>
@@ -5610,10 +5610,10 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>-329.729</v>
+        <v>-329.796</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>186.202</v>
+        <v>186.488</v>
       </c>
       <c r="D4" s="2" t="n"/>
       <c r="E4" s="2" t="n"/>
@@ -5627,10 +5627,10 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>-329.729</v>
+        <v>-329.796</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>177.202</v>
+        <v>177.488</v>
       </c>
       <c r="D5" s="2" t="n"/>
       <c r="E5" s="2" t="n"/>
@@ -5644,10 +5644,10 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>-329.729</v>
+        <v>-329.796</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>168.202</v>
+        <v>168.488</v>
       </c>
       <c r="D6" s="2" t="n"/>
       <c r="E6" s="2" t="n"/>
@@ -5661,10 +5661,10 @@
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>-329.729</v>
+        <v>-329.796</v>
       </c>
       <c r="C7" s="2" t="n">
-        <v>159.202</v>
+        <v>159.488</v>
       </c>
       <c r="D7" s="2" t="n"/>
       <c r="E7" s="2" t="n"/>
@@ -5678,10 +5678,10 @@
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>-329.729</v>
+        <v>-329.796</v>
       </c>
       <c r="C8" s="2" t="n">
-        <v>150.202</v>
+        <v>150.488</v>
       </c>
       <c r="D8" s="2" t="n"/>
       <c r="E8" s="2" t="n"/>
@@ -5695,10 +5695,10 @@
         </is>
       </c>
       <c r="B9" s="2" t="n">
-        <v>-329.729</v>
+        <v>-329.796</v>
       </c>
       <c r="C9" s="2" t="n">
-        <v>141.202</v>
+        <v>141.488</v>
       </c>
       <c r="D9" s="2" t="n"/>
       <c r="E9" s="2" t="n"/>
@@ -5712,10 +5712,10 @@
         </is>
       </c>
       <c r="B10" s="2" t="n">
-        <v>-329.729</v>
+        <v>-329.796</v>
       </c>
       <c r="C10" s="2" t="n">
-        <v>132.202</v>
+        <v>132.488</v>
       </c>
       <c r="D10" s="2" t="n"/>
       <c r="E10" s="2" t="n"/>
@@ -5729,10 +5729,10 @@
         </is>
       </c>
       <c r="B11" s="2" t="n">
-        <v>-329.729</v>
+        <v>-329.796</v>
       </c>
       <c r="C11" s="2" t="n">
-        <v>123.202</v>
+        <v>123.488</v>
       </c>
       <c r="D11" s="2" t="n"/>
       <c r="E11" s="2" t="n"/>
@@ -5746,10 +5746,10 @@
         </is>
       </c>
       <c r="B12" s="2" t="n">
-        <v>-329.729</v>
+        <v>-329.796</v>
       </c>
       <c r="C12" s="2" t="n">
-        <v>114.202</v>
+        <v>114.488</v>
       </c>
       <c r="D12" s="2" t="n"/>
       <c r="E12" s="2" t="n"/>
@@ -5763,10 +5763,10 @@
         </is>
       </c>
       <c r="B13" s="2" t="n">
-        <v>-329.729</v>
+        <v>-329.796</v>
       </c>
       <c r="C13" s="2" t="n">
-        <v>105.202</v>
+        <v>105.488</v>
       </c>
       <c r="D13" s="2" t="n"/>
       <c r="E13" s="2" t="n"/>
@@ -5780,10 +5780,10 @@
         </is>
       </c>
       <c r="B14" s="2" t="n">
-        <v>-338.729</v>
+        <v>-338.796</v>
       </c>
       <c r="C14" s="2" t="n">
-        <v>204.202</v>
+        <v>204.488</v>
       </c>
       <c r="D14" s="2" t="n"/>
       <c r="E14" s="2" t="n"/>
@@ -5797,10 +5797,10 @@
         </is>
       </c>
       <c r="B15" s="2" t="n">
-        <v>-338.729</v>
+        <v>-338.796</v>
       </c>
       <c r="C15" s="2" t="n">
-        <v>195.202</v>
+        <v>195.488</v>
       </c>
       <c r="D15" s="2" t="n"/>
       <c r="E15" s="2" t="n"/>
@@ -5814,10 +5814,10 @@
         </is>
       </c>
       <c r="B16" s="2" t="n">
-        <v>-338.729</v>
+        <v>-338.796</v>
       </c>
       <c r="C16" s="2" t="n">
-        <v>186.202</v>
+        <v>186.488</v>
       </c>
       <c r="D16" s="2" t="n"/>
       <c r="E16" s="2" t="n"/>
@@ -5831,10 +5831,10 @@
         </is>
       </c>
       <c r="B17" s="2" t="n">
-        <v>-338.729</v>
+        <v>-338.796</v>
       </c>
       <c r="C17" s="2" t="n">
-        <v>177.202</v>
+        <v>177.488</v>
       </c>
       <c r="D17" s="2" t="n"/>
       <c r="E17" s="2" t="n"/>
@@ -5848,10 +5848,10 @@
         </is>
       </c>
       <c r="B18" s="2" t="n">
-        <v>-338.729</v>
+        <v>-338.796</v>
       </c>
       <c r="C18" s="2" t="n">
-        <v>168.202</v>
+        <v>168.488</v>
       </c>
       <c r="D18" s="2" t="n"/>
       <c r="E18" s="2" t="n"/>
@@ -5865,10 +5865,10 @@
         </is>
       </c>
       <c r="B19" s="2" t="n">
-        <v>-338.729</v>
+        <v>-338.796</v>
       </c>
       <c r="C19" s="2" t="n">
-        <v>159.202</v>
+        <v>159.488</v>
       </c>
       <c r="D19" s="2" t="n"/>
       <c r="E19" s="2" t="n"/>
@@ -5882,10 +5882,10 @@
         </is>
       </c>
       <c r="B20" s="2" t="n">
-        <v>-338.729</v>
+        <v>-338.796</v>
       </c>
       <c r="C20" s="2" t="n">
-        <v>150.202</v>
+        <v>150.488</v>
       </c>
       <c r="D20" s="2" t="n"/>
       <c r="E20" s="2" t="n"/>
@@ -5899,10 +5899,10 @@
         </is>
       </c>
       <c r="B21" s="2" t="n">
-        <v>-338.729</v>
+        <v>-338.796</v>
       </c>
       <c r="C21" s="2" t="n">
-        <v>141.202</v>
+        <v>141.488</v>
       </c>
       <c r="D21" s="2" t="n"/>
       <c r="E21" s="2" t="n"/>
@@ -5916,10 +5916,10 @@
         </is>
       </c>
       <c r="B22" s="2" t="n">
-        <v>-338.729</v>
+        <v>-338.796</v>
       </c>
       <c r="C22" s="2" t="n">
-        <v>132.202</v>
+        <v>132.488</v>
       </c>
       <c r="D22" s="2" t="n"/>
       <c r="E22" s="2" t="n"/>
@@ -5933,10 +5933,10 @@
         </is>
       </c>
       <c r="B23" s="2" t="n">
-        <v>-338.729</v>
+        <v>-338.796</v>
       </c>
       <c r="C23" s="2" t="n">
-        <v>123.202</v>
+        <v>123.488</v>
       </c>
       <c r="D23" s="2" t="n"/>
       <c r="E23" s="2" t="n"/>
@@ -5950,10 +5950,10 @@
         </is>
       </c>
       <c r="B24" s="2" t="n">
-        <v>-338.729</v>
+        <v>-338.796</v>
       </c>
       <c r="C24" s="2" t="n">
-        <v>114.202</v>
+        <v>114.488</v>
       </c>
       <c r="D24" s="2" t="n"/>
       <c r="E24" s="2" t="n"/>
@@ -5967,10 +5967,10 @@
         </is>
       </c>
       <c r="B25" s="2" t="n">
-        <v>-338.729</v>
+        <v>-338.796</v>
       </c>
       <c r="C25" s="2" t="n">
-        <v>105.202</v>
+        <v>105.488</v>
       </c>
       <c r="D25" s="2" t="n"/>
       <c r="E25" s="2" t="n"/>
@@ -5984,10 +5984,10 @@
         </is>
       </c>
       <c r="B26" s="2" t="n">
-        <v>-347.729</v>
+        <v>-347.796</v>
       </c>
       <c r="C26" s="2" t="n">
-        <v>204.202</v>
+        <v>204.488</v>
       </c>
       <c r="D26" s="2" t="n"/>
       <c r="E26" s="2" t="n"/>
@@ -6001,10 +6001,10 @@
         </is>
       </c>
       <c r="B27" s="2" t="n">
-        <v>-347.729</v>
+        <v>-347.796</v>
       </c>
       <c r="C27" s="2" t="n">
-        <v>195.202</v>
+        <v>195.488</v>
       </c>
       <c r="D27" s="2" t="n"/>
       <c r="E27" s="2" t="n"/>
@@ -6018,10 +6018,10 @@
         </is>
       </c>
       <c r="B28" s="2" t="n">
-        <v>-347.729</v>
+        <v>-347.796</v>
       </c>
       <c r="C28" s="2" t="n">
-        <v>186.202</v>
+        <v>186.488</v>
       </c>
       <c r="D28" s="2" t="n"/>
       <c r="E28" s="2" t="n"/>
@@ -6035,10 +6035,10 @@
         </is>
       </c>
       <c r="B29" s="2" t="n">
-        <v>-347.729</v>
+        <v>-347.796</v>
       </c>
       <c r="C29" s="2" t="n">
-        <v>177.202</v>
+        <v>177.488</v>
       </c>
       <c r="D29" s="2" t="n"/>
       <c r="E29" s="2" t="n"/>
@@ -6052,10 +6052,10 @@
         </is>
       </c>
       <c r="B30" s="2" t="n">
-        <v>-347.729</v>
+        <v>-347.796</v>
       </c>
       <c r="C30" s="2" t="n">
-        <v>168.202</v>
+        <v>168.488</v>
       </c>
       <c r="D30" s="2" t="n"/>
       <c r="E30" s="2" t="n"/>
@@ -6069,10 +6069,10 @@
         </is>
       </c>
       <c r="B31" s="2" t="n">
-        <v>-347.729</v>
+        <v>-347.796</v>
       </c>
       <c r="C31" s="2" t="n">
-        <v>159.202</v>
+        <v>159.488</v>
       </c>
       <c r="D31" s="2" t="n"/>
       <c r="E31" s="2" t="n"/>
@@ -6086,10 +6086,10 @@
         </is>
       </c>
       <c r="B32" s="2" t="n">
-        <v>-347.729</v>
+        <v>-347.796</v>
       </c>
       <c r="C32" s="2" t="n">
-        <v>150.202</v>
+        <v>150.488</v>
       </c>
       <c r="D32" s="2" t="n"/>
       <c r="E32" s="2" t="n"/>
@@ -6103,10 +6103,10 @@
         </is>
       </c>
       <c r="B33" s="2" t="n">
-        <v>-347.729</v>
+        <v>-347.796</v>
       </c>
       <c r="C33" s="2" t="n">
-        <v>141.202</v>
+        <v>141.488</v>
       </c>
       <c r="D33" s="2" t="n"/>
       <c r="E33" s="2" t="n"/>
@@ -6120,10 +6120,10 @@
         </is>
       </c>
       <c r="B34" s="2" t="n">
-        <v>-347.729</v>
+        <v>-347.796</v>
       </c>
       <c r="C34" s="2" t="n">
-        <v>132.202</v>
+        <v>132.488</v>
       </c>
       <c r="D34" s="2" t="n"/>
       <c r="E34" s="2" t="n"/>
@@ -6137,10 +6137,10 @@
         </is>
       </c>
       <c r="B35" s="2" t="n">
-        <v>-347.729</v>
+        <v>-347.796</v>
       </c>
       <c r="C35" s="2" t="n">
-        <v>123.202</v>
+        <v>123.488</v>
       </c>
       <c r="D35" s="2" t="n"/>
       <c r="E35" s="2" t="n"/>
@@ -6154,10 +6154,10 @@
         </is>
       </c>
       <c r="B36" s="2" t="n">
-        <v>-347.729</v>
+        <v>-347.796</v>
       </c>
       <c r="C36" s="2" t="n">
-        <v>114.202</v>
+        <v>114.488</v>
       </c>
       <c r="D36" s="2" t="n"/>
       <c r="E36" s="2" t="n"/>
@@ -6171,10 +6171,10 @@
         </is>
       </c>
       <c r="B37" s="2" t="n">
-        <v>-347.729</v>
+        <v>-347.796</v>
       </c>
       <c r="C37" s="2" t="n">
-        <v>105.202</v>
+        <v>105.488</v>
       </c>
       <c r="D37" s="2" t="n"/>
       <c r="E37" s="2" t="n"/>
@@ -6188,10 +6188,10 @@
         </is>
       </c>
       <c r="B38" s="2" t="n">
-        <v>-356.729</v>
+        <v>-356.796</v>
       </c>
       <c r="C38" s="2" t="n">
-        <v>204.202</v>
+        <v>204.488</v>
       </c>
       <c r="D38" s="2" t="n"/>
       <c r="E38" s="2" t="n"/>
@@ -6205,10 +6205,10 @@
         </is>
       </c>
       <c r="B39" s="2" t="n">
-        <v>-356.729</v>
+        <v>-356.796</v>
       </c>
       <c r="C39" s="2" t="n">
-        <v>195.202</v>
+        <v>195.488</v>
       </c>
       <c r="D39" s="2" t="n"/>
       <c r="E39" s="2" t="n"/>
@@ -6222,10 +6222,10 @@
         </is>
       </c>
       <c r="B40" s="2" t="n">
-        <v>-356.729</v>
+        <v>-356.796</v>
       </c>
       <c r="C40" s="2" t="n">
-        <v>186.202</v>
+        <v>186.488</v>
       </c>
       <c r="D40" s="2" t="n"/>
       <c r="E40" s="2" t="n"/>
@@ -6239,10 +6239,10 @@
         </is>
       </c>
       <c r="B41" s="2" t="n">
-        <v>-356.729</v>
+        <v>-356.796</v>
       </c>
       <c r="C41" s="2" t="n">
-        <v>177.202</v>
+        <v>177.488</v>
       </c>
       <c r="D41" s="2" t="n"/>
       <c r="E41" s="2" t="n"/>
@@ -6256,10 +6256,10 @@
         </is>
       </c>
       <c r="B42" s="2" t="n">
-        <v>-356.729</v>
+        <v>-356.796</v>
       </c>
       <c r="C42" s="2" t="n">
-        <v>168.202</v>
+        <v>168.488</v>
       </c>
       <c r="D42" s="2" t="n"/>
       <c r="E42" s="2" t="n"/>
@@ -6273,10 +6273,10 @@
         </is>
       </c>
       <c r="B43" s="2" t="n">
-        <v>-356.729</v>
+        <v>-356.796</v>
       </c>
       <c r="C43" s="2" t="n">
-        <v>159.202</v>
+        <v>159.488</v>
       </c>
       <c r="D43" s="2" t="n"/>
       <c r="E43" s="2" t="n"/>
@@ -6290,10 +6290,10 @@
         </is>
       </c>
       <c r="B44" s="2" t="n">
-        <v>-356.729</v>
+        <v>-356.796</v>
       </c>
       <c r="C44" s="2" t="n">
-        <v>150.202</v>
+        <v>150.488</v>
       </c>
       <c r="D44" s="2" t="n"/>
       <c r="E44" s="2" t="n"/>
@@ -6307,10 +6307,10 @@
         </is>
       </c>
       <c r="B45" s="2" t="n">
-        <v>-356.729</v>
+        <v>-356.796</v>
       </c>
       <c r="C45" s="2" t="n">
-        <v>141.202</v>
+        <v>141.488</v>
       </c>
       <c r="D45" s="2" t="n"/>
       <c r="E45" s="2" t="n"/>
@@ -6324,10 +6324,10 @@
         </is>
       </c>
       <c r="B46" s="2" t="n">
-        <v>-356.729</v>
+        <v>-356.796</v>
       </c>
       <c r="C46" s="2" t="n">
-        <v>132.202</v>
+        <v>132.488</v>
       </c>
       <c r="D46" s="2" t="n"/>
       <c r="E46" s="2" t="n"/>
@@ -6341,10 +6341,10 @@
         </is>
       </c>
       <c r="B47" s="2" t="n">
-        <v>-356.729</v>
+        <v>-356.796</v>
       </c>
       <c r="C47" s="2" t="n">
-        <v>123.202</v>
+        <v>123.488</v>
       </c>
       <c r="D47" s="2" t="n"/>
       <c r="E47" s="2" t="n"/>
@@ -6358,10 +6358,10 @@
         </is>
       </c>
       <c r="B48" s="2" t="n">
-        <v>-356.729</v>
+        <v>-356.796</v>
       </c>
       <c r="C48" s="2" t="n">
-        <v>114.202</v>
+        <v>114.488</v>
       </c>
       <c r="D48" s="2" t="n"/>
       <c r="E48" s="2" t="n"/>
@@ -6375,10 +6375,10 @@
         </is>
       </c>
       <c r="B49" s="2" t="n">
-        <v>-356.729</v>
+        <v>-356.796</v>
       </c>
       <c r="C49" s="2" t="n">
-        <v>105.202</v>
+        <v>105.488</v>
       </c>
       <c r="D49" s="2" t="n"/>
       <c r="E49" s="2" t="n"/>
@@ -6392,10 +6392,10 @@
         </is>
       </c>
       <c r="B50" s="2" t="n">
-        <v>-365.729</v>
+        <v>-365.796</v>
       </c>
       <c r="C50" s="2" t="n">
-        <v>204.202</v>
+        <v>204.488</v>
       </c>
       <c r="D50" s="2" t="n"/>
       <c r="E50" s="2" t="n"/>
@@ -6409,10 +6409,10 @@
         </is>
       </c>
       <c r="B51" s="2" t="n">
-        <v>-365.729</v>
+        <v>-365.796</v>
       </c>
       <c r="C51" s="2" t="n">
-        <v>195.202</v>
+        <v>195.488</v>
       </c>
       <c r="D51" s="2" t="n"/>
       <c r="E51" s="2" t="n"/>
@@ -6426,10 +6426,10 @@
         </is>
       </c>
       <c r="B52" s="2" t="n">
-        <v>-365.729</v>
+        <v>-365.796</v>
       </c>
       <c r="C52" s="2" t="n">
-        <v>186.202</v>
+        <v>186.488</v>
       </c>
       <c r="D52" s="2" t="n"/>
       <c r="E52" s="2" t="n"/>
@@ -6443,10 +6443,10 @@
         </is>
       </c>
       <c r="B53" s="2" t="n">
-        <v>-365.729</v>
+        <v>-365.796</v>
       </c>
       <c r="C53" s="2" t="n">
-        <v>177.202</v>
+        <v>177.488</v>
       </c>
       <c r="D53" s="2" t="n"/>
       <c r="E53" s="2" t="n"/>
@@ -6460,10 +6460,10 @@
         </is>
       </c>
       <c r="B54" s="2" t="n">
-        <v>-365.729</v>
+        <v>-365.796</v>
       </c>
       <c r="C54" s="2" t="n">
-        <v>168.202</v>
+        <v>168.488</v>
       </c>
       <c r="D54" s="2" t="n"/>
       <c r="E54" s="2" t="n"/>
@@ -6477,10 +6477,10 @@
         </is>
       </c>
       <c r="B55" s="2" t="n">
-        <v>-365.729</v>
+        <v>-365.796</v>
       </c>
       <c r="C55" s="2" t="n">
-        <v>159.202</v>
+        <v>159.488</v>
       </c>
       <c r="D55" s="2" t="n"/>
       <c r="E55" s="2" t="n"/>
@@ -6494,10 +6494,10 @@
         </is>
       </c>
       <c r="B56" s="2" t="n">
-        <v>-365.729</v>
+        <v>-365.796</v>
       </c>
       <c r="C56" s="2" t="n">
-        <v>150.202</v>
+        <v>150.488</v>
       </c>
       <c r="D56" s="2" t="n"/>
       <c r="E56" s="2" t="n"/>
@@ -6511,10 +6511,10 @@
         </is>
       </c>
       <c r="B57" s="2" t="n">
-        <v>-365.729</v>
+        <v>-365.796</v>
       </c>
       <c r="C57" s="2" t="n">
-        <v>141.202</v>
+        <v>141.488</v>
       </c>
       <c r="D57" s="2" t="n"/>
       <c r="E57" s="2" t="n"/>
@@ -6528,10 +6528,10 @@
         </is>
       </c>
       <c r="B58" s="2" t="n">
-        <v>-365.729</v>
+        <v>-365.796</v>
       </c>
       <c r="C58" s="2" t="n">
-        <v>132.202</v>
+        <v>132.488</v>
       </c>
       <c r="D58" s="2" t="n"/>
       <c r="E58" s="2" t="n"/>
@@ -6545,10 +6545,10 @@
         </is>
       </c>
       <c r="B59" s="2" t="n">
-        <v>-365.729</v>
+        <v>-365.796</v>
       </c>
       <c r="C59" s="2" t="n">
-        <v>123.202</v>
+        <v>123.488</v>
       </c>
       <c r="D59" s="2" t="n"/>
       <c r="E59" s="2" t="n"/>
@@ -6562,10 +6562,10 @@
         </is>
       </c>
       <c r="B60" s="2" t="n">
-        <v>-365.729</v>
+        <v>-365.796</v>
       </c>
       <c r="C60" s="2" t="n">
-        <v>114.202</v>
+        <v>114.488</v>
       </c>
       <c r="D60" s="2" t="n"/>
       <c r="E60" s="2" t="n"/>
@@ -6579,10 +6579,10 @@
         </is>
       </c>
       <c r="B61" s="2" t="n">
-        <v>-365.729</v>
+        <v>-365.796</v>
       </c>
       <c r="C61" s="2" t="n">
-        <v>105.202</v>
+        <v>105.488</v>
       </c>
       <c r="D61" s="2" t="n"/>
       <c r="E61" s="2" t="n"/>
@@ -6596,10 +6596,10 @@
         </is>
       </c>
       <c r="B62" s="2" t="n">
-        <v>-374.729</v>
+        <v>-374.796</v>
       </c>
       <c r="C62" s="2" t="n">
-        <v>204.202</v>
+        <v>204.488</v>
       </c>
       <c r="D62" s="2" t="n"/>
       <c r="E62" s="2" t="n"/>
@@ -6613,10 +6613,10 @@
         </is>
       </c>
       <c r="B63" s="2" t="n">
-        <v>-374.729</v>
+        <v>-374.796</v>
       </c>
       <c r="C63" s="2" t="n">
-        <v>195.202</v>
+        <v>195.488</v>
       </c>
       <c r="D63" s="2" t="n"/>
       <c r="E63" s="2" t="n"/>
@@ -6630,10 +6630,10 @@
         </is>
       </c>
       <c r="B64" s="2" t="n">
-        <v>-374.729</v>
+        <v>-374.796</v>
       </c>
       <c r="C64" s="2" t="n">
-        <v>186.202</v>
+        <v>186.488</v>
       </c>
       <c r="D64" s="2" t="n"/>
       <c r="E64" s="2" t="n"/>
@@ -6647,10 +6647,10 @@
         </is>
       </c>
       <c r="B65" s="2" t="n">
-        <v>-374.729</v>
+        <v>-374.796</v>
       </c>
       <c r="C65" s="2" t="n">
-        <v>177.202</v>
+        <v>177.488</v>
       </c>
       <c r="D65" s="2" t="n"/>
       <c r="E65" s="2" t="n"/>
@@ -6664,10 +6664,10 @@
         </is>
       </c>
       <c r="B66" s="2" t="n">
-        <v>-374.729</v>
+        <v>-374.796</v>
       </c>
       <c r="C66" s="2" t="n">
-        <v>168.202</v>
+        <v>168.488</v>
       </c>
       <c r="D66" s="2" t="n"/>
       <c r="E66" s="2" t="n"/>
@@ -6681,10 +6681,10 @@
         </is>
       </c>
       <c r="B67" s="2" t="n">
-        <v>-374.729</v>
+        <v>-374.796</v>
       </c>
       <c r="C67" s="2" t="n">
-        <v>159.202</v>
+        <v>159.488</v>
       </c>
       <c r="D67" s="2" t="n"/>
       <c r="E67" s="2" t="n"/>
@@ -6698,10 +6698,10 @@
         </is>
       </c>
       <c r="B68" s="2" t="n">
-        <v>-374.729</v>
+        <v>-374.796</v>
       </c>
       <c r="C68" s="2" t="n">
-        <v>150.202</v>
+        <v>150.488</v>
       </c>
       <c r="D68" s="2" t="n"/>
       <c r="E68" s="2" t="n"/>
@@ -6715,10 +6715,10 @@
         </is>
       </c>
       <c r="B69" s="2" t="n">
-        <v>-374.729</v>
+        <v>-374.796</v>
       </c>
       <c r="C69" s="2" t="n">
-        <v>141.202</v>
+        <v>141.488</v>
       </c>
       <c r="D69" s="2" t="n"/>
       <c r="E69" s="2" t="n"/>
@@ -6732,10 +6732,10 @@
         </is>
       </c>
       <c r="B70" s="2" t="n">
-        <v>-374.729</v>
+        <v>-374.796</v>
       </c>
       <c r="C70" s="2" t="n">
-        <v>132.202</v>
+        <v>132.488</v>
       </c>
       <c r="D70" s="2" t="n"/>
       <c r="E70" s="2" t="n"/>
@@ -6749,10 +6749,10 @@
         </is>
       </c>
       <c r="B71" s="2" t="n">
-        <v>-374.729</v>
+        <v>-374.796</v>
       </c>
       <c r="C71" s="2" t="n">
-        <v>123.202</v>
+        <v>123.488</v>
       </c>
       <c r="D71" s="2" t="n"/>
       <c r="E71" s="2" t="n"/>
@@ -6766,10 +6766,10 @@
         </is>
       </c>
       <c r="B72" s="2" t="n">
-        <v>-374.729</v>
+        <v>-374.796</v>
       </c>
       <c r="C72" s="2" t="n">
-        <v>114.202</v>
+        <v>114.488</v>
       </c>
       <c r="D72" s="2" t="n"/>
       <c r="E72" s="2" t="n"/>
@@ -6783,10 +6783,10 @@
         </is>
       </c>
       <c r="B73" s="2" t="n">
-        <v>-374.729</v>
+        <v>-374.796</v>
       </c>
       <c r="C73" s="2" t="n">
-        <v>105.202</v>
+        <v>105.488</v>
       </c>
       <c r="D73" s="2" t="n"/>
       <c r="E73" s="2" t="n"/>
@@ -6800,10 +6800,10 @@
         </is>
       </c>
       <c r="B74" s="2" t="n">
-        <v>-383.729</v>
+        <v>-383.796</v>
       </c>
       <c r="C74" s="2" t="n">
-        <v>204.202</v>
+        <v>204.488</v>
       </c>
       <c r="D74" s="2" t="n"/>
       <c r="E74" s="2" t="n"/>
@@ -6817,10 +6817,10 @@
         </is>
       </c>
       <c r="B75" s="2" t="n">
-        <v>-383.729</v>
+        <v>-383.796</v>
       </c>
       <c r="C75" s="2" t="n">
-        <v>195.202</v>
+        <v>195.488</v>
       </c>
       <c r="D75" s="2" t="n"/>
       <c r="E75" s="2" t="n"/>
@@ -6834,10 +6834,10 @@
         </is>
       </c>
       <c r="B76" s="2" t="n">
-        <v>-383.729</v>
+        <v>-383.796</v>
       </c>
       <c r="C76" s="2" t="n">
-        <v>186.202</v>
+        <v>186.488</v>
       </c>
       <c r="D76" s="2" t="n"/>
       <c r="E76" s="2" t="n"/>
@@ -6851,10 +6851,10 @@
         </is>
       </c>
       <c r="B77" s="2" t="n">
-        <v>-383.729</v>
+        <v>-383.796</v>
       </c>
       <c r="C77" s="2" t="n">
-        <v>177.202</v>
+        <v>177.488</v>
       </c>
       <c r="D77" s="2" t="n"/>
       <c r="E77" s="2" t="n"/>
@@ -6868,10 +6868,10 @@
         </is>
       </c>
       <c r="B78" s="2" t="n">
-        <v>-383.729</v>
+        <v>-383.796</v>
       </c>
       <c r="C78" s="2" t="n">
-        <v>168.202</v>
+        <v>168.488</v>
       </c>
       <c r="D78" s="2" t="n"/>
       <c r="E78" s="2" t="n"/>
@@ -6885,10 +6885,10 @@
         </is>
       </c>
       <c r="B79" s="2" t="n">
-        <v>-383.729</v>
+        <v>-383.796</v>
       </c>
       <c r="C79" s="2" t="n">
-        <v>159.202</v>
+        <v>159.488</v>
       </c>
       <c r="D79" s="2" t="n"/>
       <c r="E79" s="2" t="n"/>
@@ -6902,10 +6902,10 @@
         </is>
       </c>
       <c r="B80" s="2" t="n">
-        <v>-383.729</v>
+        <v>-383.796</v>
       </c>
       <c r="C80" s="2" t="n">
-        <v>150.202</v>
+        <v>150.488</v>
       </c>
       <c r="D80" s="2" t="n"/>
       <c r="E80" s="2" t="n"/>
@@ -6919,10 +6919,10 @@
         </is>
       </c>
       <c r="B81" s="2" t="n">
-        <v>-383.729</v>
+        <v>-383.796</v>
       </c>
       <c r="C81" s="2" t="n">
-        <v>141.202</v>
+        <v>141.488</v>
       </c>
       <c r="D81" s="2" t="n"/>
       <c r="E81" s="2" t="n"/>
@@ -6936,10 +6936,10 @@
         </is>
       </c>
       <c r="B82" s="2" t="n">
-        <v>-383.729</v>
+        <v>-383.796</v>
       </c>
       <c r="C82" s="2" t="n">
-        <v>132.202</v>
+        <v>132.488</v>
       </c>
       <c r="D82" s="2" t="n"/>
       <c r="E82" s="2" t="n"/>
@@ -6953,10 +6953,10 @@
         </is>
       </c>
       <c r="B83" s="2" t="n">
-        <v>-383.729</v>
+        <v>-383.796</v>
       </c>
       <c r="C83" s="2" t="n">
-        <v>123.202</v>
+        <v>123.488</v>
       </c>
       <c r="D83" s="2" t="n"/>
       <c r="E83" s="2" t="n"/>
@@ -6970,10 +6970,10 @@
         </is>
       </c>
       <c r="B84" s="2" t="n">
-        <v>-383.729</v>
+        <v>-383.796</v>
       </c>
       <c r="C84" s="2" t="n">
-        <v>114.202</v>
+        <v>114.488</v>
       </c>
       <c r="D84" s="2" t="n"/>
       <c r="E84" s="2" t="n"/>
@@ -6987,10 +6987,10 @@
         </is>
       </c>
       <c r="B85" s="2" t="n">
-        <v>-383.729</v>
+        <v>-383.796</v>
       </c>
       <c r="C85" s="2" t="n">
-        <v>105.202</v>
+        <v>105.488</v>
       </c>
       <c r="D85" s="2" t="n"/>
       <c r="E85" s="2" t="n"/>
@@ -7004,10 +7004,10 @@
         </is>
       </c>
       <c r="B86" s="2" t="n">
-        <v>-392.729</v>
+        <v>-392.796</v>
       </c>
       <c r="C86" s="2" t="n">
-        <v>204.202</v>
+        <v>204.488</v>
       </c>
       <c r="D86" s="2" t="n"/>
       <c r="E86" s="2" t="n"/>
@@ -7021,10 +7021,10 @@
         </is>
       </c>
       <c r="B87" s="2" t="n">
-        <v>-392.729</v>
+        <v>-392.796</v>
       </c>
       <c r="C87" s="2" t="n">
-        <v>195.202</v>
+        <v>195.488</v>
       </c>
       <c r="D87" s="2" t="n"/>
       <c r="E87" s="2" t="n"/>
@@ -7038,10 +7038,10 @@
         </is>
       </c>
       <c r="B88" s="2" t="n">
-        <v>-392.729</v>
+        <v>-392.796</v>
       </c>
       <c r="C88" s="2" t="n">
-        <v>186.202</v>
+        <v>186.488</v>
       </c>
       <c r="D88" s="2" t="n"/>
       <c r="E88" s="2" t="n"/>
@@ -7055,10 +7055,10 @@
         </is>
       </c>
       <c r="B89" s="2" t="n">
-        <v>-392.729</v>
+        <v>-392.796</v>
       </c>
       <c r="C89" s="2" t="n">
-        <v>177.202</v>
+        <v>177.488</v>
       </c>
       <c r="D89" s="2" t="n"/>
       <c r="E89" s="2" t="n"/>
@@ -7072,10 +7072,10 @@
         </is>
       </c>
       <c r="B90" s="2" t="n">
-        <v>-392.729</v>
+        <v>-392.796</v>
       </c>
       <c r="C90" s="2" t="n">
-        <v>168.202</v>
+        <v>168.488</v>
       </c>
       <c r="D90" s="2" t="n"/>
       <c r="E90" s="2" t="n"/>
@@ -7089,10 +7089,10 @@
         </is>
       </c>
       <c r="B91" s="2" t="n">
-        <v>-392.729</v>
+        <v>-392.796</v>
       </c>
       <c r="C91" s="2" t="n">
-        <v>159.202</v>
+        <v>159.488</v>
       </c>
       <c r="D91" s="2" t="n"/>
       <c r="E91" s="2" t="n"/>
@@ -7106,10 +7106,10 @@
         </is>
       </c>
       <c r="B92" s="2" t="n">
-        <v>-392.729</v>
+        <v>-392.796</v>
       </c>
       <c r="C92" s="2" t="n">
-        <v>150.202</v>
+        <v>150.488</v>
       </c>
       <c r="D92" s="2" t="n"/>
       <c r="E92" s="2" t="n"/>
@@ -7123,10 +7123,10 @@
         </is>
       </c>
       <c r="B93" s="2" t="n">
-        <v>-392.729</v>
+        <v>-392.796</v>
       </c>
       <c r="C93" s="2" t="n">
-        <v>141.202</v>
+        <v>141.488</v>
       </c>
       <c r="D93" s="2" t="n"/>
       <c r="E93" s="2" t="n"/>
@@ -7140,10 +7140,10 @@
         </is>
       </c>
       <c r="B94" s="2" t="n">
-        <v>-392.729</v>
+        <v>-392.796</v>
       </c>
       <c r="C94" s="2" t="n">
-        <v>132.202</v>
+        <v>132.488</v>
       </c>
       <c r="D94" s="2" t="n"/>
       <c r="E94" s="2" t="n"/>
@@ -7157,10 +7157,10 @@
         </is>
       </c>
       <c r="B95" s="2" t="n">
-        <v>-392.729</v>
+        <v>-392.796</v>
       </c>
       <c r="C95" s="2" t="n">
-        <v>123.202</v>
+        <v>123.488</v>
       </c>
       <c r="D95" s="2" t="n"/>
       <c r="E95" s="2" t="n"/>
@@ -7174,10 +7174,10 @@
         </is>
       </c>
       <c r="B96" s="2" t="n">
-        <v>-392.729</v>
+        <v>-392.796</v>
       </c>
       <c r="C96" s="2" t="n">
-        <v>114.202</v>
+        <v>114.488</v>
       </c>
       <c r="D96" s="2" t="n"/>
       <c r="E96" s="2" t="n"/>
@@ -7191,10 +7191,10 @@
         </is>
       </c>
       <c r="B97" s="2" t="n">
-        <v>-392.729</v>
+        <v>-392.796</v>
       </c>
       <c r="C97" s="2" t="n">
-        <v>105.202</v>
+        <v>105.488</v>
       </c>
       <c r="D97" s="2" t="n"/>
       <c r="E97" s="2" t="n"/>
@@ -7204,283 +7204,4 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100DF72643B013E014A825B49D64A1110FC" ma:contentTypeVersion="17" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="f45f840bb0a575e0982080148504d801">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="898ec965-d5a3-48b2-9d91-8cd3ed319c77" xmlns:ns3="34a6835a-a421-4fc1-9891-838ec1df6c1f" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="1578e7a6edb9656aff92510688ad8ae5" ns2:_="" ns3:_="">
-    <xsd:import namespace="898ec965-d5a3-48b2-9d91-8cd3ed319c77"/>
-    <xsd:import namespace="34a6835a-a421-4fc1-9891-838ec1df6c1f"/>
-    <xsd:element name="properties">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element name="documentManagement">
-            <xsd:complexType>
-              <xsd:all>
-                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceAutoTags" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
-                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
-                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
-                <xsd:element ref="ns3:SharedWithUsers" minOccurs="0"/>
-                <xsd:element ref="ns3:SharedWithDetails" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceBillingMetadata" minOccurs="0"/>
-              </xsd:all>
-            </xsd:complexType>
-          </xsd:element>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="898ec965-d5a3-48b2-9d91-8cd3ed319c77" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceAutoTags" ma:index="10" nillable="true" ma:displayName="MediaServiceAutoTags" ma:internalName="MediaServiceAutoTags" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaLengthInSeconds" ma:index="11" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Unknown"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceDateTaken" ma:index="12" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="14" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="d3514cfa-118c-47c7-8064-f16f79621ace" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="MediaServiceGenerationTime" ma:index="16" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceEventHashCode" ma:index="17" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceOCR" ma:index="18" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceLocation" ma:index="19" nillable="true" ma:displayName="Location" ma:indexed="true" ma:internalName="MediaServiceLocation" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="20" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceSearchProperties" ma:index="23" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceBillingMetadata" ma:index="24" nillable="true" ma:displayName="MediaServiceBillingMetadata" ma:hidden="true" ma:internalName="MediaServiceBillingMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="34a6835a-a421-4fc1-9891-838ec1df6c1f" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="TaxCatchAll" ma:index="15" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{fdb65f81-2f44-4049-bc2f-903088f674cc}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="34a6835a-a421-4fc1-9891-838ec1df6c1f">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:MultiChoiceLookup">
-            <xsd:sequence>
-              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="SharedWithUsers" ma:index="21" nillable="true" ma:displayName="Shared With" ma:internalName="SharedWithUsers" ma:readOnly="true">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:UserMulti">
-            <xsd:sequence>
-              <xsd:element name="UserInfo" minOccurs="0" maxOccurs="unbounded">
-                <xsd:complexType>
-                  <xsd:sequence>
-                    <xsd:element name="DisplayName" type="xsd:string" minOccurs="0"/>
-                    <xsd:element name="AccountId" type="dms:UserId" minOccurs="0" nillable="true"/>
-                    <xsd:element name="AccountType" type="xsd:string" minOccurs="0"/>
-                  </xsd:sequence>
-                </xsd:complexType>
-              </xsd:element>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="SharedWithDetails" ma:index="22" nillable="true" ma:displayName="Shared With Details" ma:internalName="SharedWithDetails" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
-    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
-    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
-    <xsd:element name="coreProperties" type="CT_coreProperties"/>
-    <xsd:complexType name="CT_coreProperties">
-      <xsd:all>
-        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
-        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
-        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
-          <xsd:annotation>
-            <xsd:documentation>
-                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
-                    </xsd:documentation>
-          </xsd:annotation>
-        </xsd:element>
-        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-      </xsd:all>
-    </xsd:complexType>
-  </xsd:schema>
-  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
-    <xs:element name="Person">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:DisplayName" minOccurs="0"/>
-          <xs:element ref="pc:AccountId" minOccurs="0"/>
-          <xs:element ref="pc:AccountType" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="DisplayName" type="xs:string"/>
-    <xs:element name="AccountId" type="xs:string"/>
-    <xs:element name="AccountType" type="xs:string"/>
-    <xs:element name="BDCAssociatedEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-        <xs:attribute ref="pc:EntityNamespace"/>
-        <xs:attribute ref="pc:EntityName"/>
-        <xs:attribute ref="pc:SystemInstanceName"/>
-        <xs:attribute ref="pc:AssociationName"/>
-      </xs:complexType>
-    </xs:element>
-    <xs:attribute name="EntityNamespace" type="xs:string"/>
-    <xs:attribute name="EntityName" type="xs:string"/>
-    <xs:attribute name="SystemInstanceName" type="xs:string"/>
-    <xs:attribute name="AssociationName" type="xs:string"/>
-    <xs:element name="BDCEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
-          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
-          <xs:element ref="pc:EntityId1" minOccurs="0"/>
-          <xs:element ref="pc:EntityId2" minOccurs="0"/>
-          <xs:element ref="pc:EntityId3" minOccurs="0"/>
-          <xs:element ref="pc:EntityId4" minOccurs="0"/>
-          <xs:element ref="pc:EntityId5" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="EntityDisplayName" type="xs:string"/>
-    <xs:element name="EntityInstanceReference" type="xs:string"/>
-    <xs:element name="EntityId1" type="xs:string"/>
-    <xs:element name="EntityId2" type="xs:string"/>
-    <xs:element name="EntityId3" type="xs:string"/>
-    <xs:element name="EntityId4" type="xs:string"/>
-    <xs:element name="EntityId5" type="xs:string"/>
-    <xs:element name="Terms">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermInfo">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermName" minOccurs="0"/>
-          <xs:element ref="pc:TermId" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermName" type="xs:string"/>
-    <xs:element name="TermId" type="xs:string"/>
-  </xs:schema>
-</ct:contentTypeSchema>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="898ec965-d5a3-48b2-9d91-8cd3ed319c77">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="34a6835a-a421-4fc1-9891-838ec1df6c1f" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A0E6EAEC-7369-4F84-8566-D70A17CA8F88}"/>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{61196B03-2FFF-4F62-B05F-456981366424}"/>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C72BDEA0-C8F3-40B4-886F-A98417D1111B}"/>
 </file>
</xml_diff>

<commit_message>
fix(plate-config): regenerate Stations 3-4 from Lefty-confirmed corner measurements
These are the real fix -- taken after confirming the Go /L hand-qualifier
fix actually holds Lefty (earlier attempts at these corners were measured
before that was confirmed working, so the hand active during jogging was
uncertain). Clean 9.00mm grids for both. Stations 1-2 untouched.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/config/plate_configs/plate_stations.xlsx
+++ b/config/plate_configs/plate_stations.xlsx
@@ -3884,10 +3884,10 @@
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>-229.662</v>
+        <v>-192.434</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>270.084</v>
+        <v>283.254</v>
       </c>
       <c r="D2" s="2" t="n"/>
       <c r="E2" s="2" t="n"/>
@@ -3901,10 +3901,10 @@
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>-229.662</v>
+        <v>-192.434</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>261.084</v>
+        <v>274.254</v>
       </c>
       <c r="D3" s="2" t="n"/>
       <c r="E3" s="2" t="n"/>
@@ -3918,10 +3918,10 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>-229.662</v>
+        <v>-192.434</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>252.084</v>
+        <v>265.254</v>
       </c>
       <c r="D4" s="2" t="n"/>
       <c r="E4" s="2" t="n"/>
@@ -3935,10 +3935,10 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>-229.662</v>
+        <v>-192.434</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>243.084</v>
+        <v>256.254</v>
       </c>
       <c r="D5" s="2" t="n"/>
       <c r="E5" s="2" t="n"/>
@@ -3952,10 +3952,10 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>-229.662</v>
+        <v>-192.434</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>234.084</v>
+        <v>247.254</v>
       </c>
       <c r="D6" s="2" t="n"/>
       <c r="E6" s="2" t="n"/>
@@ -3969,10 +3969,10 @@
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>-229.662</v>
+        <v>-192.434</v>
       </c>
       <c r="C7" s="2" t="n">
-        <v>225.084</v>
+        <v>238.254</v>
       </c>
       <c r="D7" s="2" t="n"/>
       <c r="E7" s="2" t="n"/>
@@ -3986,10 +3986,10 @@
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>-229.662</v>
+        <v>-192.434</v>
       </c>
       <c r="C8" s="2" t="n">
-        <v>216.084</v>
+        <v>229.254</v>
       </c>
       <c r="D8" s="2" t="n"/>
       <c r="E8" s="2" t="n"/>
@@ -4003,10 +4003,10 @@
         </is>
       </c>
       <c r="B9" s="2" t="n">
-        <v>-229.662</v>
+        <v>-192.434</v>
       </c>
       <c r="C9" s="2" t="n">
-        <v>207.084</v>
+        <v>220.254</v>
       </c>
       <c r="D9" s="2" t="n"/>
       <c r="E9" s="2" t="n"/>
@@ -4020,10 +4020,10 @@
         </is>
       </c>
       <c r="B10" s="2" t="n">
-        <v>-229.662</v>
+        <v>-192.434</v>
       </c>
       <c r="C10" s="2" t="n">
-        <v>198.084</v>
+        <v>211.254</v>
       </c>
       <c r="D10" s="2" t="n"/>
       <c r="E10" s="2" t="n"/>
@@ -4037,10 +4037,10 @@
         </is>
       </c>
       <c r="B11" s="2" t="n">
-        <v>-229.662</v>
+        <v>-192.434</v>
       </c>
       <c r="C11" s="2" t="n">
-        <v>189.084</v>
+        <v>202.254</v>
       </c>
       <c r="D11" s="2" t="n"/>
       <c r="E11" s="2" t="n"/>
@@ -4054,10 +4054,10 @@
         </is>
       </c>
       <c r="B12" s="2" t="n">
-        <v>-229.662</v>
+        <v>-192.434</v>
       </c>
       <c r="C12" s="2" t="n">
-        <v>180.084</v>
+        <v>193.254</v>
       </c>
       <c r="D12" s="2" t="n"/>
       <c r="E12" s="2" t="n"/>
@@ -4071,10 +4071,10 @@
         </is>
       </c>
       <c r="B13" s="2" t="n">
-        <v>-229.662</v>
+        <v>-192.434</v>
       </c>
       <c r="C13" s="2" t="n">
-        <v>171.084</v>
+        <v>184.254</v>
       </c>
       <c r="D13" s="2" t="n"/>
       <c r="E13" s="2" t="n"/>
@@ -4088,10 +4088,10 @@
         </is>
       </c>
       <c r="B14" s="2" t="n">
-        <v>-238.662</v>
+        <v>-201.434</v>
       </c>
       <c r="C14" s="2" t="n">
-        <v>270.084</v>
+        <v>283.254</v>
       </c>
       <c r="D14" s="2" t="n"/>
       <c r="E14" s="2" t="n"/>
@@ -4105,10 +4105,10 @@
         </is>
       </c>
       <c r="B15" s="2" t="n">
-        <v>-238.662</v>
+        <v>-201.434</v>
       </c>
       <c r="C15" s="2" t="n">
-        <v>261.084</v>
+        <v>274.254</v>
       </c>
       <c r="D15" s="2" t="n"/>
       <c r="E15" s="2" t="n"/>
@@ -4122,10 +4122,10 @@
         </is>
       </c>
       <c r="B16" s="2" t="n">
-        <v>-238.662</v>
+        <v>-201.434</v>
       </c>
       <c r="C16" s="2" t="n">
-        <v>252.084</v>
+        <v>265.254</v>
       </c>
       <c r="D16" s="2" t="n"/>
       <c r="E16" s="2" t="n"/>
@@ -4139,10 +4139,10 @@
         </is>
       </c>
       <c r="B17" s="2" t="n">
-        <v>-238.662</v>
+        <v>-201.434</v>
       </c>
       <c r="C17" s="2" t="n">
-        <v>243.084</v>
+        <v>256.254</v>
       </c>
       <c r="D17" s="2" t="n"/>
       <c r="E17" s="2" t="n"/>
@@ -4156,10 +4156,10 @@
         </is>
       </c>
       <c r="B18" s="2" t="n">
-        <v>-238.662</v>
+        <v>-201.434</v>
       </c>
       <c r="C18" s="2" t="n">
-        <v>234.084</v>
+        <v>247.254</v>
       </c>
       <c r="D18" s="2" t="n"/>
       <c r="E18" s="2" t="n"/>
@@ -4173,10 +4173,10 @@
         </is>
       </c>
       <c r="B19" s="2" t="n">
-        <v>-238.662</v>
+        <v>-201.434</v>
       </c>
       <c r="C19" s="2" t="n">
-        <v>225.084</v>
+        <v>238.254</v>
       </c>
       <c r="D19" s="2" t="n"/>
       <c r="E19" s="2" t="n"/>
@@ -4190,10 +4190,10 @@
         </is>
       </c>
       <c r="B20" s="2" t="n">
-        <v>-238.662</v>
+        <v>-201.434</v>
       </c>
       <c r="C20" s="2" t="n">
-        <v>216.084</v>
+        <v>229.254</v>
       </c>
       <c r="D20" s="2" t="n"/>
       <c r="E20" s="2" t="n"/>
@@ -4207,10 +4207,10 @@
         </is>
       </c>
       <c r="B21" s="2" t="n">
-        <v>-238.662</v>
+        <v>-201.434</v>
       </c>
       <c r="C21" s="2" t="n">
-        <v>207.084</v>
+        <v>220.254</v>
       </c>
       <c r="D21" s="2" t="n"/>
       <c r="E21" s="2" t="n"/>
@@ -4224,10 +4224,10 @@
         </is>
       </c>
       <c r="B22" s="2" t="n">
-        <v>-238.662</v>
+        <v>-201.434</v>
       </c>
       <c r="C22" s="2" t="n">
-        <v>198.084</v>
+        <v>211.254</v>
       </c>
       <c r="D22" s="2" t="n"/>
       <c r="E22" s="2" t="n"/>
@@ -4241,10 +4241,10 @@
         </is>
       </c>
       <c r="B23" s="2" t="n">
-        <v>-238.662</v>
+        <v>-201.434</v>
       </c>
       <c r="C23" s="2" t="n">
-        <v>189.084</v>
+        <v>202.254</v>
       </c>
       <c r="D23" s="2" t="n"/>
       <c r="E23" s="2" t="n"/>
@@ -4258,10 +4258,10 @@
         </is>
       </c>
       <c r="B24" s="2" t="n">
-        <v>-238.662</v>
+        <v>-201.434</v>
       </c>
       <c r="C24" s="2" t="n">
-        <v>180.084</v>
+        <v>193.254</v>
       </c>
       <c r="D24" s="2" t="n"/>
       <c r="E24" s="2" t="n"/>
@@ -4275,10 +4275,10 @@
         </is>
       </c>
       <c r="B25" s="2" t="n">
-        <v>-238.662</v>
+        <v>-201.434</v>
       </c>
       <c r="C25" s="2" t="n">
-        <v>171.084</v>
+        <v>184.254</v>
       </c>
       <c r="D25" s="2" t="n"/>
       <c r="E25" s="2" t="n"/>
@@ -4292,10 +4292,10 @@
         </is>
       </c>
       <c r="B26" s="2" t="n">
-        <v>-247.662</v>
+        <v>-210.434</v>
       </c>
       <c r="C26" s="2" t="n">
-        <v>270.084</v>
+        <v>283.254</v>
       </c>
       <c r="D26" s="2" t="n"/>
       <c r="E26" s="2" t="n"/>
@@ -4309,10 +4309,10 @@
         </is>
       </c>
       <c r="B27" s="2" t="n">
-        <v>-247.662</v>
+        <v>-210.434</v>
       </c>
       <c r="C27" s="2" t="n">
-        <v>261.084</v>
+        <v>274.254</v>
       </c>
       <c r="D27" s="2" t="n"/>
       <c r="E27" s="2" t="n"/>
@@ -4326,10 +4326,10 @@
         </is>
       </c>
       <c r="B28" s="2" t="n">
-        <v>-247.662</v>
+        <v>-210.434</v>
       </c>
       <c r="C28" s="2" t="n">
-        <v>252.084</v>
+        <v>265.254</v>
       </c>
       <c r="D28" s="2" t="n"/>
       <c r="E28" s="2" t="n"/>
@@ -4343,10 +4343,10 @@
         </is>
       </c>
       <c r="B29" s="2" t="n">
-        <v>-247.662</v>
+        <v>-210.434</v>
       </c>
       <c r="C29" s="2" t="n">
-        <v>243.084</v>
+        <v>256.254</v>
       </c>
       <c r="D29" s="2" t="n"/>
       <c r="E29" s="2" t="n"/>
@@ -4360,10 +4360,10 @@
         </is>
       </c>
       <c r="B30" s="2" t="n">
-        <v>-247.662</v>
+        <v>-210.434</v>
       </c>
       <c r="C30" s="2" t="n">
-        <v>234.084</v>
+        <v>247.254</v>
       </c>
       <c r="D30" s="2" t="n"/>
       <c r="E30" s="2" t="n"/>
@@ -4377,10 +4377,10 @@
         </is>
       </c>
       <c r="B31" s="2" t="n">
-        <v>-247.662</v>
+        <v>-210.434</v>
       </c>
       <c r="C31" s="2" t="n">
-        <v>225.084</v>
+        <v>238.254</v>
       </c>
       <c r="D31" s="2" t="n"/>
       <c r="E31" s="2" t="n"/>
@@ -4394,10 +4394,10 @@
         </is>
       </c>
       <c r="B32" s="2" t="n">
-        <v>-247.662</v>
+        <v>-210.434</v>
       </c>
       <c r="C32" s="2" t="n">
-        <v>216.084</v>
+        <v>229.254</v>
       </c>
       <c r="D32" s="2" t="n"/>
       <c r="E32" s="2" t="n"/>
@@ -4411,10 +4411,10 @@
         </is>
       </c>
       <c r="B33" s="2" t="n">
-        <v>-247.662</v>
+        <v>-210.434</v>
       </c>
       <c r="C33" s="2" t="n">
-        <v>207.084</v>
+        <v>220.254</v>
       </c>
       <c r="D33" s="2" t="n"/>
       <c r="E33" s="2" t="n"/>
@@ -4428,10 +4428,10 @@
         </is>
       </c>
       <c r="B34" s="2" t="n">
-        <v>-247.662</v>
+        <v>-210.434</v>
       </c>
       <c r="C34" s="2" t="n">
-        <v>198.084</v>
+        <v>211.254</v>
       </c>
       <c r="D34" s="2" t="n"/>
       <c r="E34" s="2" t="n"/>
@@ -4445,10 +4445,10 @@
         </is>
       </c>
       <c r="B35" s="2" t="n">
-        <v>-247.662</v>
+        <v>-210.434</v>
       </c>
       <c r="C35" s="2" t="n">
-        <v>189.084</v>
+        <v>202.254</v>
       </c>
       <c r="D35" s="2" t="n"/>
       <c r="E35" s="2" t="n"/>
@@ -4462,10 +4462,10 @@
         </is>
       </c>
       <c r="B36" s="2" t="n">
-        <v>-247.662</v>
+        <v>-210.434</v>
       </c>
       <c r="C36" s="2" t="n">
-        <v>180.084</v>
+        <v>193.254</v>
       </c>
       <c r="D36" s="2" t="n"/>
       <c r="E36" s="2" t="n"/>
@@ -4479,10 +4479,10 @@
         </is>
       </c>
       <c r="B37" s="2" t="n">
-        <v>-247.662</v>
+        <v>-210.434</v>
       </c>
       <c r="C37" s="2" t="n">
-        <v>171.084</v>
+        <v>184.254</v>
       </c>
       <c r="D37" s="2" t="n"/>
       <c r="E37" s="2" t="n"/>
@@ -4496,10 +4496,10 @@
         </is>
       </c>
       <c r="B38" s="2" t="n">
-        <v>-256.662</v>
+        <v>-219.434</v>
       </c>
       <c r="C38" s="2" t="n">
-        <v>270.084</v>
+        <v>283.254</v>
       </c>
       <c r="D38" s="2" t="n"/>
       <c r="E38" s="2" t="n"/>
@@ -4513,10 +4513,10 @@
         </is>
       </c>
       <c r="B39" s="2" t="n">
-        <v>-256.662</v>
+        <v>-219.434</v>
       </c>
       <c r="C39" s="2" t="n">
-        <v>261.084</v>
+        <v>274.254</v>
       </c>
       <c r="D39" s="2" t="n"/>
       <c r="E39" s="2" t="n"/>
@@ -4530,10 +4530,10 @@
         </is>
       </c>
       <c r="B40" s="2" t="n">
-        <v>-256.662</v>
+        <v>-219.434</v>
       </c>
       <c r="C40" s="2" t="n">
-        <v>252.084</v>
+        <v>265.254</v>
       </c>
       <c r="D40" s="2" t="n"/>
       <c r="E40" s="2" t="n"/>
@@ -4547,10 +4547,10 @@
         </is>
       </c>
       <c r="B41" s="2" t="n">
-        <v>-256.662</v>
+        <v>-219.434</v>
       </c>
       <c r="C41" s="2" t="n">
-        <v>243.084</v>
+        <v>256.254</v>
       </c>
       <c r="D41" s="2" t="n"/>
       <c r="E41" s="2" t="n"/>
@@ -4564,10 +4564,10 @@
         </is>
       </c>
       <c r="B42" s="2" t="n">
-        <v>-256.662</v>
+        <v>-219.434</v>
       </c>
       <c r="C42" s="2" t="n">
-        <v>234.084</v>
+        <v>247.254</v>
       </c>
       <c r="D42" s="2" t="n"/>
       <c r="E42" s="2" t="n"/>
@@ -4581,10 +4581,10 @@
         </is>
       </c>
       <c r="B43" s="2" t="n">
-        <v>-256.662</v>
+        <v>-219.434</v>
       </c>
       <c r="C43" s="2" t="n">
-        <v>225.084</v>
+        <v>238.254</v>
       </c>
       <c r="D43" s="2" t="n"/>
       <c r="E43" s="2" t="n"/>
@@ -4598,10 +4598,10 @@
         </is>
       </c>
       <c r="B44" s="2" t="n">
-        <v>-256.662</v>
+        <v>-219.434</v>
       </c>
       <c r="C44" s="2" t="n">
-        <v>216.084</v>
+        <v>229.254</v>
       </c>
       <c r="D44" s="2" t="n"/>
       <c r="E44" s="2" t="n"/>
@@ -4615,10 +4615,10 @@
         </is>
       </c>
       <c r="B45" s="2" t="n">
-        <v>-256.662</v>
+        <v>-219.434</v>
       </c>
       <c r="C45" s="2" t="n">
-        <v>207.084</v>
+        <v>220.254</v>
       </c>
       <c r="D45" s="2" t="n"/>
       <c r="E45" s="2" t="n"/>
@@ -4632,10 +4632,10 @@
         </is>
       </c>
       <c r="B46" s="2" t="n">
-        <v>-256.662</v>
+        <v>-219.434</v>
       </c>
       <c r="C46" s="2" t="n">
-        <v>198.084</v>
+        <v>211.254</v>
       </c>
       <c r="D46" s="2" t="n"/>
       <c r="E46" s="2" t="n"/>
@@ -4649,10 +4649,10 @@
         </is>
       </c>
       <c r="B47" s="2" t="n">
-        <v>-256.662</v>
+        <v>-219.434</v>
       </c>
       <c r="C47" s="2" t="n">
-        <v>189.084</v>
+        <v>202.254</v>
       </c>
       <c r="D47" s="2" t="n"/>
       <c r="E47" s="2" t="n"/>
@@ -4666,10 +4666,10 @@
         </is>
       </c>
       <c r="B48" s="2" t="n">
-        <v>-256.662</v>
+        <v>-219.434</v>
       </c>
       <c r="C48" s="2" t="n">
-        <v>180.084</v>
+        <v>193.254</v>
       </c>
       <c r="D48" s="2" t="n"/>
       <c r="E48" s="2" t="n"/>
@@ -4683,10 +4683,10 @@
         </is>
       </c>
       <c r="B49" s="2" t="n">
-        <v>-256.662</v>
+        <v>-219.434</v>
       </c>
       <c r="C49" s="2" t="n">
-        <v>171.084</v>
+        <v>184.254</v>
       </c>
       <c r="D49" s="2" t="n"/>
       <c r="E49" s="2" t="n"/>
@@ -4700,10 +4700,10 @@
         </is>
       </c>
       <c r="B50" s="2" t="n">
-        <v>-265.662</v>
+        <v>-228.434</v>
       </c>
       <c r="C50" s="2" t="n">
-        <v>270.084</v>
+        <v>283.254</v>
       </c>
       <c r="D50" s="2" t="n"/>
       <c r="E50" s="2" t="n"/>
@@ -4717,10 +4717,10 @@
         </is>
       </c>
       <c r="B51" s="2" t="n">
-        <v>-265.662</v>
+        <v>-228.434</v>
       </c>
       <c r="C51" s="2" t="n">
-        <v>261.084</v>
+        <v>274.254</v>
       </c>
       <c r="D51" s="2" t="n"/>
       <c r="E51" s="2" t="n"/>
@@ -4734,10 +4734,10 @@
         </is>
       </c>
       <c r="B52" s="2" t="n">
-        <v>-265.662</v>
+        <v>-228.434</v>
       </c>
       <c r="C52" s="2" t="n">
-        <v>252.084</v>
+        <v>265.254</v>
       </c>
       <c r="D52" s="2" t="n"/>
       <c r="E52" s="2" t="n"/>
@@ -4751,10 +4751,10 @@
         </is>
       </c>
       <c r="B53" s="2" t="n">
-        <v>-265.662</v>
+        <v>-228.434</v>
       </c>
       <c r="C53" s="2" t="n">
-        <v>243.084</v>
+        <v>256.254</v>
       </c>
       <c r="D53" s="2" t="n"/>
       <c r="E53" s="2" t="n"/>
@@ -4768,10 +4768,10 @@
         </is>
       </c>
       <c r="B54" s="2" t="n">
-        <v>-265.662</v>
+        <v>-228.434</v>
       </c>
       <c r="C54" s="2" t="n">
-        <v>234.084</v>
+        <v>247.254</v>
       </c>
       <c r="D54" s="2" t="n"/>
       <c r="E54" s="2" t="n"/>
@@ -4785,10 +4785,10 @@
         </is>
       </c>
       <c r="B55" s="2" t="n">
-        <v>-265.662</v>
+        <v>-228.434</v>
       </c>
       <c r="C55" s="2" t="n">
-        <v>225.084</v>
+        <v>238.254</v>
       </c>
       <c r="D55" s="2" t="n"/>
       <c r="E55" s="2" t="n"/>
@@ -4802,10 +4802,10 @@
         </is>
       </c>
       <c r="B56" s="2" t="n">
-        <v>-265.662</v>
+        <v>-228.434</v>
       </c>
       <c r="C56" s="2" t="n">
-        <v>216.084</v>
+        <v>229.254</v>
       </c>
       <c r="D56" s="2" t="n"/>
       <c r="E56" s="2" t="n"/>
@@ -4819,10 +4819,10 @@
         </is>
       </c>
       <c r="B57" s="2" t="n">
-        <v>-265.662</v>
+        <v>-228.434</v>
       </c>
       <c r="C57" s="2" t="n">
-        <v>207.084</v>
+        <v>220.254</v>
       </c>
       <c r="D57" s="2" t="n"/>
       <c r="E57" s="2" t="n"/>
@@ -4836,10 +4836,10 @@
         </is>
       </c>
       <c r="B58" s="2" t="n">
-        <v>-265.662</v>
+        <v>-228.434</v>
       </c>
       <c r="C58" s="2" t="n">
-        <v>198.084</v>
+        <v>211.254</v>
       </c>
       <c r="D58" s="2" t="n"/>
       <c r="E58" s="2" t="n"/>
@@ -4853,10 +4853,10 @@
         </is>
       </c>
       <c r="B59" s="2" t="n">
-        <v>-265.662</v>
+        <v>-228.434</v>
       </c>
       <c r="C59" s="2" t="n">
-        <v>189.084</v>
+        <v>202.254</v>
       </c>
       <c r="D59" s="2" t="n"/>
       <c r="E59" s="2" t="n"/>
@@ -4870,10 +4870,10 @@
         </is>
       </c>
       <c r="B60" s="2" t="n">
-        <v>-265.662</v>
+        <v>-228.434</v>
       </c>
       <c r="C60" s="2" t="n">
-        <v>180.084</v>
+        <v>193.254</v>
       </c>
       <c r="D60" s="2" t="n"/>
       <c r="E60" s="2" t="n"/>
@@ -4887,10 +4887,10 @@
         </is>
       </c>
       <c r="B61" s="2" t="n">
-        <v>-265.662</v>
+        <v>-228.434</v>
       </c>
       <c r="C61" s="2" t="n">
-        <v>171.084</v>
+        <v>184.254</v>
       </c>
       <c r="D61" s="2" t="n"/>
       <c r="E61" s="2" t="n"/>
@@ -4904,10 +4904,10 @@
         </is>
       </c>
       <c r="B62" s="2" t="n">
-        <v>-274.662</v>
+        <v>-237.434</v>
       </c>
       <c r="C62" s="2" t="n">
-        <v>270.084</v>
+        <v>283.254</v>
       </c>
       <c r="D62" s="2" t="n"/>
       <c r="E62" s="2" t="n"/>
@@ -4921,10 +4921,10 @@
         </is>
       </c>
       <c r="B63" s="2" t="n">
-        <v>-274.662</v>
+        <v>-237.434</v>
       </c>
       <c r="C63" s="2" t="n">
-        <v>261.084</v>
+        <v>274.254</v>
       </c>
       <c r="D63" s="2" t="n"/>
       <c r="E63" s="2" t="n"/>
@@ -4938,10 +4938,10 @@
         </is>
       </c>
       <c r="B64" s="2" t="n">
-        <v>-274.662</v>
+        <v>-237.434</v>
       </c>
       <c r="C64" s="2" t="n">
-        <v>252.084</v>
+        <v>265.254</v>
       </c>
       <c r="D64" s="2" t="n"/>
       <c r="E64" s="2" t="n"/>
@@ -4955,10 +4955,10 @@
         </is>
       </c>
       <c r="B65" s="2" t="n">
-        <v>-274.662</v>
+        <v>-237.434</v>
       </c>
       <c r="C65" s="2" t="n">
-        <v>243.084</v>
+        <v>256.254</v>
       </c>
       <c r="D65" s="2" t="n"/>
       <c r="E65" s="2" t="n"/>
@@ -4972,10 +4972,10 @@
         </is>
       </c>
       <c r="B66" s="2" t="n">
-        <v>-274.662</v>
+        <v>-237.434</v>
       </c>
       <c r="C66" s="2" t="n">
-        <v>234.084</v>
+        <v>247.254</v>
       </c>
       <c r="D66" s="2" t="n"/>
       <c r="E66" s="2" t="n"/>
@@ -4989,10 +4989,10 @@
         </is>
       </c>
       <c r="B67" s="2" t="n">
-        <v>-274.662</v>
+        <v>-237.434</v>
       </c>
       <c r="C67" s="2" t="n">
-        <v>225.084</v>
+        <v>238.254</v>
       </c>
       <c r="D67" s="2" t="n"/>
       <c r="E67" s="2" t="n"/>
@@ -5006,10 +5006,10 @@
         </is>
       </c>
       <c r="B68" s="2" t="n">
-        <v>-274.662</v>
+        <v>-237.434</v>
       </c>
       <c r="C68" s="2" t="n">
-        <v>216.084</v>
+        <v>229.254</v>
       </c>
       <c r="D68" s="2" t="n"/>
       <c r="E68" s="2" t="n"/>
@@ -5023,10 +5023,10 @@
         </is>
       </c>
       <c r="B69" s="2" t="n">
-        <v>-274.662</v>
+        <v>-237.434</v>
       </c>
       <c r="C69" s="2" t="n">
-        <v>207.084</v>
+        <v>220.254</v>
       </c>
       <c r="D69" s="2" t="n"/>
       <c r="E69" s="2" t="n"/>
@@ -5040,10 +5040,10 @@
         </is>
       </c>
       <c r="B70" s="2" t="n">
-        <v>-274.662</v>
+        <v>-237.434</v>
       </c>
       <c r="C70" s="2" t="n">
-        <v>198.084</v>
+        <v>211.254</v>
       </c>
       <c r="D70" s="2" t="n"/>
       <c r="E70" s="2" t="n"/>
@@ -5057,10 +5057,10 @@
         </is>
       </c>
       <c r="B71" s="2" t="n">
-        <v>-274.662</v>
+        <v>-237.434</v>
       </c>
       <c r="C71" s="2" t="n">
-        <v>189.084</v>
+        <v>202.254</v>
       </c>
       <c r="D71" s="2" t="n"/>
       <c r="E71" s="2" t="n"/>
@@ -5074,10 +5074,10 @@
         </is>
       </c>
       <c r="B72" s="2" t="n">
-        <v>-274.662</v>
+        <v>-237.434</v>
       </c>
       <c r="C72" s="2" t="n">
-        <v>180.084</v>
+        <v>193.254</v>
       </c>
       <c r="D72" s="2" t="n"/>
       <c r="E72" s="2" t="n"/>
@@ -5091,10 +5091,10 @@
         </is>
       </c>
       <c r="B73" s="2" t="n">
-        <v>-274.662</v>
+        <v>-237.434</v>
       </c>
       <c r="C73" s="2" t="n">
-        <v>171.084</v>
+        <v>184.254</v>
       </c>
       <c r="D73" s="2" t="n"/>
       <c r="E73" s="2" t="n"/>
@@ -5108,10 +5108,10 @@
         </is>
       </c>
       <c r="B74" s="2" t="n">
-        <v>-283.662</v>
+        <v>-246.434</v>
       </c>
       <c r="C74" s="2" t="n">
-        <v>270.084</v>
+        <v>283.254</v>
       </c>
       <c r="D74" s="2" t="n"/>
       <c r="E74" s="2" t="n"/>
@@ -5125,10 +5125,10 @@
         </is>
       </c>
       <c r="B75" s="2" t="n">
-        <v>-283.662</v>
+        <v>-246.434</v>
       </c>
       <c r="C75" s="2" t="n">
-        <v>261.084</v>
+        <v>274.254</v>
       </c>
       <c r="D75" s="2" t="n"/>
       <c r="E75" s="2" t="n"/>
@@ -5142,10 +5142,10 @@
         </is>
       </c>
       <c r="B76" s="2" t="n">
-        <v>-283.662</v>
+        <v>-246.434</v>
       </c>
       <c r="C76" s="2" t="n">
-        <v>252.084</v>
+        <v>265.254</v>
       </c>
       <c r="D76" s="2" t="n"/>
       <c r="E76" s="2" t="n"/>
@@ -5159,10 +5159,10 @@
         </is>
       </c>
       <c r="B77" s="2" t="n">
-        <v>-283.662</v>
+        <v>-246.434</v>
       </c>
       <c r="C77" s="2" t="n">
-        <v>243.084</v>
+        <v>256.254</v>
       </c>
       <c r="D77" s="2" t="n"/>
       <c r="E77" s="2" t="n"/>
@@ -5176,10 +5176,10 @@
         </is>
       </c>
       <c r="B78" s="2" t="n">
-        <v>-283.662</v>
+        <v>-246.434</v>
       </c>
       <c r="C78" s="2" t="n">
-        <v>234.084</v>
+        <v>247.254</v>
       </c>
       <c r="D78" s="2" t="n"/>
       <c r="E78" s="2" t="n"/>
@@ -5193,10 +5193,10 @@
         </is>
       </c>
       <c r="B79" s="2" t="n">
-        <v>-283.662</v>
+        <v>-246.434</v>
       </c>
       <c r="C79" s="2" t="n">
-        <v>225.084</v>
+        <v>238.254</v>
       </c>
       <c r="D79" s="2" t="n"/>
       <c r="E79" s="2" t="n"/>
@@ -5210,10 +5210,10 @@
         </is>
       </c>
       <c r="B80" s="2" t="n">
-        <v>-283.662</v>
+        <v>-246.434</v>
       </c>
       <c r="C80" s="2" t="n">
-        <v>216.084</v>
+        <v>229.254</v>
       </c>
       <c r="D80" s="2" t="n"/>
       <c r="E80" s="2" t="n"/>
@@ -5227,10 +5227,10 @@
         </is>
       </c>
       <c r="B81" s="2" t="n">
-        <v>-283.662</v>
+        <v>-246.434</v>
       </c>
       <c r="C81" s="2" t="n">
-        <v>207.084</v>
+        <v>220.254</v>
       </c>
       <c r="D81" s="2" t="n"/>
       <c r="E81" s="2" t="n"/>
@@ -5244,10 +5244,10 @@
         </is>
       </c>
       <c r="B82" s="2" t="n">
-        <v>-283.662</v>
+        <v>-246.434</v>
       </c>
       <c r="C82" s="2" t="n">
-        <v>198.084</v>
+        <v>211.254</v>
       </c>
       <c r="D82" s="2" t="n"/>
       <c r="E82" s="2" t="n"/>
@@ -5261,10 +5261,10 @@
         </is>
       </c>
       <c r="B83" s="2" t="n">
-        <v>-283.662</v>
+        <v>-246.434</v>
       </c>
       <c r="C83" s="2" t="n">
-        <v>189.084</v>
+        <v>202.254</v>
       </c>
       <c r="D83" s="2" t="n"/>
       <c r="E83" s="2" t="n"/>
@@ -5278,10 +5278,10 @@
         </is>
       </c>
       <c r="B84" s="2" t="n">
-        <v>-283.662</v>
+        <v>-246.434</v>
       </c>
       <c r="C84" s="2" t="n">
-        <v>180.084</v>
+        <v>193.254</v>
       </c>
       <c r="D84" s="2" t="n"/>
       <c r="E84" s="2" t="n"/>
@@ -5295,10 +5295,10 @@
         </is>
       </c>
       <c r="B85" s="2" t="n">
-        <v>-283.662</v>
+        <v>-246.434</v>
       </c>
       <c r="C85" s="2" t="n">
-        <v>171.084</v>
+        <v>184.254</v>
       </c>
       <c r="D85" s="2" t="n"/>
       <c r="E85" s="2" t="n"/>
@@ -5312,10 +5312,10 @@
         </is>
       </c>
       <c r="B86" s="2" t="n">
-        <v>-292.662</v>
+        <v>-255.434</v>
       </c>
       <c r="C86" s="2" t="n">
-        <v>270.084</v>
+        <v>283.254</v>
       </c>
       <c r="D86" s="2" t="n"/>
       <c r="E86" s="2" t="n"/>
@@ -5329,10 +5329,10 @@
         </is>
       </c>
       <c r="B87" s="2" t="n">
-        <v>-292.662</v>
+        <v>-255.434</v>
       </c>
       <c r="C87" s="2" t="n">
-        <v>261.084</v>
+        <v>274.254</v>
       </c>
       <c r="D87" s="2" t="n"/>
       <c r="E87" s="2" t="n"/>
@@ -5346,10 +5346,10 @@
         </is>
       </c>
       <c r="B88" s="2" t="n">
-        <v>-292.662</v>
+        <v>-255.434</v>
       </c>
       <c r="C88" s="2" t="n">
-        <v>252.084</v>
+        <v>265.254</v>
       </c>
       <c r="D88" s="2" t="n"/>
       <c r="E88" s="2" t="n"/>
@@ -5363,10 +5363,10 @@
         </is>
       </c>
       <c r="B89" s="2" t="n">
-        <v>-292.662</v>
+        <v>-255.434</v>
       </c>
       <c r="C89" s="2" t="n">
-        <v>243.084</v>
+        <v>256.254</v>
       </c>
       <c r="D89" s="2" t="n"/>
       <c r="E89" s="2" t="n"/>
@@ -5380,10 +5380,10 @@
         </is>
       </c>
       <c r="B90" s="2" t="n">
-        <v>-292.662</v>
+        <v>-255.434</v>
       </c>
       <c r="C90" s="2" t="n">
-        <v>234.084</v>
+        <v>247.254</v>
       </c>
       <c r="D90" s="2" t="n"/>
       <c r="E90" s="2" t="n"/>
@@ -5397,10 +5397,10 @@
         </is>
       </c>
       <c r="B91" s="2" t="n">
-        <v>-292.662</v>
+        <v>-255.434</v>
       </c>
       <c r="C91" s="2" t="n">
-        <v>225.084</v>
+        <v>238.254</v>
       </c>
       <c r="D91" s="2" t="n"/>
       <c r="E91" s="2" t="n"/>
@@ -5414,10 +5414,10 @@
         </is>
       </c>
       <c r="B92" s="2" t="n">
-        <v>-292.662</v>
+        <v>-255.434</v>
       </c>
       <c r="C92" s="2" t="n">
-        <v>216.084</v>
+        <v>229.254</v>
       </c>
       <c r="D92" s="2" t="n"/>
       <c r="E92" s="2" t="n"/>
@@ -5431,10 +5431,10 @@
         </is>
       </c>
       <c r="B93" s="2" t="n">
-        <v>-292.662</v>
+        <v>-255.434</v>
       </c>
       <c r="C93" s="2" t="n">
-        <v>207.084</v>
+        <v>220.254</v>
       </c>
       <c r="D93" s="2" t="n"/>
       <c r="E93" s="2" t="n"/>
@@ -5448,10 +5448,10 @@
         </is>
       </c>
       <c r="B94" s="2" t="n">
-        <v>-292.662</v>
+        <v>-255.434</v>
       </c>
       <c r="C94" s="2" t="n">
-        <v>198.084</v>
+        <v>211.254</v>
       </c>
       <c r="D94" s="2" t="n"/>
       <c r="E94" s="2" t="n"/>
@@ -5465,10 +5465,10 @@
         </is>
       </c>
       <c r="B95" s="2" t="n">
-        <v>-292.662</v>
+        <v>-255.434</v>
       </c>
       <c r="C95" s="2" t="n">
-        <v>189.084</v>
+        <v>202.254</v>
       </c>
       <c r="D95" s="2" t="n"/>
       <c r="E95" s="2" t="n"/>
@@ -5482,10 +5482,10 @@
         </is>
       </c>
       <c r="B96" s="2" t="n">
-        <v>-292.662</v>
+        <v>-255.434</v>
       </c>
       <c r="C96" s="2" t="n">
-        <v>180.084</v>
+        <v>193.254</v>
       </c>
       <c r="D96" s="2" t="n"/>
       <c r="E96" s="2" t="n"/>
@@ -5499,10 +5499,10 @@
         </is>
       </c>
       <c r="B97" s="2" t="n">
-        <v>-292.662</v>
+        <v>-255.434</v>
       </c>
       <c r="C97" s="2" t="n">
-        <v>171.084</v>
+        <v>184.254</v>
       </c>
       <c r="D97" s="2" t="n"/>
       <c r="E97" s="2" t="n"/>
@@ -5576,10 +5576,10 @@
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>-329.796</v>
+        <v>-292.526</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>204.488</v>
+        <v>218.16</v>
       </c>
       <c r="D2" s="2" t="n"/>
       <c r="E2" s="2" t="n"/>
@@ -5593,10 +5593,10 @@
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>-329.796</v>
+        <v>-292.526</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>195.488</v>
+        <v>209.16</v>
       </c>
       <c r="D3" s="2" t="n"/>
       <c r="E3" s="2" t="n"/>
@@ -5610,10 +5610,10 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>-329.796</v>
+        <v>-292.526</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>186.488</v>
+        <v>200.16</v>
       </c>
       <c r="D4" s="2" t="n"/>
       <c r="E4" s="2" t="n"/>
@@ -5627,10 +5627,10 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>-329.796</v>
+        <v>-292.526</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>177.488</v>
+        <v>191.16</v>
       </c>
       <c r="D5" s="2" t="n"/>
       <c r="E5" s="2" t="n"/>
@@ -5644,10 +5644,10 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>-329.796</v>
+        <v>-292.526</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>168.488</v>
+        <v>182.16</v>
       </c>
       <c r="D6" s="2" t="n"/>
       <c r="E6" s="2" t="n"/>
@@ -5661,10 +5661,10 @@
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>-329.796</v>
+        <v>-292.526</v>
       </c>
       <c r="C7" s="2" t="n">
-        <v>159.488</v>
+        <v>173.16</v>
       </c>
       <c r="D7" s="2" t="n"/>
       <c r="E7" s="2" t="n"/>
@@ -5678,10 +5678,10 @@
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>-329.796</v>
+        <v>-292.526</v>
       </c>
       <c r="C8" s="2" t="n">
-        <v>150.488</v>
+        <v>164.16</v>
       </c>
       <c r="D8" s="2" t="n"/>
       <c r="E8" s="2" t="n"/>
@@ -5695,10 +5695,10 @@
         </is>
       </c>
       <c r="B9" s="2" t="n">
-        <v>-329.796</v>
+        <v>-292.526</v>
       </c>
       <c r="C9" s="2" t="n">
-        <v>141.488</v>
+        <v>155.16</v>
       </c>
       <c r="D9" s="2" t="n"/>
       <c r="E9" s="2" t="n"/>
@@ -5712,10 +5712,10 @@
         </is>
       </c>
       <c r="B10" s="2" t="n">
-        <v>-329.796</v>
+        <v>-292.526</v>
       </c>
       <c r="C10" s="2" t="n">
-        <v>132.488</v>
+        <v>146.16</v>
       </c>
       <c r="D10" s="2" t="n"/>
       <c r="E10" s="2" t="n"/>
@@ -5729,10 +5729,10 @@
         </is>
       </c>
       <c r="B11" s="2" t="n">
-        <v>-329.796</v>
+        <v>-292.526</v>
       </c>
       <c r="C11" s="2" t="n">
-        <v>123.488</v>
+        <v>137.16</v>
       </c>
       <c r="D11" s="2" t="n"/>
       <c r="E11" s="2" t="n"/>
@@ -5746,10 +5746,10 @@
         </is>
       </c>
       <c r="B12" s="2" t="n">
-        <v>-329.796</v>
+        <v>-292.526</v>
       </c>
       <c r="C12" s="2" t="n">
-        <v>114.488</v>
+        <v>128.16</v>
       </c>
       <c r="D12" s="2" t="n"/>
       <c r="E12" s="2" t="n"/>
@@ -5763,10 +5763,10 @@
         </is>
       </c>
       <c r="B13" s="2" t="n">
-        <v>-329.796</v>
+        <v>-292.526</v>
       </c>
       <c r="C13" s="2" t="n">
-        <v>105.488</v>
+        <v>119.16</v>
       </c>
       <c r="D13" s="2" t="n"/>
       <c r="E13" s="2" t="n"/>
@@ -5780,10 +5780,10 @@
         </is>
       </c>
       <c r="B14" s="2" t="n">
-        <v>-338.796</v>
+        <v>-301.526</v>
       </c>
       <c r="C14" s="2" t="n">
-        <v>204.488</v>
+        <v>218.16</v>
       </c>
       <c r="D14" s="2" t="n"/>
       <c r="E14" s="2" t="n"/>
@@ -5797,10 +5797,10 @@
         </is>
       </c>
       <c r="B15" s="2" t="n">
-        <v>-338.796</v>
+        <v>-301.526</v>
       </c>
       <c r="C15" s="2" t="n">
-        <v>195.488</v>
+        <v>209.16</v>
       </c>
       <c r="D15" s="2" t="n"/>
       <c r="E15" s="2" t="n"/>
@@ -5814,10 +5814,10 @@
         </is>
       </c>
       <c r="B16" s="2" t="n">
-        <v>-338.796</v>
+        <v>-301.526</v>
       </c>
       <c r="C16" s="2" t="n">
-        <v>186.488</v>
+        <v>200.16</v>
       </c>
       <c r="D16" s="2" t="n"/>
       <c r="E16" s="2" t="n"/>
@@ -5831,10 +5831,10 @@
         </is>
       </c>
       <c r="B17" s="2" t="n">
-        <v>-338.796</v>
+        <v>-301.526</v>
       </c>
       <c r="C17" s="2" t="n">
-        <v>177.488</v>
+        <v>191.16</v>
       </c>
       <c r="D17" s="2" t="n"/>
       <c r="E17" s="2" t="n"/>
@@ -5848,10 +5848,10 @@
         </is>
       </c>
       <c r="B18" s="2" t="n">
-        <v>-338.796</v>
+        <v>-301.526</v>
       </c>
       <c r="C18" s="2" t="n">
-        <v>168.488</v>
+        <v>182.16</v>
       </c>
       <c r="D18" s="2" t="n"/>
       <c r="E18" s="2" t="n"/>
@@ -5865,10 +5865,10 @@
         </is>
       </c>
       <c r="B19" s="2" t="n">
-        <v>-338.796</v>
+        <v>-301.526</v>
       </c>
       <c r="C19" s="2" t="n">
-        <v>159.488</v>
+        <v>173.16</v>
       </c>
       <c r="D19" s="2" t="n"/>
       <c r="E19" s="2" t="n"/>
@@ -5882,10 +5882,10 @@
         </is>
       </c>
       <c r="B20" s="2" t="n">
-        <v>-338.796</v>
+        <v>-301.526</v>
       </c>
       <c r="C20" s="2" t="n">
-        <v>150.488</v>
+        <v>164.16</v>
       </c>
       <c r="D20" s="2" t="n"/>
       <c r="E20" s="2" t="n"/>
@@ -5899,10 +5899,10 @@
         </is>
       </c>
       <c r="B21" s="2" t="n">
-        <v>-338.796</v>
+        <v>-301.526</v>
       </c>
       <c r="C21" s="2" t="n">
-        <v>141.488</v>
+        <v>155.16</v>
       </c>
       <c r="D21" s="2" t="n"/>
       <c r="E21" s="2" t="n"/>
@@ -5916,10 +5916,10 @@
         </is>
       </c>
       <c r="B22" s="2" t="n">
-        <v>-338.796</v>
+        <v>-301.526</v>
       </c>
       <c r="C22" s="2" t="n">
-        <v>132.488</v>
+        <v>146.16</v>
       </c>
       <c r="D22" s="2" t="n"/>
       <c r="E22" s="2" t="n"/>
@@ -5933,10 +5933,10 @@
         </is>
       </c>
       <c r="B23" s="2" t="n">
-        <v>-338.796</v>
+        <v>-301.526</v>
       </c>
       <c r="C23" s="2" t="n">
-        <v>123.488</v>
+        <v>137.16</v>
       </c>
       <c r="D23" s="2" t="n"/>
       <c r="E23" s="2" t="n"/>
@@ -5950,10 +5950,10 @@
         </is>
       </c>
       <c r="B24" s="2" t="n">
-        <v>-338.796</v>
+        <v>-301.526</v>
       </c>
       <c r="C24" s="2" t="n">
-        <v>114.488</v>
+        <v>128.16</v>
       </c>
       <c r="D24" s="2" t="n"/>
       <c r="E24" s="2" t="n"/>
@@ -5967,10 +5967,10 @@
         </is>
       </c>
       <c r="B25" s="2" t="n">
-        <v>-338.796</v>
+        <v>-301.526</v>
       </c>
       <c r="C25" s="2" t="n">
-        <v>105.488</v>
+        <v>119.16</v>
       </c>
       <c r="D25" s="2" t="n"/>
       <c r="E25" s="2" t="n"/>
@@ -5984,10 +5984,10 @@
         </is>
       </c>
       <c r="B26" s="2" t="n">
-        <v>-347.796</v>
+        <v>-310.526</v>
       </c>
       <c r="C26" s="2" t="n">
-        <v>204.488</v>
+        <v>218.16</v>
       </c>
       <c r="D26" s="2" t="n"/>
       <c r="E26" s="2" t="n"/>
@@ -6001,10 +6001,10 @@
         </is>
       </c>
       <c r="B27" s="2" t="n">
-        <v>-347.796</v>
+        <v>-310.526</v>
       </c>
       <c r="C27" s="2" t="n">
-        <v>195.488</v>
+        <v>209.16</v>
       </c>
       <c r="D27" s="2" t="n"/>
       <c r="E27" s="2" t="n"/>
@@ -6018,10 +6018,10 @@
         </is>
       </c>
       <c r="B28" s="2" t="n">
-        <v>-347.796</v>
+        <v>-310.526</v>
       </c>
       <c r="C28" s="2" t="n">
-        <v>186.488</v>
+        <v>200.16</v>
       </c>
       <c r="D28" s="2" t="n"/>
       <c r="E28" s="2" t="n"/>
@@ -6035,10 +6035,10 @@
         </is>
       </c>
       <c r="B29" s="2" t="n">
-        <v>-347.796</v>
+        <v>-310.526</v>
       </c>
       <c r="C29" s="2" t="n">
-        <v>177.488</v>
+        <v>191.16</v>
       </c>
       <c r="D29" s="2" t="n"/>
       <c r="E29" s="2" t="n"/>
@@ -6052,10 +6052,10 @@
         </is>
       </c>
       <c r="B30" s="2" t="n">
-        <v>-347.796</v>
+        <v>-310.526</v>
       </c>
       <c r="C30" s="2" t="n">
-        <v>168.488</v>
+        <v>182.16</v>
       </c>
       <c r="D30" s="2" t="n"/>
       <c r="E30" s="2" t="n"/>
@@ -6069,10 +6069,10 @@
         </is>
       </c>
       <c r="B31" s="2" t="n">
-        <v>-347.796</v>
+        <v>-310.526</v>
       </c>
       <c r="C31" s="2" t="n">
-        <v>159.488</v>
+        <v>173.16</v>
       </c>
       <c r="D31" s="2" t="n"/>
       <c r="E31" s="2" t="n"/>
@@ -6086,10 +6086,10 @@
         </is>
       </c>
       <c r="B32" s="2" t="n">
-        <v>-347.796</v>
+        <v>-310.526</v>
       </c>
       <c r="C32" s="2" t="n">
-        <v>150.488</v>
+        <v>164.16</v>
       </c>
       <c r="D32" s="2" t="n"/>
       <c r="E32" s="2" t="n"/>
@@ -6103,10 +6103,10 @@
         </is>
       </c>
       <c r="B33" s="2" t="n">
-        <v>-347.796</v>
+        <v>-310.526</v>
       </c>
       <c r="C33" s="2" t="n">
-        <v>141.488</v>
+        <v>155.16</v>
       </c>
       <c r="D33" s="2" t="n"/>
       <c r="E33" s="2" t="n"/>
@@ -6120,10 +6120,10 @@
         </is>
       </c>
       <c r="B34" s="2" t="n">
-        <v>-347.796</v>
+        <v>-310.526</v>
       </c>
       <c r="C34" s="2" t="n">
-        <v>132.488</v>
+        <v>146.16</v>
       </c>
       <c r="D34" s="2" t="n"/>
       <c r="E34" s="2" t="n"/>
@@ -6137,10 +6137,10 @@
         </is>
       </c>
       <c r="B35" s="2" t="n">
-        <v>-347.796</v>
+        <v>-310.526</v>
       </c>
       <c r="C35" s="2" t="n">
-        <v>123.488</v>
+        <v>137.16</v>
       </c>
       <c r="D35" s="2" t="n"/>
       <c r="E35" s="2" t="n"/>
@@ -6154,10 +6154,10 @@
         </is>
       </c>
       <c r="B36" s="2" t="n">
-        <v>-347.796</v>
+        <v>-310.526</v>
       </c>
       <c r="C36" s="2" t="n">
-        <v>114.488</v>
+        <v>128.16</v>
       </c>
       <c r="D36" s="2" t="n"/>
       <c r="E36" s="2" t="n"/>
@@ -6171,10 +6171,10 @@
         </is>
       </c>
       <c r="B37" s="2" t="n">
-        <v>-347.796</v>
+        <v>-310.526</v>
       </c>
       <c r="C37" s="2" t="n">
-        <v>105.488</v>
+        <v>119.16</v>
       </c>
       <c r="D37" s="2" t="n"/>
       <c r="E37" s="2" t="n"/>
@@ -6188,10 +6188,10 @@
         </is>
       </c>
       <c r="B38" s="2" t="n">
-        <v>-356.796</v>
+        <v>-319.526</v>
       </c>
       <c r="C38" s="2" t="n">
-        <v>204.488</v>
+        <v>218.16</v>
       </c>
       <c r="D38" s="2" t="n"/>
       <c r="E38" s="2" t="n"/>
@@ -6205,10 +6205,10 @@
         </is>
       </c>
       <c r="B39" s="2" t="n">
-        <v>-356.796</v>
+        <v>-319.526</v>
       </c>
       <c r="C39" s="2" t="n">
-        <v>195.488</v>
+        <v>209.16</v>
       </c>
       <c r="D39" s="2" t="n"/>
       <c r="E39" s="2" t="n"/>
@@ -6222,10 +6222,10 @@
         </is>
       </c>
       <c r="B40" s="2" t="n">
-        <v>-356.796</v>
+        <v>-319.526</v>
       </c>
       <c r="C40" s="2" t="n">
-        <v>186.488</v>
+        <v>200.16</v>
       </c>
       <c r="D40" s="2" t="n"/>
       <c r="E40" s="2" t="n"/>
@@ -6239,10 +6239,10 @@
         </is>
       </c>
       <c r="B41" s="2" t="n">
-        <v>-356.796</v>
+        <v>-319.526</v>
       </c>
       <c r="C41" s="2" t="n">
-        <v>177.488</v>
+        <v>191.16</v>
       </c>
       <c r="D41" s="2" t="n"/>
       <c r="E41" s="2" t="n"/>
@@ -6256,10 +6256,10 @@
         </is>
       </c>
       <c r="B42" s="2" t="n">
-        <v>-356.796</v>
+        <v>-319.526</v>
       </c>
       <c r="C42" s="2" t="n">
-        <v>168.488</v>
+        <v>182.16</v>
       </c>
       <c r="D42" s="2" t="n"/>
       <c r="E42" s="2" t="n"/>
@@ -6273,10 +6273,10 @@
         </is>
       </c>
       <c r="B43" s="2" t="n">
-        <v>-356.796</v>
+        <v>-319.526</v>
       </c>
       <c r="C43" s="2" t="n">
-        <v>159.488</v>
+        <v>173.16</v>
       </c>
       <c r="D43" s="2" t="n"/>
       <c r="E43" s="2" t="n"/>
@@ -6290,10 +6290,10 @@
         </is>
       </c>
       <c r="B44" s="2" t="n">
-        <v>-356.796</v>
+        <v>-319.526</v>
       </c>
       <c r="C44" s="2" t="n">
-        <v>150.488</v>
+        <v>164.16</v>
       </c>
       <c r="D44" s="2" t="n"/>
       <c r="E44" s="2" t="n"/>
@@ -6307,10 +6307,10 @@
         </is>
       </c>
       <c r="B45" s="2" t="n">
-        <v>-356.796</v>
+        <v>-319.526</v>
       </c>
       <c r="C45" s="2" t="n">
-        <v>141.488</v>
+        <v>155.16</v>
       </c>
       <c r="D45" s="2" t="n"/>
       <c r="E45" s="2" t="n"/>
@@ -6324,10 +6324,10 @@
         </is>
       </c>
       <c r="B46" s="2" t="n">
-        <v>-356.796</v>
+        <v>-319.526</v>
       </c>
       <c r="C46" s="2" t="n">
-        <v>132.488</v>
+        <v>146.16</v>
       </c>
       <c r="D46" s="2" t="n"/>
       <c r="E46" s="2" t="n"/>
@@ -6341,10 +6341,10 @@
         </is>
       </c>
       <c r="B47" s="2" t="n">
-        <v>-356.796</v>
+        <v>-319.526</v>
       </c>
       <c r="C47" s="2" t="n">
-        <v>123.488</v>
+        <v>137.16</v>
       </c>
       <c r="D47" s="2" t="n"/>
       <c r="E47" s="2" t="n"/>
@@ -6358,10 +6358,10 @@
         </is>
       </c>
       <c r="B48" s="2" t="n">
-        <v>-356.796</v>
+        <v>-319.526</v>
       </c>
       <c r="C48" s="2" t="n">
-        <v>114.488</v>
+        <v>128.16</v>
       </c>
       <c r="D48" s="2" t="n"/>
       <c r="E48" s="2" t="n"/>
@@ -6375,10 +6375,10 @@
         </is>
       </c>
       <c r="B49" s="2" t="n">
-        <v>-356.796</v>
+        <v>-319.526</v>
       </c>
       <c r="C49" s="2" t="n">
-        <v>105.488</v>
+        <v>119.16</v>
       </c>
       <c r="D49" s="2" t="n"/>
       <c r="E49" s="2" t="n"/>
@@ -6392,10 +6392,10 @@
         </is>
       </c>
       <c r="B50" s="2" t="n">
-        <v>-365.796</v>
+        <v>-328.526</v>
       </c>
       <c r="C50" s="2" t="n">
-        <v>204.488</v>
+        <v>218.16</v>
       </c>
       <c r="D50" s="2" t="n"/>
       <c r="E50" s="2" t="n"/>
@@ -6409,10 +6409,10 @@
         </is>
       </c>
       <c r="B51" s="2" t="n">
-        <v>-365.796</v>
+        <v>-328.526</v>
       </c>
       <c r="C51" s="2" t="n">
-        <v>195.488</v>
+        <v>209.16</v>
       </c>
       <c r="D51" s="2" t="n"/>
       <c r="E51" s="2" t="n"/>
@@ -6426,10 +6426,10 @@
         </is>
       </c>
       <c r="B52" s="2" t="n">
-        <v>-365.796</v>
+        <v>-328.526</v>
       </c>
       <c r="C52" s="2" t="n">
-        <v>186.488</v>
+        <v>200.16</v>
       </c>
       <c r="D52" s="2" t="n"/>
       <c r="E52" s="2" t="n"/>
@@ -6443,10 +6443,10 @@
         </is>
       </c>
       <c r="B53" s="2" t="n">
-        <v>-365.796</v>
+        <v>-328.526</v>
       </c>
       <c r="C53" s="2" t="n">
-        <v>177.488</v>
+        <v>191.16</v>
       </c>
       <c r="D53" s="2" t="n"/>
       <c r="E53" s="2" t="n"/>
@@ -6460,10 +6460,10 @@
         </is>
       </c>
       <c r="B54" s="2" t="n">
-        <v>-365.796</v>
+        <v>-328.526</v>
       </c>
       <c r="C54" s="2" t="n">
-        <v>168.488</v>
+        <v>182.16</v>
       </c>
       <c r="D54" s="2" t="n"/>
       <c r="E54" s="2" t="n"/>
@@ -6477,10 +6477,10 @@
         </is>
       </c>
       <c r="B55" s="2" t="n">
-        <v>-365.796</v>
+        <v>-328.526</v>
       </c>
       <c r="C55" s="2" t="n">
-        <v>159.488</v>
+        <v>173.16</v>
       </c>
       <c r="D55" s="2" t="n"/>
       <c r="E55" s="2" t="n"/>
@@ -6494,10 +6494,10 @@
         </is>
       </c>
       <c r="B56" s="2" t="n">
-        <v>-365.796</v>
+        <v>-328.526</v>
       </c>
       <c r="C56" s="2" t="n">
-        <v>150.488</v>
+        <v>164.16</v>
       </c>
       <c r="D56" s="2" t="n"/>
       <c r="E56" s="2" t="n"/>
@@ -6511,10 +6511,10 @@
         </is>
       </c>
       <c r="B57" s="2" t="n">
-        <v>-365.796</v>
+        <v>-328.526</v>
       </c>
       <c r="C57" s="2" t="n">
-        <v>141.488</v>
+        <v>155.16</v>
       </c>
       <c r="D57" s="2" t="n"/>
       <c r="E57" s="2" t="n"/>
@@ -6528,10 +6528,10 @@
         </is>
       </c>
       <c r="B58" s="2" t="n">
-        <v>-365.796</v>
+        <v>-328.526</v>
       </c>
       <c r="C58" s="2" t="n">
-        <v>132.488</v>
+        <v>146.16</v>
       </c>
       <c r="D58" s="2" t="n"/>
       <c r="E58" s="2" t="n"/>
@@ -6545,10 +6545,10 @@
         </is>
       </c>
       <c r="B59" s="2" t="n">
-        <v>-365.796</v>
+        <v>-328.526</v>
       </c>
       <c r="C59" s="2" t="n">
-        <v>123.488</v>
+        <v>137.16</v>
       </c>
       <c r="D59" s="2" t="n"/>
       <c r="E59" s="2" t="n"/>
@@ -6562,10 +6562,10 @@
         </is>
       </c>
       <c r="B60" s="2" t="n">
-        <v>-365.796</v>
+        <v>-328.526</v>
       </c>
       <c r="C60" s="2" t="n">
-        <v>114.488</v>
+        <v>128.16</v>
       </c>
       <c r="D60" s="2" t="n"/>
       <c r="E60" s="2" t="n"/>
@@ -6579,10 +6579,10 @@
         </is>
       </c>
       <c r="B61" s="2" t="n">
-        <v>-365.796</v>
+        <v>-328.526</v>
       </c>
       <c r="C61" s="2" t="n">
-        <v>105.488</v>
+        <v>119.16</v>
       </c>
       <c r="D61" s="2" t="n"/>
       <c r="E61" s="2" t="n"/>
@@ -6596,10 +6596,10 @@
         </is>
       </c>
       <c r="B62" s="2" t="n">
-        <v>-374.796</v>
+        <v>-337.526</v>
       </c>
       <c r="C62" s="2" t="n">
-        <v>204.488</v>
+        <v>218.16</v>
       </c>
       <c r="D62" s="2" t="n"/>
       <c r="E62" s="2" t="n"/>
@@ -6613,10 +6613,10 @@
         </is>
       </c>
       <c r="B63" s="2" t="n">
-        <v>-374.796</v>
+        <v>-337.526</v>
       </c>
       <c r="C63" s="2" t="n">
-        <v>195.488</v>
+        <v>209.16</v>
       </c>
       <c r="D63" s="2" t="n"/>
       <c r="E63" s="2" t="n"/>
@@ -6630,10 +6630,10 @@
         </is>
       </c>
       <c r="B64" s="2" t="n">
-        <v>-374.796</v>
+        <v>-337.526</v>
       </c>
       <c r="C64" s="2" t="n">
-        <v>186.488</v>
+        <v>200.16</v>
       </c>
       <c r="D64" s="2" t="n"/>
       <c r="E64" s="2" t="n"/>
@@ -6647,10 +6647,10 @@
         </is>
       </c>
       <c r="B65" s="2" t="n">
-        <v>-374.796</v>
+        <v>-337.526</v>
       </c>
       <c r="C65" s="2" t="n">
-        <v>177.488</v>
+        <v>191.16</v>
       </c>
       <c r="D65" s="2" t="n"/>
       <c r="E65" s="2" t="n"/>
@@ -6664,10 +6664,10 @@
         </is>
       </c>
       <c r="B66" s="2" t="n">
-        <v>-374.796</v>
+        <v>-337.526</v>
       </c>
       <c r="C66" s="2" t="n">
-        <v>168.488</v>
+        <v>182.16</v>
       </c>
       <c r="D66" s="2" t="n"/>
       <c r="E66" s="2" t="n"/>
@@ -6681,10 +6681,10 @@
         </is>
       </c>
       <c r="B67" s="2" t="n">
-        <v>-374.796</v>
+        <v>-337.526</v>
       </c>
       <c r="C67" s="2" t="n">
-        <v>159.488</v>
+        <v>173.16</v>
       </c>
       <c r="D67" s="2" t="n"/>
       <c r="E67" s="2" t="n"/>
@@ -6698,10 +6698,10 @@
         </is>
       </c>
       <c r="B68" s="2" t="n">
-        <v>-374.796</v>
+        <v>-337.526</v>
       </c>
       <c r="C68" s="2" t="n">
-        <v>150.488</v>
+        <v>164.16</v>
       </c>
       <c r="D68" s="2" t="n"/>
       <c r="E68" s="2" t="n"/>
@@ -6715,10 +6715,10 @@
         </is>
       </c>
       <c r="B69" s="2" t="n">
-        <v>-374.796</v>
+        <v>-337.526</v>
       </c>
       <c r="C69" s="2" t="n">
-        <v>141.488</v>
+        <v>155.16</v>
       </c>
       <c r="D69" s="2" t="n"/>
       <c r="E69" s="2" t="n"/>
@@ -6732,10 +6732,10 @@
         </is>
       </c>
       <c r="B70" s="2" t="n">
-        <v>-374.796</v>
+        <v>-337.526</v>
       </c>
       <c r="C70" s="2" t="n">
-        <v>132.488</v>
+        <v>146.16</v>
       </c>
       <c r="D70" s="2" t="n"/>
       <c r="E70" s="2" t="n"/>
@@ -6749,10 +6749,10 @@
         </is>
       </c>
       <c r="B71" s="2" t="n">
-        <v>-374.796</v>
+        <v>-337.526</v>
       </c>
       <c r="C71" s="2" t="n">
-        <v>123.488</v>
+        <v>137.16</v>
       </c>
       <c r="D71" s="2" t="n"/>
       <c r="E71" s="2" t="n"/>
@@ -6766,10 +6766,10 @@
         </is>
       </c>
       <c r="B72" s="2" t="n">
-        <v>-374.796</v>
+        <v>-337.526</v>
       </c>
       <c r="C72" s="2" t="n">
-        <v>114.488</v>
+        <v>128.16</v>
       </c>
       <c r="D72" s="2" t="n"/>
       <c r="E72" s="2" t="n"/>
@@ -6783,10 +6783,10 @@
         </is>
       </c>
       <c r="B73" s="2" t="n">
-        <v>-374.796</v>
+        <v>-337.526</v>
       </c>
       <c r="C73" s="2" t="n">
-        <v>105.488</v>
+        <v>119.16</v>
       </c>
       <c r="D73" s="2" t="n"/>
       <c r="E73" s="2" t="n"/>
@@ -6800,10 +6800,10 @@
         </is>
       </c>
       <c r="B74" s="2" t="n">
-        <v>-383.796</v>
+        <v>-346.526</v>
       </c>
       <c r="C74" s="2" t="n">
-        <v>204.488</v>
+        <v>218.16</v>
       </c>
       <c r="D74" s="2" t="n"/>
       <c r="E74" s="2" t="n"/>
@@ -6817,10 +6817,10 @@
         </is>
       </c>
       <c r="B75" s="2" t="n">
-        <v>-383.796</v>
+        <v>-346.526</v>
       </c>
       <c r="C75" s="2" t="n">
-        <v>195.488</v>
+        <v>209.16</v>
       </c>
       <c r="D75" s="2" t="n"/>
       <c r="E75" s="2" t="n"/>
@@ -6834,10 +6834,10 @@
         </is>
       </c>
       <c r="B76" s="2" t="n">
-        <v>-383.796</v>
+        <v>-346.526</v>
       </c>
       <c r="C76" s="2" t="n">
-        <v>186.488</v>
+        <v>200.16</v>
       </c>
       <c r="D76" s="2" t="n"/>
       <c r="E76" s="2" t="n"/>
@@ -6851,10 +6851,10 @@
         </is>
       </c>
       <c r="B77" s="2" t="n">
-        <v>-383.796</v>
+        <v>-346.526</v>
       </c>
       <c r="C77" s="2" t="n">
-        <v>177.488</v>
+        <v>191.16</v>
       </c>
       <c r="D77" s="2" t="n"/>
       <c r="E77" s="2" t="n"/>
@@ -6868,10 +6868,10 @@
         </is>
       </c>
       <c r="B78" s="2" t="n">
-        <v>-383.796</v>
+        <v>-346.526</v>
       </c>
       <c r="C78" s="2" t="n">
-        <v>168.488</v>
+        <v>182.16</v>
       </c>
       <c r="D78" s="2" t="n"/>
       <c r="E78" s="2" t="n"/>
@@ -6885,10 +6885,10 @@
         </is>
       </c>
       <c r="B79" s="2" t="n">
-        <v>-383.796</v>
+        <v>-346.526</v>
       </c>
       <c r="C79" s="2" t="n">
-        <v>159.488</v>
+        <v>173.16</v>
       </c>
       <c r="D79" s="2" t="n"/>
       <c r="E79" s="2" t="n"/>
@@ -6902,10 +6902,10 @@
         </is>
       </c>
       <c r="B80" s="2" t="n">
-        <v>-383.796</v>
+        <v>-346.526</v>
       </c>
       <c r="C80" s="2" t="n">
-        <v>150.488</v>
+        <v>164.16</v>
       </c>
       <c r="D80" s="2" t="n"/>
       <c r="E80" s="2" t="n"/>
@@ -6919,10 +6919,10 @@
         </is>
       </c>
       <c r="B81" s="2" t="n">
-        <v>-383.796</v>
+        <v>-346.526</v>
       </c>
       <c r="C81" s="2" t="n">
-        <v>141.488</v>
+        <v>155.16</v>
       </c>
       <c r="D81" s="2" t="n"/>
       <c r="E81" s="2" t="n"/>
@@ -6936,10 +6936,10 @@
         </is>
       </c>
       <c r="B82" s="2" t="n">
-        <v>-383.796</v>
+        <v>-346.526</v>
       </c>
       <c r="C82" s="2" t="n">
-        <v>132.488</v>
+        <v>146.16</v>
       </c>
       <c r="D82" s="2" t="n"/>
       <c r="E82" s="2" t="n"/>
@@ -6953,10 +6953,10 @@
         </is>
       </c>
       <c r="B83" s="2" t="n">
-        <v>-383.796</v>
+        <v>-346.526</v>
       </c>
       <c r="C83" s="2" t="n">
-        <v>123.488</v>
+        <v>137.16</v>
       </c>
       <c r="D83" s="2" t="n"/>
       <c r="E83" s="2" t="n"/>
@@ -6970,10 +6970,10 @@
         </is>
       </c>
       <c r="B84" s="2" t="n">
-        <v>-383.796</v>
+        <v>-346.526</v>
       </c>
       <c r="C84" s="2" t="n">
-        <v>114.488</v>
+        <v>128.16</v>
       </c>
       <c r="D84" s="2" t="n"/>
       <c r="E84" s="2" t="n"/>
@@ -6987,10 +6987,10 @@
         </is>
       </c>
       <c r="B85" s="2" t="n">
-        <v>-383.796</v>
+        <v>-346.526</v>
       </c>
       <c r="C85" s="2" t="n">
-        <v>105.488</v>
+        <v>119.16</v>
       </c>
       <c r="D85" s="2" t="n"/>
       <c r="E85" s="2" t="n"/>
@@ -7004,10 +7004,10 @@
         </is>
       </c>
       <c r="B86" s="2" t="n">
-        <v>-392.796</v>
+        <v>-355.526</v>
       </c>
       <c r="C86" s="2" t="n">
-        <v>204.488</v>
+        <v>218.16</v>
       </c>
       <c r="D86" s="2" t="n"/>
       <c r="E86" s="2" t="n"/>
@@ -7021,10 +7021,10 @@
         </is>
       </c>
       <c r="B87" s="2" t="n">
-        <v>-392.796</v>
+        <v>-355.526</v>
       </c>
       <c r="C87" s="2" t="n">
-        <v>195.488</v>
+        <v>209.16</v>
       </c>
       <c r="D87" s="2" t="n"/>
       <c r="E87" s="2" t="n"/>
@@ -7038,10 +7038,10 @@
         </is>
       </c>
       <c r="B88" s="2" t="n">
-        <v>-392.796</v>
+        <v>-355.526</v>
       </c>
       <c r="C88" s="2" t="n">
-        <v>186.488</v>
+        <v>200.16</v>
       </c>
       <c r="D88" s="2" t="n"/>
       <c r="E88" s="2" t="n"/>
@@ -7055,10 +7055,10 @@
         </is>
       </c>
       <c r="B89" s="2" t="n">
-        <v>-392.796</v>
+        <v>-355.526</v>
       </c>
       <c r="C89" s="2" t="n">
-        <v>177.488</v>
+        <v>191.16</v>
       </c>
       <c r="D89" s="2" t="n"/>
       <c r="E89" s="2" t="n"/>
@@ -7072,10 +7072,10 @@
         </is>
       </c>
       <c r="B90" s="2" t="n">
-        <v>-392.796</v>
+        <v>-355.526</v>
       </c>
       <c r="C90" s="2" t="n">
-        <v>168.488</v>
+        <v>182.16</v>
       </c>
       <c r="D90" s="2" t="n"/>
       <c r="E90" s="2" t="n"/>
@@ -7089,10 +7089,10 @@
         </is>
       </c>
       <c r="B91" s="2" t="n">
-        <v>-392.796</v>
+        <v>-355.526</v>
       </c>
       <c r="C91" s="2" t="n">
-        <v>159.488</v>
+        <v>173.16</v>
       </c>
       <c r="D91" s="2" t="n"/>
       <c r="E91" s="2" t="n"/>
@@ -7106,10 +7106,10 @@
         </is>
       </c>
       <c r="B92" s="2" t="n">
-        <v>-392.796</v>
+        <v>-355.526</v>
       </c>
       <c r="C92" s="2" t="n">
-        <v>150.488</v>
+        <v>164.16</v>
       </c>
       <c r="D92" s="2" t="n"/>
       <c r="E92" s="2" t="n"/>
@@ -7123,10 +7123,10 @@
         </is>
       </c>
       <c r="B93" s="2" t="n">
-        <v>-392.796</v>
+        <v>-355.526</v>
       </c>
       <c r="C93" s="2" t="n">
-        <v>141.488</v>
+        <v>155.16</v>
       </c>
       <c r="D93" s="2" t="n"/>
       <c r="E93" s="2" t="n"/>
@@ -7140,10 +7140,10 @@
         </is>
       </c>
       <c r="B94" s="2" t="n">
-        <v>-392.796</v>
+        <v>-355.526</v>
       </c>
       <c r="C94" s="2" t="n">
-        <v>132.488</v>
+        <v>146.16</v>
       </c>
       <c r="D94" s="2" t="n"/>
       <c r="E94" s="2" t="n"/>
@@ -7157,10 +7157,10 @@
         </is>
       </c>
       <c r="B95" s="2" t="n">
-        <v>-392.796</v>
+        <v>-355.526</v>
       </c>
       <c r="C95" s="2" t="n">
-        <v>123.488</v>
+        <v>137.16</v>
       </c>
       <c r="D95" s="2" t="n"/>
       <c r="E95" s="2" t="n"/>
@@ -7174,10 +7174,10 @@
         </is>
       </c>
       <c r="B96" s="2" t="n">
-        <v>-392.796</v>
+        <v>-355.526</v>
       </c>
       <c r="C96" s="2" t="n">
-        <v>114.488</v>
+        <v>128.16</v>
       </c>
       <c r="D96" s="2" t="n"/>
       <c r="E96" s="2" t="n"/>
@@ -7191,10 +7191,10 @@
         </is>
       </c>
       <c r="B97" s="2" t="n">
-        <v>-392.796</v>
+        <v>-355.526</v>
       </c>
       <c r="C97" s="2" t="n">
-        <v>105.488</v>
+        <v>119.16</v>
       </c>
       <c r="D97" s="2" t="n"/>
       <c r="E97" s="2" t="n"/>
@@ -7204,4 +7204,283 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100DF72643B013E014A825B49D64A1110FC" ma:contentTypeVersion="17" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="f45f840bb0a575e0982080148504d801">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="898ec965-d5a3-48b2-9d91-8cd3ed319c77" xmlns:ns3="34a6835a-a421-4fc1-9891-838ec1df6c1f" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="1578e7a6edb9656aff92510688ad8ae5" ns2:_="" ns3:_="">
+    <xsd:import namespace="898ec965-d5a3-48b2-9d91-8cd3ed319c77"/>
+    <xsd:import namespace="34a6835a-a421-4fc1-9891-838ec1df6c1f"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceAutoTags" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
+                <xsd:element ref="ns3:SharedWithUsers" minOccurs="0"/>
+                <xsd:element ref="ns3:SharedWithDetails" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceBillingMetadata" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="898ec965-d5a3-48b2-9d91-8cd3ed319c77" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceAutoTags" ma:index="10" nillable="true" ma:displayName="MediaServiceAutoTags" ma:internalName="MediaServiceAutoTags" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="11" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="12" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="14" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="d3514cfa-118c-47c7-8064-f16f79621ace" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="16" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="17" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="18" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceLocation" ma:index="19" nillable="true" ma:displayName="Location" ma:indexed="true" ma:internalName="MediaServiceLocation" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="20" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="23" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceBillingMetadata" ma:index="24" nillable="true" ma:displayName="MediaServiceBillingMetadata" ma:hidden="true" ma:internalName="MediaServiceBillingMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="34a6835a-a421-4fc1-9891-838ec1df6c1f" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="15" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{fdb65f81-2f44-4049-bc2f-903088f674cc}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="34a6835a-a421-4fc1-9891-838ec1df6c1f">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="SharedWithUsers" ma:index="21" nillable="true" ma:displayName="Shared With" ma:internalName="SharedWithUsers" ma:readOnly="true">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:UserMulti">
+            <xsd:sequence>
+              <xsd:element name="UserInfo" minOccurs="0" maxOccurs="unbounded">
+                <xsd:complexType>
+                  <xsd:sequence>
+                    <xsd:element name="DisplayName" type="xsd:string" minOccurs="0"/>
+                    <xsd:element name="AccountId" type="dms:UserId" minOccurs="0" nillable="true"/>
+                    <xsd:element name="AccountType" type="xsd:string" minOccurs="0"/>
+                  </xsd:sequence>
+                </xsd:complexType>
+              </xsd:element>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="SharedWithDetails" ma:index="22" nillable="true" ma:displayName="Shared With Details" ma:internalName="SharedWithDetails" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="898ec965-d5a3-48b2-9d91-8cd3ed319c77">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="34a6835a-a421-4fc1-9891-838ec1df6c1f" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CC7667ED-6274-4B86-8AC0-0A173BF4DD60}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2345460B-A773-4EEA-9FEB-D937D6B138D1}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2704089A-2B5C-43B2-9D1E-A5B823B06348}"/>
 </file>
</xml_diff>

<commit_message>
fix(config): plate 2 Y offset -2mm -> -1mm net from original
-2mm overshot -- pipette started hitting the opposite side of the
well. Added +1mm back to the already-shifted values, netting -1mm
from the original coordinates instead of -2mm.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/config/plate_configs/plate_stations.xlsx
+++ b/config/plate_configs/plate_stations.xlsx
@@ -2194,7 +2194,7 @@
         <v>288.836</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>219.674</v>
+        <v>220.674</v>
       </c>
       <c r="D2" s="2" t="n"/>
       <c r="E2" s="2" t="n"/>
@@ -2211,7 +2211,7 @@
         <v>288.836</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>210.674</v>
+        <v>211.674</v>
       </c>
       <c r="D3" s="2" t="n"/>
       <c r="E3" s="2" t="n"/>
@@ -2228,7 +2228,7 @@
         <v>288.836</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>201.674</v>
+        <v>202.674</v>
       </c>
       <c r="D4" s="2" t="n"/>
       <c r="E4" s="2" t="n"/>
@@ -2245,7 +2245,7 @@
         <v>288.836</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>192.674</v>
+        <v>193.674</v>
       </c>
       <c r="D5" s="2" t="n"/>
       <c r="E5" s="2" t="n"/>
@@ -2262,7 +2262,7 @@
         <v>288.836</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>183.674</v>
+        <v>184.674</v>
       </c>
       <c r="D6" s="2" t="n"/>
       <c r="E6" s="2" t="n"/>
@@ -2279,7 +2279,7 @@
         <v>288.836</v>
       </c>
       <c r="C7" s="2" t="n">
-        <v>174.674</v>
+        <v>175.674</v>
       </c>
       <c r="D7" s="2" t="n"/>
       <c r="E7" s="2" t="n"/>
@@ -2296,7 +2296,7 @@
         <v>288.836</v>
       </c>
       <c r="C8" s="2" t="n">
-        <v>165.674</v>
+        <v>166.674</v>
       </c>
       <c r="D8" s="2" t="n"/>
       <c r="E8" s="2" t="n"/>
@@ -2313,7 +2313,7 @@
         <v>288.836</v>
       </c>
       <c r="C9" s="2" t="n">
-        <v>156.674</v>
+        <v>157.674</v>
       </c>
       <c r="D9" s="2" t="n"/>
       <c r="E9" s="2" t="n"/>
@@ -2330,7 +2330,7 @@
         <v>288.836</v>
       </c>
       <c r="C10" s="2" t="n">
-        <v>147.674</v>
+        <v>148.674</v>
       </c>
       <c r="D10" s="2" t="n"/>
       <c r="E10" s="2" t="n"/>
@@ -2347,7 +2347,7 @@
         <v>288.836</v>
       </c>
       <c r="C11" s="2" t="n">
-        <v>138.674</v>
+        <v>139.674</v>
       </c>
       <c r="D11" s="2" t="n"/>
       <c r="E11" s="2" t="n"/>
@@ -2364,7 +2364,7 @@
         <v>288.836</v>
       </c>
       <c r="C12" s="2" t="n">
-        <v>129.674</v>
+        <v>130.674</v>
       </c>
       <c r="D12" s="2" t="n"/>
       <c r="E12" s="2" t="n"/>
@@ -2381,7 +2381,7 @@
         <v>288.836</v>
       </c>
       <c r="C13" s="2" t="n">
-        <v>120.674</v>
+        <v>121.674</v>
       </c>
       <c r="D13" s="2" t="n"/>
       <c r="E13" s="2" t="n"/>
@@ -2398,7 +2398,7 @@
         <v>297.836</v>
       </c>
       <c r="C14" s="2" t="n">
-        <v>219.674</v>
+        <v>220.674</v>
       </c>
       <c r="D14" s="2" t="n"/>
       <c r="E14" s="2" t="n"/>
@@ -2415,7 +2415,7 @@
         <v>297.836</v>
       </c>
       <c r="C15" s="2" t="n">
-        <v>210.674</v>
+        <v>211.674</v>
       </c>
       <c r="D15" s="2" t="n"/>
       <c r="E15" s="2" t="n"/>
@@ -2432,7 +2432,7 @@
         <v>297.836</v>
       </c>
       <c r="C16" s="2" t="n">
-        <v>201.674</v>
+        <v>202.674</v>
       </c>
       <c r="D16" s="2" t="n"/>
       <c r="E16" s="2" t="n"/>
@@ -2449,7 +2449,7 @@
         <v>297.836</v>
       </c>
       <c r="C17" s="2" t="n">
-        <v>192.674</v>
+        <v>193.674</v>
       </c>
       <c r="D17" s="2" t="n"/>
       <c r="E17" s="2" t="n"/>
@@ -2466,7 +2466,7 @@
         <v>297.836</v>
       </c>
       <c r="C18" s="2" t="n">
-        <v>183.674</v>
+        <v>184.674</v>
       </c>
       <c r="D18" s="2" t="n"/>
       <c r="E18" s="2" t="n"/>
@@ -2483,7 +2483,7 @@
         <v>297.836</v>
       </c>
       <c r="C19" s="2" t="n">
-        <v>174.674</v>
+        <v>175.674</v>
       </c>
       <c r="D19" s="2" t="n"/>
       <c r="E19" s="2" t="n"/>
@@ -2500,7 +2500,7 @@
         <v>297.836</v>
       </c>
       <c r="C20" s="2" t="n">
-        <v>165.674</v>
+        <v>166.674</v>
       </c>
       <c r="D20" s="2" t="n"/>
       <c r="E20" s="2" t="n"/>
@@ -2517,7 +2517,7 @@
         <v>297.836</v>
       </c>
       <c r="C21" s="2" t="n">
-        <v>156.674</v>
+        <v>157.674</v>
       </c>
       <c r="D21" s="2" t="n"/>
       <c r="E21" s="2" t="n"/>
@@ -2534,7 +2534,7 @@
         <v>297.836</v>
       </c>
       <c r="C22" s="2" t="n">
-        <v>147.674</v>
+        <v>148.674</v>
       </c>
       <c r="D22" s="2" t="n"/>
       <c r="E22" s="2" t="n"/>
@@ -2551,7 +2551,7 @@
         <v>297.836</v>
       </c>
       <c r="C23" s="2" t="n">
-        <v>138.674</v>
+        <v>139.674</v>
       </c>
       <c r="D23" s="2" t="n"/>
       <c r="E23" s="2" t="n"/>
@@ -2568,7 +2568,7 @@
         <v>297.836</v>
       </c>
       <c r="C24" s="2" t="n">
-        <v>129.674</v>
+        <v>130.674</v>
       </c>
       <c r="D24" s="2" t="n"/>
       <c r="E24" s="2" t="n"/>
@@ -2585,7 +2585,7 @@
         <v>297.836</v>
       </c>
       <c r="C25" s="2" t="n">
-        <v>120.674</v>
+        <v>121.674</v>
       </c>
       <c r="D25" s="2" t="n"/>
       <c r="E25" s="2" t="n"/>
@@ -2602,7 +2602,7 @@
         <v>306.836</v>
       </c>
       <c r="C26" s="2" t="n">
-        <v>219.674</v>
+        <v>220.674</v>
       </c>
       <c r="D26" s="2" t="n"/>
       <c r="E26" s="2" t="n"/>
@@ -2619,7 +2619,7 @@
         <v>306.836</v>
       </c>
       <c r="C27" s="2" t="n">
-        <v>210.674</v>
+        <v>211.674</v>
       </c>
       <c r="D27" s="2" t="n"/>
       <c r="E27" s="2" t="n"/>
@@ -2636,7 +2636,7 @@
         <v>306.836</v>
       </c>
       <c r="C28" s="2" t="n">
-        <v>201.674</v>
+        <v>202.674</v>
       </c>
       <c r="D28" s="2" t="n"/>
       <c r="E28" s="2" t="n"/>
@@ -2653,7 +2653,7 @@
         <v>306.836</v>
       </c>
       <c r="C29" s="2" t="n">
-        <v>192.674</v>
+        <v>193.674</v>
       </c>
       <c r="D29" s="2" t="n"/>
       <c r="E29" s="2" t="n"/>
@@ -2670,7 +2670,7 @@
         <v>306.836</v>
       </c>
       <c r="C30" s="2" t="n">
-        <v>183.674</v>
+        <v>184.674</v>
       </c>
       <c r="D30" s="2" t="n"/>
       <c r="E30" s="2" t="n"/>
@@ -2687,7 +2687,7 @@
         <v>306.836</v>
       </c>
       <c r="C31" s="2" t="n">
-        <v>174.674</v>
+        <v>175.674</v>
       </c>
       <c r="D31" s="2" t="n"/>
       <c r="E31" s="2" t="n"/>
@@ -2704,7 +2704,7 @@
         <v>306.836</v>
       </c>
       <c r="C32" s="2" t="n">
-        <v>165.674</v>
+        <v>166.674</v>
       </c>
       <c r="D32" s="2" t="n"/>
       <c r="E32" s="2" t="n"/>
@@ -2721,7 +2721,7 @@
         <v>306.836</v>
       </c>
       <c r="C33" s="2" t="n">
-        <v>156.674</v>
+        <v>157.674</v>
       </c>
       <c r="D33" s="2" t="n"/>
       <c r="E33" s="2" t="n"/>
@@ -2738,7 +2738,7 @@
         <v>306.836</v>
       </c>
       <c r="C34" s="2" t="n">
-        <v>147.674</v>
+        <v>148.674</v>
       </c>
       <c r="D34" s="2" t="n"/>
       <c r="E34" s="2" t="n"/>
@@ -2755,7 +2755,7 @@
         <v>306.836</v>
       </c>
       <c r="C35" s="2" t="n">
-        <v>138.674</v>
+        <v>139.674</v>
       </c>
       <c r="D35" s="2" t="n"/>
       <c r="E35" s="2" t="n"/>
@@ -2772,7 +2772,7 @@
         <v>306.836</v>
       </c>
       <c r="C36" s="2" t="n">
-        <v>129.674</v>
+        <v>130.674</v>
       </c>
       <c r="D36" s="2" t="n"/>
       <c r="E36" s="2" t="n"/>
@@ -2789,7 +2789,7 @@
         <v>306.836</v>
       </c>
       <c r="C37" s="2" t="n">
-        <v>120.674</v>
+        <v>121.674</v>
       </c>
       <c r="D37" s="2" t="n"/>
       <c r="E37" s="2" t="n"/>
@@ -2806,7 +2806,7 @@
         <v>315.836</v>
       </c>
       <c r="C38" s="2" t="n">
-        <v>219.674</v>
+        <v>220.674</v>
       </c>
       <c r="D38" s="2" t="n"/>
       <c r="E38" s="2" t="n"/>
@@ -2823,7 +2823,7 @@
         <v>315.836</v>
       </c>
       <c r="C39" s="2" t="n">
-        <v>210.674</v>
+        <v>211.674</v>
       </c>
       <c r="D39" s="2" t="n"/>
       <c r="E39" s="2" t="n"/>
@@ -2840,7 +2840,7 @@
         <v>315.836</v>
       </c>
       <c r="C40" s="2" t="n">
-        <v>201.674</v>
+        <v>202.674</v>
       </c>
       <c r="D40" s="2" t="n"/>
       <c r="E40" s="2" t="n"/>
@@ -2857,7 +2857,7 @@
         <v>315.836</v>
       </c>
       <c r="C41" s="2" t="n">
-        <v>192.674</v>
+        <v>193.674</v>
       </c>
       <c r="D41" s="2" t="n"/>
       <c r="E41" s="2" t="n"/>
@@ -2874,7 +2874,7 @@
         <v>315.836</v>
       </c>
       <c r="C42" s="2" t="n">
-        <v>183.674</v>
+        <v>184.674</v>
       </c>
       <c r="D42" s="2" t="n"/>
       <c r="E42" s="2" t="n"/>
@@ -2891,7 +2891,7 @@
         <v>315.836</v>
       </c>
       <c r="C43" s="2" t="n">
-        <v>174.674</v>
+        <v>175.674</v>
       </c>
       <c r="D43" s="2" t="n"/>
       <c r="E43" s="2" t="n"/>
@@ -2908,7 +2908,7 @@
         <v>315.836</v>
       </c>
       <c r="C44" s="2" t="n">
-        <v>165.674</v>
+        <v>166.674</v>
       </c>
       <c r="D44" s="2" t="n"/>
       <c r="E44" s="2" t="n"/>
@@ -2925,7 +2925,7 @@
         <v>315.836</v>
       </c>
       <c r="C45" s="2" t="n">
-        <v>156.674</v>
+        <v>157.674</v>
       </c>
       <c r="D45" s="2" t="n"/>
       <c r="E45" s="2" t="n"/>
@@ -2942,7 +2942,7 @@
         <v>315.836</v>
       </c>
       <c r="C46" s="2" t="n">
-        <v>147.674</v>
+        <v>148.674</v>
       </c>
       <c r="D46" s="2" t="n"/>
       <c r="E46" s="2" t="n"/>
@@ -2959,7 +2959,7 @@
         <v>315.836</v>
       </c>
       <c r="C47" s="2" t="n">
-        <v>138.674</v>
+        <v>139.674</v>
       </c>
       <c r="D47" s="2" t="n"/>
       <c r="E47" s="2" t="n"/>
@@ -2976,7 +2976,7 @@
         <v>315.836</v>
       </c>
       <c r="C48" s="2" t="n">
-        <v>129.674</v>
+        <v>130.674</v>
       </c>
       <c r="D48" s="2" t="n"/>
       <c r="E48" s="2" t="n"/>
@@ -2993,7 +2993,7 @@
         <v>315.836</v>
       </c>
       <c r="C49" s="2" t="n">
-        <v>120.674</v>
+        <v>121.674</v>
       </c>
       <c r="D49" s="2" t="n"/>
       <c r="E49" s="2" t="n"/>
@@ -3010,7 +3010,7 @@
         <v>324.836</v>
       </c>
       <c r="C50" s="2" t="n">
-        <v>219.674</v>
+        <v>220.674</v>
       </c>
       <c r="D50" s="2" t="n"/>
       <c r="E50" s="2" t="n"/>
@@ -3027,7 +3027,7 @@
         <v>324.836</v>
       </c>
       <c r="C51" s="2" t="n">
-        <v>210.674</v>
+        <v>211.674</v>
       </c>
       <c r="D51" s="2" t="n"/>
       <c r="E51" s="2" t="n"/>
@@ -3044,7 +3044,7 @@
         <v>324.836</v>
       </c>
       <c r="C52" s="2" t="n">
-        <v>201.674</v>
+        <v>202.674</v>
       </c>
       <c r="D52" s="2" t="n"/>
       <c r="E52" s="2" t="n"/>
@@ -3061,7 +3061,7 @@
         <v>324.836</v>
       </c>
       <c r="C53" s="2" t="n">
-        <v>192.674</v>
+        <v>193.674</v>
       </c>
       <c r="D53" s="2" t="n"/>
       <c r="E53" s="2" t="n"/>
@@ -3078,7 +3078,7 @@
         <v>324.836</v>
       </c>
       <c r="C54" s="2" t="n">
-        <v>183.674</v>
+        <v>184.674</v>
       </c>
       <c r="D54" s="2" t="n"/>
       <c r="E54" s="2" t="n"/>
@@ -3095,7 +3095,7 @@
         <v>324.836</v>
       </c>
       <c r="C55" s="2" t="n">
-        <v>174.674</v>
+        <v>175.674</v>
       </c>
       <c r="D55" s="2" t="n"/>
       <c r="E55" s="2" t="n"/>
@@ -3112,7 +3112,7 @@
         <v>324.836</v>
       </c>
       <c r="C56" s="2" t="n">
-        <v>165.674</v>
+        <v>166.674</v>
       </c>
       <c r="D56" s="2" t="n"/>
       <c r="E56" s="2" t="n"/>
@@ -3129,7 +3129,7 @@
         <v>324.836</v>
       </c>
       <c r="C57" s="2" t="n">
-        <v>156.674</v>
+        <v>157.674</v>
       </c>
       <c r="D57" s="2" t="n"/>
       <c r="E57" s="2" t="n"/>
@@ -3146,7 +3146,7 @@
         <v>324.836</v>
       </c>
       <c r="C58" s="2" t="n">
-        <v>147.674</v>
+        <v>148.674</v>
       </c>
       <c r="D58" s="2" t="n"/>
       <c r="E58" s="2" t="n"/>
@@ -3163,7 +3163,7 @@
         <v>324.836</v>
       </c>
       <c r="C59" s="2" t="n">
-        <v>138.674</v>
+        <v>139.674</v>
       </c>
       <c r="D59" s="2" t="n"/>
       <c r="E59" s="2" t="n"/>
@@ -3180,7 +3180,7 @@
         <v>324.836</v>
       </c>
       <c r="C60" s="2" t="n">
-        <v>129.674</v>
+        <v>130.674</v>
       </c>
       <c r="D60" s="2" t="n"/>
       <c r="E60" s="2" t="n"/>
@@ -3197,7 +3197,7 @@
         <v>324.836</v>
       </c>
       <c r="C61" s="2" t="n">
-        <v>120.674</v>
+        <v>121.674</v>
       </c>
       <c r="D61" s="2" t="n"/>
       <c r="E61" s="2" t="n"/>
@@ -3214,7 +3214,7 @@
         <v>333.836</v>
       </c>
       <c r="C62" s="2" t="n">
-        <v>219.674</v>
+        <v>220.674</v>
       </c>
       <c r="D62" s="2" t="n"/>
       <c r="E62" s="2" t="n"/>
@@ -3231,7 +3231,7 @@
         <v>333.836</v>
       </c>
       <c r="C63" s="2" t="n">
-        <v>210.674</v>
+        <v>211.674</v>
       </c>
       <c r="D63" s="2" t="n"/>
       <c r="E63" s="2" t="n"/>
@@ -3248,7 +3248,7 @@
         <v>333.836</v>
       </c>
       <c r="C64" s="2" t="n">
-        <v>201.674</v>
+        <v>202.674</v>
       </c>
       <c r="D64" s="2" t="n"/>
       <c r="E64" s="2" t="n"/>
@@ -3265,7 +3265,7 @@
         <v>333.836</v>
       </c>
       <c r="C65" s="2" t="n">
-        <v>192.674</v>
+        <v>193.674</v>
       </c>
       <c r="D65" s="2" t="n"/>
       <c r="E65" s="2" t="n"/>
@@ -3282,7 +3282,7 @@
         <v>333.836</v>
       </c>
       <c r="C66" s="2" t="n">
-        <v>183.674</v>
+        <v>184.674</v>
       </c>
       <c r="D66" s="2" t="n"/>
       <c r="E66" s="2" t="n"/>
@@ -3299,7 +3299,7 @@
         <v>333.836</v>
       </c>
       <c r="C67" s="2" t="n">
-        <v>174.674</v>
+        <v>175.674</v>
       </c>
       <c r="D67" s="2" t="n"/>
       <c r="E67" s="2" t="n"/>
@@ -3316,7 +3316,7 @@
         <v>333.836</v>
       </c>
       <c r="C68" s="2" t="n">
-        <v>165.674</v>
+        <v>166.674</v>
       </c>
       <c r="D68" s="2" t="n"/>
       <c r="E68" s="2" t="n"/>
@@ -3333,7 +3333,7 @@
         <v>333.836</v>
       </c>
       <c r="C69" s="2" t="n">
-        <v>156.674</v>
+        <v>157.674</v>
       </c>
       <c r="D69" s="2" t="n"/>
       <c r="E69" s="2" t="n"/>
@@ -3350,7 +3350,7 @@
         <v>333.836</v>
       </c>
       <c r="C70" s="2" t="n">
-        <v>147.674</v>
+        <v>148.674</v>
       </c>
       <c r="D70" s="2" t="n"/>
       <c r="E70" s="2" t="n"/>
@@ -3367,7 +3367,7 @@
         <v>333.836</v>
       </c>
       <c r="C71" s="2" t="n">
-        <v>138.674</v>
+        <v>139.674</v>
       </c>
       <c r="D71" s="2" t="n"/>
       <c r="E71" s="2" t="n"/>
@@ -3384,7 +3384,7 @@
         <v>333.836</v>
       </c>
       <c r="C72" s="2" t="n">
-        <v>129.674</v>
+        <v>130.674</v>
       </c>
       <c r="D72" s="2" t="n"/>
       <c r="E72" s="2" t="n"/>
@@ -3401,7 +3401,7 @@
         <v>333.836</v>
       </c>
       <c r="C73" s="2" t="n">
-        <v>120.674</v>
+        <v>121.674</v>
       </c>
       <c r="D73" s="2" t="n"/>
       <c r="E73" s="2" t="n"/>
@@ -3418,7 +3418,7 @@
         <v>342.836</v>
       </c>
       <c r="C74" s="2" t="n">
-        <v>219.674</v>
+        <v>220.674</v>
       </c>
       <c r="D74" s="2" t="n"/>
       <c r="E74" s="2" t="n"/>
@@ -3435,7 +3435,7 @@
         <v>342.836</v>
       </c>
       <c r="C75" s="2" t="n">
-        <v>210.674</v>
+        <v>211.674</v>
       </c>
       <c r="D75" s="2" t="n"/>
       <c r="E75" s="2" t="n"/>
@@ -3452,7 +3452,7 @@
         <v>342.836</v>
       </c>
       <c r="C76" s="2" t="n">
-        <v>201.674</v>
+        <v>202.674</v>
       </c>
       <c r="D76" s="2" t="n"/>
       <c r="E76" s="2" t="n"/>
@@ -3469,7 +3469,7 @@
         <v>342.836</v>
       </c>
       <c r="C77" s="2" t="n">
-        <v>192.674</v>
+        <v>193.674</v>
       </c>
       <c r="D77" s="2" t="n"/>
       <c r="E77" s="2" t="n"/>
@@ -3486,7 +3486,7 @@
         <v>342.836</v>
       </c>
       <c r="C78" s="2" t="n">
-        <v>183.674</v>
+        <v>184.674</v>
       </c>
       <c r="D78" s="2" t="n"/>
       <c r="E78" s="2" t="n"/>
@@ -3503,7 +3503,7 @@
         <v>342.836</v>
       </c>
       <c r="C79" s="2" t="n">
-        <v>174.674</v>
+        <v>175.674</v>
       </c>
       <c r="D79" s="2" t="n"/>
       <c r="E79" s="2" t="n"/>
@@ -3520,7 +3520,7 @@
         <v>342.836</v>
       </c>
       <c r="C80" s="2" t="n">
-        <v>165.674</v>
+        <v>166.674</v>
       </c>
       <c r="D80" s="2" t="n"/>
       <c r="E80" s="2" t="n"/>
@@ -3537,7 +3537,7 @@
         <v>342.836</v>
       </c>
       <c r="C81" s="2" t="n">
-        <v>156.674</v>
+        <v>157.674</v>
       </c>
       <c r="D81" s="2" t="n"/>
       <c r="E81" s="2" t="n"/>
@@ -3554,7 +3554,7 @@
         <v>342.836</v>
       </c>
       <c r="C82" s="2" t="n">
-        <v>147.674</v>
+        <v>148.674</v>
       </c>
       <c r="D82" s="2" t="n"/>
       <c r="E82" s="2" t="n"/>
@@ -3571,7 +3571,7 @@
         <v>342.836</v>
       </c>
       <c r="C83" s="2" t="n">
-        <v>138.674</v>
+        <v>139.674</v>
       </c>
       <c r="D83" s="2" t="n"/>
       <c r="E83" s="2" t="n"/>
@@ -3588,7 +3588,7 @@
         <v>342.836</v>
       </c>
       <c r="C84" s="2" t="n">
-        <v>129.674</v>
+        <v>130.674</v>
       </c>
       <c r="D84" s="2" t="n"/>
       <c r="E84" s="2" t="n"/>
@@ -3605,7 +3605,7 @@
         <v>342.836</v>
       </c>
       <c r="C85" s="2" t="n">
-        <v>120.674</v>
+        <v>121.674</v>
       </c>
       <c r="D85" s="2" t="n"/>
       <c r="E85" s="2" t="n"/>
@@ -3622,7 +3622,7 @@
         <v>351.836</v>
       </c>
       <c r="C86" s="2" t="n">
-        <v>219.674</v>
+        <v>220.674</v>
       </c>
       <c r="D86" s="2" t="n"/>
       <c r="E86" s="2" t="n"/>
@@ -3639,7 +3639,7 @@
         <v>351.836</v>
       </c>
       <c r="C87" s="2" t="n">
-        <v>210.674</v>
+        <v>211.674</v>
       </c>
       <c r="D87" s="2" t="n"/>
       <c r="E87" s="2" t="n"/>
@@ -3656,7 +3656,7 @@
         <v>351.836</v>
       </c>
       <c r="C88" s="2" t="n">
-        <v>201.674</v>
+        <v>202.674</v>
       </c>
       <c r="D88" s="2" t="n"/>
       <c r="E88" s="2" t="n"/>
@@ -3673,7 +3673,7 @@
         <v>351.836</v>
       </c>
       <c r="C89" s="2" t="n">
-        <v>192.674</v>
+        <v>193.674</v>
       </c>
       <c r="D89" s="2" t="n"/>
       <c r="E89" s="2" t="n"/>
@@ -3690,7 +3690,7 @@
         <v>351.836</v>
       </c>
       <c r="C90" s="2" t="n">
-        <v>183.674</v>
+        <v>184.674</v>
       </c>
       <c r="D90" s="2" t="n"/>
       <c r="E90" s="2" t="n"/>
@@ -3707,7 +3707,7 @@
         <v>351.836</v>
       </c>
       <c r="C91" s="2" t="n">
-        <v>174.674</v>
+        <v>175.674</v>
       </c>
       <c r="D91" s="2" t="n"/>
       <c r="E91" s="2" t="n"/>
@@ -3724,7 +3724,7 @@
         <v>351.836</v>
       </c>
       <c r="C92" s="2" t="n">
-        <v>165.674</v>
+        <v>166.674</v>
       </c>
       <c r="D92" s="2" t="n"/>
       <c r="E92" s="2" t="n"/>
@@ -3741,7 +3741,7 @@
         <v>351.836</v>
       </c>
       <c r="C93" s="2" t="n">
-        <v>156.674</v>
+        <v>157.674</v>
       </c>
       <c r="D93" s="2" t="n"/>
       <c r="E93" s="2" t="n"/>
@@ -3758,7 +3758,7 @@
         <v>351.836</v>
       </c>
       <c r="C94" s="2" t="n">
-        <v>147.674</v>
+        <v>148.674</v>
       </c>
       <c r="D94" s="2" t="n"/>
       <c r="E94" s="2" t="n"/>
@@ -3775,7 +3775,7 @@
         <v>351.836</v>
       </c>
       <c r="C95" s="2" t="n">
-        <v>138.674</v>
+        <v>139.674</v>
       </c>
       <c r="D95" s="2" t="n"/>
       <c r="E95" s="2" t="n"/>
@@ -3792,7 +3792,7 @@
         <v>351.836</v>
       </c>
       <c r="C96" s="2" t="n">
-        <v>129.674</v>
+        <v>130.674</v>
       </c>
       <c r="D96" s="2" t="n"/>
       <c r="E96" s="2" t="n"/>
@@ -3809,7 +3809,7 @@
         <v>351.836</v>
       </c>
       <c r="C97" s="2" t="n">
-        <v>120.674</v>
+        <v>121.674</v>
       </c>
       <c r="D97" s="2" t="n"/>
       <c r="E97" s="2" t="n"/>
@@ -7201,283 +7201,4 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100DF72643B013E014A825B49D64A1110FC" ma:contentTypeVersion="17" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="f45f840bb0a575e0982080148504d801">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="898ec965-d5a3-48b2-9d91-8cd3ed319c77" xmlns:ns3="34a6835a-a421-4fc1-9891-838ec1df6c1f" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="1578e7a6edb9656aff92510688ad8ae5" ns2:_="" ns3:_="">
-    <xsd:import namespace="898ec965-d5a3-48b2-9d91-8cd3ed319c77"/>
-    <xsd:import namespace="34a6835a-a421-4fc1-9891-838ec1df6c1f"/>
-    <xsd:element name="properties">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element name="documentManagement">
-            <xsd:complexType>
-              <xsd:all>
-                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceAutoTags" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
-                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
-                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
-                <xsd:element ref="ns3:SharedWithUsers" minOccurs="0"/>
-                <xsd:element ref="ns3:SharedWithDetails" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceBillingMetadata" minOccurs="0"/>
-              </xsd:all>
-            </xsd:complexType>
-          </xsd:element>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="898ec965-d5a3-48b2-9d91-8cd3ed319c77" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceAutoTags" ma:index="10" nillable="true" ma:displayName="MediaServiceAutoTags" ma:internalName="MediaServiceAutoTags" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaLengthInSeconds" ma:index="11" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Unknown"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceDateTaken" ma:index="12" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="14" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="d3514cfa-118c-47c7-8064-f16f79621ace" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="MediaServiceGenerationTime" ma:index="16" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceEventHashCode" ma:index="17" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceOCR" ma:index="18" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceLocation" ma:index="19" nillable="true" ma:displayName="Location" ma:indexed="true" ma:internalName="MediaServiceLocation" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="20" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceSearchProperties" ma:index="23" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceBillingMetadata" ma:index="24" nillable="true" ma:displayName="MediaServiceBillingMetadata" ma:hidden="true" ma:internalName="MediaServiceBillingMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="34a6835a-a421-4fc1-9891-838ec1df6c1f" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="TaxCatchAll" ma:index="15" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{fdb65f81-2f44-4049-bc2f-903088f674cc}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="34a6835a-a421-4fc1-9891-838ec1df6c1f">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:MultiChoiceLookup">
-            <xsd:sequence>
-              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="SharedWithUsers" ma:index="21" nillable="true" ma:displayName="Shared With" ma:internalName="SharedWithUsers" ma:readOnly="true">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:UserMulti">
-            <xsd:sequence>
-              <xsd:element name="UserInfo" minOccurs="0" maxOccurs="unbounded">
-                <xsd:complexType>
-                  <xsd:sequence>
-                    <xsd:element name="DisplayName" type="xsd:string" minOccurs="0"/>
-                    <xsd:element name="AccountId" type="dms:UserId" minOccurs="0" nillable="true"/>
-                    <xsd:element name="AccountType" type="xsd:string" minOccurs="0"/>
-                  </xsd:sequence>
-                </xsd:complexType>
-              </xsd:element>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="SharedWithDetails" ma:index="22" nillable="true" ma:displayName="Shared With Details" ma:internalName="SharedWithDetails" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
-    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
-    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
-    <xsd:element name="coreProperties" type="CT_coreProperties"/>
-    <xsd:complexType name="CT_coreProperties">
-      <xsd:all>
-        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
-        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
-        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
-          <xsd:annotation>
-            <xsd:documentation>
-                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
-                    </xsd:documentation>
-          </xsd:annotation>
-        </xsd:element>
-        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-      </xsd:all>
-    </xsd:complexType>
-  </xsd:schema>
-  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
-    <xs:element name="Person">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:DisplayName" minOccurs="0"/>
-          <xs:element ref="pc:AccountId" minOccurs="0"/>
-          <xs:element ref="pc:AccountType" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="DisplayName" type="xs:string"/>
-    <xs:element name="AccountId" type="xs:string"/>
-    <xs:element name="AccountType" type="xs:string"/>
-    <xs:element name="BDCAssociatedEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-        <xs:attribute ref="pc:EntityNamespace"/>
-        <xs:attribute ref="pc:EntityName"/>
-        <xs:attribute ref="pc:SystemInstanceName"/>
-        <xs:attribute ref="pc:AssociationName"/>
-      </xs:complexType>
-    </xs:element>
-    <xs:attribute name="EntityNamespace" type="xs:string"/>
-    <xs:attribute name="EntityName" type="xs:string"/>
-    <xs:attribute name="SystemInstanceName" type="xs:string"/>
-    <xs:attribute name="AssociationName" type="xs:string"/>
-    <xs:element name="BDCEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
-          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
-          <xs:element ref="pc:EntityId1" minOccurs="0"/>
-          <xs:element ref="pc:EntityId2" minOccurs="0"/>
-          <xs:element ref="pc:EntityId3" minOccurs="0"/>
-          <xs:element ref="pc:EntityId4" minOccurs="0"/>
-          <xs:element ref="pc:EntityId5" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="EntityDisplayName" type="xs:string"/>
-    <xs:element name="EntityInstanceReference" type="xs:string"/>
-    <xs:element name="EntityId1" type="xs:string"/>
-    <xs:element name="EntityId2" type="xs:string"/>
-    <xs:element name="EntityId3" type="xs:string"/>
-    <xs:element name="EntityId4" type="xs:string"/>
-    <xs:element name="EntityId5" type="xs:string"/>
-    <xs:element name="Terms">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermInfo">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermName" minOccurs="0"/>
-          <xs:element ref="pc:TermId" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermName" type="xs:string"/>
-    <xs:element name="TermId" type="xs:string"/>
-  </xs:schema>
-</ct:contentTypeSchema>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="898ec965-d5a3-48b2-9d91-8cd3ed319c77">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="34a6835a-a421-4fc1-9891-838ec1df6c1f" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{65AE6621-CA74-4AF4-8B54-6A86D885C6C7}"/>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{41CBF686-DCEB-48C2-8EFA-8989A34E9970}"/>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A67D7C0C-22BC-443A-9997-0F77FC8B40C4}"/>
 </file>
</xml_diff>

<commit_message>
fix(config): plate 3 Y offset +0.5mm for all wells
Operator request: pipette needs to move 0.5mm further in Y for every
well on plate 3. Data-only change to plate_stations.xlsx's Station 3
sheet -- X, well labels, and row order untouched; other stations
untouched.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/config/plate_configs/plate_stations.xlsx
+++ b/config/plate_configs/plate_stations.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-93" yWindow="-93" windowWidth="21520" windowHeight="12800" tabRatio="600" firstSheet="0" activeTab="3" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Station 1" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Station 2" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Station 3" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Station 4" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Station 1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Station 2" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Station 3" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Station 4" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -3885,7 +3885,7 @@
         <v>-192.434</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>283.254</v>
+        <v>283.754</v>
       </c>
       <c r="D2" s="2" t="n"/>
       <c r="E2" s="2" t="n"/>
@@ -3902,7 +3902,7 @@
         <v>-192.434</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>274.254</v>
+        <v>274.754</v>
       </c>
       <c r="D3" s="2" t="n"/>
       <c r="E3" s="2" t="n"/>
@@ -3919,7 +3919,7 @@
         <v>-192.434</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>265.254</v>
+        <v>265.754</v>
       </c>
       <c r="D4" s="2" t="n"/>
       <c r="E4" s="2" t="n"/>
@@ -3936,7 +3936,7 @@
         <v>-192.434</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>256.254</v>
+        <v>256.754</v>
       </c>
       <c r="D5" s="2" t="n"/>
       <c r="E5" s="2" t="n"/>
@@ -3953,7 +3953,7 @@
         <v>-192.434</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>247.254</v>
+        <v>247.754</v>
       </c>
       <c r="D6" s="2" t="n"/>
       <c r="E6" s="2" t="n"/>
@@ -3970,7 +3970,7 @@
         <v>-192.434</v>
       </c>
       <c r="C7" s="2" t="n">
-        <v>238.254</v>
+        <v>238.754</v>
       </c>
       <c r="D7" s="2" t="n"/>
       <c r="E7" s="2" t="n"/>
@@ -3987,7 +3987,7 @@
         <v>-192.434</v>
       </c>
       <c r="C8" s="2" t="n">
-        <v>229.254</v>
+        <v>229.754</v>
       </c>
       <c r="D8" s="2" t="n"/>
       <c r="E8" s="2" t="n"/>
@@ -4004,7 +4004,7 @@
         <v>-192.434</v>
       </c>
       <c r="C9" s="2" t="n">
-        <v>220.254</v>
+        <v>220.754</v>
       </c>
       <c r="D9" s="2" t="n"/>
       <c r="E9" s="2" t="n"/>
@@ -4021,7 +4021,7 @@
         <v>-192.434</v>
       </c>
       <c r="C10" s="2" t="n">
-        <v>211.254</v>
+        <v>211.754</v>
       </c>
       <c r="D10" s="2" t="n"/>
       <c r="E10" s="2" t="n"/>
@@ -4038,7 +4038,7 @@
         <v>-192.434</v>
       </c>
       <c r="C11" s="2" t="n">
-        <v>202.254</v>
+        <v>202.754</v>
       </c>
       <c r="D11" s="2" t="n"/>
       <c r="E11" s="2" t="n"/>
@@ -4055,7 +4055,7 @@
         <v>-192.434</v>
       </c>
       <c r="C12" s="2" t="n">
-        <v>193.254</v>
+        <v>193.754</v>
       </c>
       <c r="D12" s="2" t="n"/>
       <c r="E12" s="2" t="n"/>
@@ -4072,7 +4072,7 @@
         <v>-192.434</v>
       </c>
       <c r="C13" s="2" t="n">
-        <v>184.254</v>
+        <v>184.754</v>
       </c>
       <c r="D13" s="2" t="n"/>
       <c r="E13" s="2" t="n"/>
@@ -4089,7 +4089,7 @@
         <v>-201.434</v>
       </c>
       <c r="C14" s="2" t="n">
-        <v>283.254</v>
+        <v>283.754</v>
       </c>
       <c r="D14" s="2" t="n"/>
       <c r="E14" s="2" t="n"/>
@@ -4106,7 +4106,7 @@
         <v>-201.434</v>
       </c>
       <c r="C15" s="2" t="n">
-        <v>274.254</v>
+        <v>274.754</v>
       </c>
       <c r="D15" s="2" t="n"/>
       <c r="E15" s="2" t="n"/>
@@ -4123,7 +4123,7 @@
         <v>-201.434</v>
       </c>
       <c r="C16" s="2" t="n">
-        <v>265.254</v>
+        <v>265.754</v>
       </c>
       <c r="D16" s="2" t="n"/>
       <c r="E16" s="2" t="n"/>
@@ -4140,7 +4140,7 @@
         <v>-201.434</v>
       </c>
       <c r="C17" s="2" t="n">
-        <v>256.254</v>
+        <v>256.754</v>
       </c>
       <c r="D17" s="2" t="n"/>
       <c r="E17" s="2" t="n"/>
@@ -4157,7 +4157,7 @@
         <v>-201.434</v>
       </c>
       <c r="C18" s="2" t="n">
-        <v>247.254</v>
+        <v>247.754</v>
       </c>
       <c r="D18" s="2" t="n"/>
       <c r="E18" s="2" t="n"/>
@@ -4174,7 +4174,7 @@
         <v>-201.434</v>
       </c>
       <c r="C19" s="2" t="n">
-        <v>238.254</v>
+        <v>238.754</v>
       </c>
       <c r="D19" s="2" t="n"/>
       <c r="E19" s="2" t="n"/>
@@ -4191,7 +4191,7 @@
         <v>-201.434</v>
       </c>
       <c r="C20" s="2" t="n">
-        <v>229.254</v>
+        <v>229.754</v>
       </c>
       <c r="D20" s="2" t="n"/>
       <c r="E20" s="2" t="n"/>
@@ -4208,7 +4208,7 @@
         <v>-201.434</v>
       </c>
       <c r="C21" s="2" t="n">
-        <v>220.254</v>
+        <v>220.754</v>
       </c>
       <c r="D21" s="2" t="n"/>
       <c r="E21" s="2" t="n"/>
@@ -4225,7 +4225,7 @@
         <v>-201.434</v>
       </c>
       <c r="C22" s="2" t="n">
-        <v>211.254</v>
+        <v>211.754</v>
       </c>
       <c r="D22" s="2" t="n"/>
       <c r="E22" s="2" t="n"/>
@@ -4242,7 +4242,7 @@
         <v>-201.434</v>
       </c>
       <c r="C23" s="2" t="n">
-        <v>202.254</v>
+        <v>202.754</v>
       </c>
       <c r="D23" s="2" t="n"/>
       <c r="E23" s="2" t="n"/>
@@ -4259,7 +4259,7 @@
         <v>-201.434</v>
       </c>
       <c r="C24" s="2" t="n">
-        <v>193.254</v>
+        <v>193.754</v>
       </c>
       <c r="D24" s="2" t="n"/>
       <c r="E24" s="2" t="n"/>
@@ -4276,7 +4276,7 @@
         <v>-201.434</v>
       </c>
       <c r="C25" s="2" t="n">
-        <v>184.254</v>
+        <v>184.754</v>
       </c>
       <c r="D25" s="2" t="n"/>
       <c r="E25" s="2" t="n"/>
@@ -4293,7 +4293,7 @@
         <v>-210.434</v>
       </c>
       <c r="C26" s="2" t="n">
-        <v>283.254</v>
+        <v>283.754</v>
       </c>
       <c r="D26" s="2" t="n"/>
       <c r="E26" s="2" t="n"/>
@@ -4310,7 +4310,7 @@
         <v>-210.434</v>
       </c>
       <c r="C27" s="2" t="n">
-        <v>274.254</v>
+        <v>274.754</v>
       </c>
       <c r="D27" s="2" t="n"/>
       <c r="E27" s="2" t="n"/>
@@ -4327,7 +4327,7 @@
         <v>-210.434</v>
       </c>
       <c r="C28" s="2" t="n">
-        <v>265.254</v>
+        <v>265.754</v>
       </c>
       <c r="D28" s="2" t="n"/>
       <c r="E28" s="2" t="n"/>
@@ -4344,7 +4344,7 @@
         <v>-210.434</v>
       </c>
       <c r="C29" s="2" t="n">
-        <v>256.254</v>
+        <v>256.754</v>
       </c>
       <c r="D29" s="2" t="n"/>
       <c r="E29" s="2" t="n"/>
@@ -4361,7 +4361,7 @@
         <v>-210.434</v>
       </c>
       <c r="C30" s="2" t="n">
-        <v>247.254</v>
+        <v>247.754</v>
       </c>
       <c r="D30" s="2" t="n"/>
       <c r="E30" s="2" t="n"/>
@@ -4378,7 +4378,7 @@
         <v>-210.434</v>
       </c>
       <c r="C31" s="2" t="n">
-        <v>238.254</v>
+        <v>238.754</v>
       </c>
       <c r="D31" s="2" t="n"/>
       <c r="E31" s="2" t="n"/>
@@ -4395,7 +4395,7 @@
         <v>-210.434</v>
       </c>
       <c r="C32" s="2" t="n">
-        <v>229.254</v>
+        <v>229.754</v>
       </c>
       <c r="D32" s="2" t="n"/>
       <c r="E32" s="2" t="n"/>
@@ -4412,7 +4412,7 @@
         <v>-210.434</v>
       </c>
       <c r="C33" s="2" t="n">
-        <v>220.254</v>
+        <v>220.754</v>
       </c>
       <c r="D33" s="2" t="n"/>
       <c r="E33" s="2" t="n"/>
@@ -4429,7 +4429,7 @@
         <v>-210.434</v>
       </c>
       <c r="C34" s="2" t="n">
-        <v>211.254</v>
+        <v>211.754</v>
       </c>
       <c r="D34" s="2" t="n"/>
       <c r="E34" s="2" t="n"/>
@@ -4446,7 +4446,7 @@
         <v>-210.434</v>
       </c>
       <c r="C35" s="2" t="n">
-        <v>202.254</v>
+        <v>202.754</v>
       </c>
       <c r="D35" s="2" t="n"/>
       <c r="E35" s="2" t="n"/>
@@ -4463,7 +4463,7 @@
         <v>-210.434</v>
       </c>
       <c r="C36" s="2" t="n">
-        <v>193.254</v>
+        <v>193.754</v>
       </c>
       <c r="D36" s="2" t="n"/>
       <c r="E36" s="2" t="n"/>
@@ -4480,7 +4480,7 @@
         <v>-210.434</v>
       </c>
       <c r="C37" s="2" t="n">
-        <v>184.254</v>
+        <v>184.754</v>
       </c>
       <c r="D37" s="2" t="n"/>
       <c r="E37" s="2" t="n"/>
@@ -4497,7 +4497,7 @@
         <v>-219.434</v>
       </c>
       <c r="C38" s="2" t="n">
-        <v>283.254</v>
+        <v>283.754</v>
       </c>
       <c r="D38" s="2" t="n"/>
       <c r="E38" s="2" t="n"/>
@@ -4514,7 +4514,7 @@
         <v>-219.434</v>
       </c>
       <c r="C39" s="2" t="n">
-        <v>274.254</v>
+        <v>274.754</v>
       </c>
       <c r="D39" s="2" t="n"/>
       <c r="E39" s="2" t="n"/>
@@ -4531,7 +4531,7 @@
         <v>-219.434</v>
       </c>
       <c r="C40" s="2" t="n">
-        <v>265.254</v>
+        <v>265.754</v>
       </c>
       <c r="D40" s="2" t="n"/>
       <c r="E40" s="2" t="n"/>
@@ -4548,7 +4548,7 @@
         <v>-219.434</v>
       </c>
       <c r="C41" s="2" t="n">
-        <v>256.254</v>
+        <v>256.754</v>
       </c>
       <c r="D41" s="2" t="n"/>
       <c r="E41" s="2" t="n"/>
@@ -4565,7 +4565,7 @@
         <v>-219.434</v>
       </c>
       <c r="C42" s="2" t="n">
-        <v>247.254</v>
+        <v>247.754</v>
       </c>
       <c r="D42" s="2" t="n"/>
       <c r="E42" s="2" t="n"/>
@@ -4582,7 +4582,7 @@
         <v>-219.434</v>
       </c>
       <c r="C43" s="2" t="n">
-        <v>238.254</v>
+        <v>238.754</v>
       </c>
       <c r="D43" s="2" t="n"/>
       <c r="E43" s="2" t="n"/>
@@ -4599,7 +4599,7 @@
         <v>-219.434</v>
       </c>
       <c r="C44" s="2" t="n">
-        <v>229.254</v>
+        <v>229.754</v>
       </c>
       <c r="D44" s="2" t="n"/>
       <c r="E44" s="2" t="n"/>
@@ -4616,7 +4616,7 @@
         <v>-219.434</v>
       </c>
       <c r="C45" s="2" t="n">
-        <v>220.254</v>
+        <v>220.754</v>
       </c>
       <c r="D45" s="2" t="n"/>
       <c r="E45" s="2" t="n"/>
@@ -4633,7 +4633,7 @@
         <v>-219.434</v>
       </c>
       <c r="C46" s="2" t="n">
-        <v>211.254</v>
+        <v>211.754</v>
       </c>
       <c r="D46" s="2" t="n"/>
       <c r="E46" s="2" t="n"/>
@@ -4650,7 +4650,7 @@
         <v>-219.434</v>
       </c>
       <c r="C47" s="2" t="n">
-        <v>202.254</v>
+        <v>202.754</v>
       </c>
       <c r="D47" s="2" t="n"/>
       <c r="E47" s="2" t="n"/>
@@ -4667,7 +4667,7 @@
         <v>-219.434</v>
       </c>
       <c r="C48" s="2" t="n">
-        <v>193.254</v>
+        <v>193.754</v>
       </c>
       <c r="D48" s="2" t="n"/>
       <c r="E48" s="2" t="n"/>
@@ -4684,7 +4684,7 @@
         <v>-219.434</v>
       </c>
       <c r="C49" s="2" t="n">
-        <v>184.254</v>
+        <v>184.754</v>
       </c>
       <c r="D49" s="2" t="n"/>
       <c r="E49" s="2" t="n"/>
@@ -4701,7 +4701,7 @@
         <v>-228.434</v>
       </c>
       <c r="C50" s="2" t="n">
-        <v>283.254</v>
+        <v>283.754</v>
       </c>
       <c r="D50" s="2" t="n"/>
       <c r="E50" s="2" t="n"/>
@@ -4718,7 +4718,7 @@
         <v>-228.434</v>
       </c>
       <c r="C51" s="2" t="n">
-        <v>274.254</v>
+        <v>274.754</v>
       </c>
       <c r="D51" s="2" t="n"/>
       <c r="E51" s="2" t="n"/>
@@ -4735,7 +4735,7 @@
         <v>-228.434</v>
       </c>
       <c r="C52" s="2" t="n">
-        <v>265.254</v>
+        <v>265.754</v>
       </c>
       <c r="D52" s="2" t="n"/>
       <c r="E52" s="2" t="n"/>
@@ -4752,7 +4752,7 @@
         <v>-228.434</v>
       </c>
       <c r="C53" s="2" t="n">
-        <v>256.254</v>
+        <v>256.754</v>
       </c>
       <c r="D53" s="2" t="n"/>
       <c r="E53" s="2" t="n"/>
@@ -4769,7 +4769,7 @@
         <v>-228.434</v>
       </c>
       <c r="C54" s="2" t="n">
-        <v>247.254</v>
+        <v>247.754</v>
       </c>
       <c r="D54" s="2" t="n"/>
       <c r="E54" s="2" t="n"/>
@@ -4786,7 +4786,7 @@
         <v>-228.434</v>
       </c>
       <c r="C55" s="2" t="n">
-        <v>238.254</v>
+        <v>238.754</v>
       </c>
       <c r="D55" s="2" t="n"/>
       <c r="E55" s="2" t="n"/>
@@ -4803,7 +4803,7 @@
         <v>-228.434</v>
       </c>
       <c r="C56" s="2" t="n">
-        <v>229.254</v>
+        <v>229.754</v>
       </c>
       <c r="D56" s="2" t="n"/>
       <c r="E56" s="2" t="n"/>
@@ -4820,7 +4820,7 @@
         <v>-228.434</v>
       </c>
       <c r="C57" s="2" t="n">
-        <v>220.254</v>
+        <v>220.754</v>
       </c>
       <c r="D57" s="2" t="n"/>
       <c r="E57" s="2" t="n"/>
@@ -4837,7 +4837,7 @@
         <v>-228.434</v>
       </c>
       <c r="C58" s="2" t="n">
-        <v>211.254</v>
+        <v>211.754</v>
       </c>
       <c r="D58" s="2" t="n"/>
       <c r="E58" s="2" t="n"/>
@@ -4854,7 +4854,7 @@
         <v>-228.434</v>
       </c>
       <c r="C59" s="2" t="n">
-        <v>202.254</v>
+        <v>202.754</v>
       </c>
       <c r="D59" s="2" t="n"/>
       <c r="E59" s="2" t="n"/>
@@ -4871,7 +4871,7 @@
         <v>-228.434</v>
       </c>
       <c r="C60" s="2" t="n">
-        <v>193.254</v>
+        <v>193.754</v>
       </c>
       <c r="D60" s="2" t="n"/>
       <c r="E60" s="2" t="n"/>
@@ -4888,7 +4888,7 @@
         <v>-228.434</v>
       </c>
       <c r="C61" s="2" t="n">
-        <v>184.254</v>
+        <v>184.754</v>
       </c>
       <c r="D61" s="2" t="n"/>
       <c r="E61" s="2" t="n"/>
@@ -4905,7 +4905,7 @@
         <v>-237.434</v>
       </c>
       <c r="C62" s="2" t="n">
-        <v>283.254</v>
+        <v>283.754</v>
       </c>
       <c r="D62" s="2" t="n"/>
       <c r="E62" s="2" t="n"/>
@@ -4922,7 +4922,7 @@
         <v>-237.434</v>
       </c>
       <c r="C63" s="2" t="n">
-        <v>274.254</v>
+        <v>274.754</v>
       </c>
       <c r="D63" s="2" t="n"/>
       <c r="E63" s="2" t="n"/>
@@ -4939,7 +4939,7 @@
         <v>-237.434</v>
       </c>
       <c r="C64" s="2" t="n">
-        <v>265.254</v>
+        <v>265.754</v>
       </c>
       <c r="D64" s="2" t="n"/>
       <c r="E64" s="2" t="n"/>
@@ -4956,7 +4956,7 @@
         <v>-237.434</v>
       </c>
       <c r="C65" s="2" t="n">
-        <v>256.254</v>
+        <v>256.754</v>
       </c>
       <c r="D65" s="2" t="n"/>
       <c r="E65" s="2" t="n"/>
@@ -4973,7 +4973,7 @@
         <v>-237.434</v>
       </c>
       <c r="C66" s="2" t="n">
-        <v>247.254</v>
+        <v>247.754</v>
       </c>
       <c r="D66" s="2" t="n"/>
       <c r="E66" s="2" t="n"/>
@@ -4990,7 +4990,7 @@
         <v>-237.434</v>
       </c>
       <c r="C67" s="2" t="n">
-        <v>238.254</v>
+        <v>238.754</v>
       </c>
       <c r="D67" s="2" t="n"/>
       <c r="E67" s="2" t="n"/>
@@ -5007,7 +5007,7 @@
         <v>-237.434</v>
       </c>
       <c r="C68" s="2" t="n">
-        <v>229.254</v>
+        <v>229.754</v>
       </c>
       <c r="D68" s="2" t="n"/>
       <c r="E68" s="2" t="n"/>
@@ -5024,7 +5024,7 @@
         <v>-237.434</v>
       </c>
       <c r="C69" s="2" t="n">
-        <v>220.254</v>
+        <v>220.754</v>
       </c>
       <c r="D69" s="2" t="n"/>
       <c r="E69" s="2" t="n"/>
@@ -5041,7 +5041,7 @@
         <v>-237.434</v>
       </c>
       <c r="C70" s="2" t="n">
-        <v>211.254</v>
+        <v>211.754</v>
       </c>
       <c r="D70" s="2" t="n"/>
       <c r="E70" s="2" t="n"/>
@@ -5058,7 +5058,7 @@
         <v>-237.434</v>
       </c>
       <c r="C71" s="2" t="n">
-        <v>202.254</v>
+        <v>202.754</v>
       </c>
       <c r="D71" s="2" t="n"/>
       <c r="E71" s="2" t="n"/>
@@ -5075,7 +5075,7 @@
         <v>-237.434</v>
       </c>
       <c r="C72" s="2" t="n">
-        <v>193.254</v>
+        <v>193.754</v>
       </c>
       <c r="D72" s="2" t="n"/>
       <c r="E72" s="2" t="n"/>
@@ -5092,7 +5092,7 @@
         <v>-237.434</v>
       </c>
       <c r="C73" s="2" t="n">
-        <v>184.254</v>
+        <v>184.754</v>
       </c>
       <c r="D73" s="2" t="n"/>
       <c r="E73" s="2" t="n"/>
@@ -5109,7 +5109,7 @@
         <v>-246.434</v>
       </c>
       <c r="C74" s="2" t="n">
-        <v>283.254</v>
+        <v>283.754</v>
       </c>
       <c r="D74" s="2" t="n"/>
       <c r="E74" s="2" t="n"/>
@@ -5126,7 +5126,7 @@
         <v>-246.434</v>
       </c>
       <c r="C75" s="2" t="n">
-        <v>274.254</v>
+        <v>274.754</v>
       </c>
       <c r="D75" s="2" t="n"/>
       <c r="E75" s="2" t="n"/>
@@ -5143,7 +5143,7 @@
         <v>-246.434</v>
       </c>
       <c r="C76" s="2" t="n">
-        <v>265.254</v>
+        <v>265.754</v>
       </c>
       <c r="D76" s="2" t="n"/>
       <c r="E76" s="2" t="n"/>
@@ -5160,7 +5160,7 @@
         <v>-246.434</v>
       </c>
       <c r="C77" s="2" t="n">
-        <v>256.254</v>
+        <v>256.754</v>
       </c>
       <c r="D77" s="2" t="n"/>
       <c r="E77" s="2" t="n"/>
@@ -5177,7 +5177,7 @@
         <v>-246.434</v>
       </c>
       <c r="C78" s="2" t="n">
-        <v>247.254</v>
+        <v>247.754</v>
       </c>
       <c r="D78" s="2" t="n"/>
       <c r="E78" s="2" t="n"/>
@@ -5194,7 +5194,7 @@
         <v>-246.434</v>
       </c>
       <c r="C79" s="2" t="n">
-        <v>238.254</v>
+        <v>238.754</v>
       </c>
       <c r="D79" s="2" t="n"/>
       <c r="E79" s="2" t="n"/>
@@ -5211,7 +5211,7 @@
         <v>-246.434</v>
       </c>
       <c r="C80" s="2" t="n">
-        <v>229.254</v>
+        <v>229.754</v>
       </c>
       <c r="D80" s="2" t="n"/>
       <c r="E80" s="2" t="n"/>
@@ -5228,7 +5228,7 @@
         <v>-246.434</v>
       </c>
       <c r="C81" s="2" t="n">
-        <v>220.254</v>
+        <v>220.754</v>
       </c>
       <c r="D81" s="2" t="n"/>
       <c r="E81" s="2" t="n"/>
@@ -5245,7 +5245,7 @@
         <v>-246.434</v>
       </c>
       <c r="C82" s="2" t="n">
-        <v>211.254</v>
+        <v>211.754</v>
       </c>
       <c r="D82" s="2" t="n"/>
       <c r="E82" s="2" t="n"/>
@@ -5262,7 +5262,7 @@
         <v>-246.434</v>
       </c>
       <c r="C83" s="2" t="n">
-        <v>202.254</v>
+        <v>202.754</v>
       </c>
       <c r="D83" s="2" t="n"/>
       <c r="E83" s="2" t="n"/>
@@ -5279,7 +5279,7 @@
         <v>-246.434</v>
       </c>
       <c r="C84" s="2" t="n">
-        <v>193.254</v>
+        <v>193.754</v>
       </c>
       <c r="D84" s="2" t="n"/>
       <c r="E84" s="2" t="n"/>
@@ -5296,7 +5296,7 @@
         <v>-246.434</v>
       </c>
       <c r="C85" s="2" t="n">
-        <v>184.254</v>
+        <v>184.754</v>
       </c>
       <c r="D85" s="2" t="n"/>
       <c r="E85" s="2" t="n"/>
@@ -5313,7 +5313,7 @@
         <v>-255.434</v>
       </c>
       <c r="C86" s="2" t="n">
-        <v>283.254</v>
+        <v>283.754</v>
       </c>
       <c r="D86" s="2" t="n"/>
       <c r="E86" s="2" t="n"/>
@@ -5330,7 +5330,7 @@
         <v>-255.434</v>
       </c>
       <c r="C87" s="2" t="n">
-        <v>274.254</v>
+        <v>274.754</v>
       </c>
       <c r="D87" s="2" t="n"/>
       <c r="E87" s="2" t="n"/>
@@ -5347,7 +5347,7 @@
         <v>-255.434</v>
       </c>
       <c r="C88" s="2" t="n">
-        <v>265.254</v>
+        <v>265.754</v>
       </c>
       <c r="D88" s="2" t="n"/>
       <c r="E88" s="2" t="n"/>
@@ -5364,7 +5364,7 @@
         <v>-255.434</v>
       </c>
       <c r="C89" s="2" t="n">
-        <v>256.254</v>
+        <v>256.754</v>
       </c>
       <c r="D89" s="2" t="n"/>
       <c r="E89" s="2" t="n"/>
@@ -5381,7 +5381,7 @@
         <v>-255.434</v>
       </c>
       <c r="C90" s="2" t="n">
-        <v>247.254</v>
+        <v>247.754</v>
       </c>
       <c r="D90" s="2" t="n"/>
       <c r="E90" s="2" t="n"/>
@@ -5398,7 +5398,7 @@
         <v>-255.434</v>
       </c>
       <c r="C91" s="2" t="n">
-        <v>238.254</v>
+        <v>238.754</v>
       </c>
       <c r="D91" s="2" t="n"/>
       <c r="E91" s="2" t="n"/>
@@ -5415,7 +5415,7 @@
         <v>-255.434</v>
       </c>
       <c r="C92" s="2" t="n">
-        <v>229.254</v>
+        <v>229.754</v>
       </c>
       <c r="D92" s="2" t="n"/>
       <c r="E92" s="2" t="n"/>
@@ -5432,7 +5432,7 @@
         <v>-255.434</v>
       </c>
       <c r="C93" s="2" t="n">
-        <v>220.254</v>
+        <v>220.754</v>
       </c>
       <c r="D93" s="2" t="n"/>
       <c r="E93" s="2" t="n"/>
@@ -5449,7 +5449,7 @@
         <v>-255.434</v>
       </c>
       <c r="C94" s="2" t="n">
-        <v>211.254</v>
+        <v>211.754</v>
       </c>
       <c r="D94" s="2" t="n"/>
       <c r="E94" s="2" t="n"/>
@@ -5466,7 +5466,7 @@
         <v>-255.434</v>
       </c>
       <c r="C95" s="2" t="n">
-        <v>202.254</v>
+        <v>202.754</v>
       </c>
       <c r="D95" s="2" t="n"/>
       <c r="E95" s="2" t="n"/>
@@ -5483,7 +5483,7 @@
         <v>-255.434</v>
       </c>
       <c r="C96" s="2" t="n">
-        <v>193.254</v>
+        <v>193.754</v>
       </c>
       <c r="D96" s="2" t="n"/>
       <c r="E96" s="2" t="n"/>
@@ -5500,7 +5500,7 @@
         <v>-255.434</v>
       </c>
       <c r="C97" s="2" t="n">
-        <v>184.254</v>
+        <v>184.754</v>
       </c>
       <c r="D97" s="2" t="n"/>
       <c r="E97" s="2" t="n"/>

</xml_diff>